<commit_message>
data: hourly update 2026-06-29 13:09Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-06-29.xlsx
+++ b/data/output/workbook/2026-06-29.xlsx
@@ -550,7 +550,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="9410700"/>
+    <ext cx="10125075" cy="10048875"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -580,7 +580,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="9810750"/>
+    <ext cx="10125075" cy="9401175"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -953,7 +953,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 04:21</t>
+          <t>2026-06-29 09:09</t>
         </is>
       </c>
     </row>
@@ -4529,7 +4529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q74"/>
+  <dimension ref="A1:Q78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4546,823 +4546,823 @@
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="28" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="28" t="inlineStr">
         <is>
           <t>Cincinnati Reds offense vs Milwaukee Brewers defense</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="29" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="29" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B61" s="29" t="inlineStr">
+      <c r="B65" s="29" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C61" s="29" t="inlineStr">
+      <c r="C65" s="29" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D61" s="29" t="inlineStr">
+      <c r="D65" s="29" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E61" s="29" t="inlineStr">
+      <c r="E65" s="29" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F61" s="29" t="inlineStr">
+      <c r="F65" s="29" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G61" s="29" t="inlineStr">
+      <c r="G65" s="29" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H61" s="29" t="inlineStr">
+      <c r="H65" s="29" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I61" s="29" t="inlineStr">
+      <c r="I65" s="29" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J61" s="29" t="inlineStr">
+      <c r="J65" s="29" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K61" s="29" t="inlineStr">
+      <c r="K65" s="29" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L61" s="29" t="inlineStr">
+      <c r="L65" s="29" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M61" s="29" t="inlineStr">
+      <c r="M65" s="29" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N61" s="29" t="inlineStr">
+      <c r="N65" s="29" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O61" s="29" t="inlineStr">
+      <c r="O65" s="29" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P61" s="29" t="inlineStr">
+      <c r="P65" s="29" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q61" s="29" t="inlineStr">
+      <c r="Q65" s="29" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="30" t="inlineStr">
-        <is>
-          <t>Runs/G</t>
-        </is>
-      </c>
-      <c r="B62" s="31" t="n">
-        <v>4.132</v>
-      </c>
-      <c r="C62" s="31" t="n">
-        <v>4.433</v>
-      </c>
-      <c r="D62" s="31" t="n">
-        <v>4.65</v>
-      </c>
-      <c r="E62" s="31" t="n">
-        <v>4.867</v>
-      </c>
-      <c r="F62" s="31" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="G62" s="31" t="n">
-        <v>5</v>
-      </c>
-      <c r="H62" s="32" t="inlineStr">
-        <is>
-          <t>8th</t>
-        </is>
-      </c>
-      <c r="I62" s="31" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="J62" s="35" t="inlineStr">
-        <is>
-          <t>11th</t>
-        </is>
-      </c>
-      <c r="K62" s="31" t="n">
-        <v>3</v>
-      </c>
-      <c r="L62" s="31" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="M62" s="31" t="n">
-        <v>3.267</v>
-      </c>
-      <c r="N62" s="31" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="O62" s="31" t="n">
-        <v>4.033</v>
-      </c>
-      <c r="P62" s="31" t="n">
-        <v>3.784</v>
-      </c>
-      <c r="Q62" s="34" t="inlineStr">
-        <is>
-          <t>Opp Runs/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="30" t="inlineStr">
-        <is>
-          <t>Hits/G</t>
-        </is>
-      </c>
-      <c r="B63" s="31" t="n">
-        <v>7.216</v>
-      </c>
-      <c r="C63" s="31" t="n">
-        <v>7.345</v>
-      </c>
-      <c r="D63" s="31" t="n">
-        <v>7.632</v>
-      </c>
-      <c r="E63" s="31" t="n">
-        <v>8</v>
-      </c>
-      <c r="F63" s="31" t="n">
-        <v>7.667</v>
-      </c>
-      <c r="G63" s="31" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="H63" s="35" t="inlineStr">
-        <is>
-          <t>16th</t>
-        </is>
-      </c>
-      <c r="I63" s="31" t="inlineStr"/>
-      <c r="J63" s="32" t="inlineStr">
-        <is>
-          <t>4th</t>
-        </is>
-      </c>
-      <c r="K63" s="31" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="L63" s="31" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="M63" s="31" t="n">
-        <v>6.308</v>
-      </c>
-      <c r="N63" s="31" t="n">
-        <v>6.722</v>
-      </c>
-      <c r="O63" s="31" t="n">
-        <v>7.536</v>
-      </c>
-      <c r="P63" s="31" t="n">
-        <v>7.371</v>
-      </c>
-      <c r="Q63" s="34" t="inlineStr">
-        <is>
-          <t>Opp Hits/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="30" t="inlineStr">
-        <is>
-          <t>HR/G</t>
-        </is>
-      </c>
-      <c r="B64" s="31" t="n">
-        <v>1.216</v>
-      </c>
-      <c r="C64" s="31" t="n">
-        <v>1.241</v>
-      </c>
-      <c r="D64" s="31" t="n">
-        <v>1.263</v>
-      </c>
-      <c r="E64" s="31" t="n">
-        <v>1.643</v>
-      </c>
-      <c r="F64" s="31" t="n">
-        <v>0.889</v>
-      </c>
-      <c r="G64" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="H64" s="35" t="inlineStr">
-        <is>
-          <t>13th</t>
-        </is>
-      </c>
-      <c r="I64" s="31" t="inlineStr"/>
-      <c r="J64" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K64" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L64" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M64" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N64" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O64" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P64" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q64" s="34" t="inlineStr">
-        <is>
-          <t>Opp HR/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="30" t="inlineStr">
-        <is>
-          <t>Batter K/G</t>
-        </is>
-      </c>
-      <c r="B65" s="31" t="n">
-        <v>9.27</v>
-      </c>
-      <c r="C65" s="31" t="n">
-        <v>9.103</v>
-      </c>
-      <c r="D65" s="31" t="n">
-        <v>9.420999999999999</v>
-      </c>
-      <c r="E65" s="31" t="n">
-        <v>9.286</v>
-      </c>
-      <c r="F65" s="31" t="n">
-        <v>8.888999999999999</v>
-      </c>
-      <c r="G65" s="31" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="H65" s="33" t="inlineStr">
-        <is>
-          <t>22nd</t>
-        </is>
-      </c>
-      <c r="I65" s="31" t="inlineStr"/>
-      <c r="J65" s="32" t="inlineStr">
-        <is>
-          <t>5th</t>
-        </is>
-      </c>
-      <c r="K65" s="31" t="n">
-        <v>10</v>
-      </c>
-      <c r="L65" s="31" t="n">
-        <v>10.625</v>
-      </c>
-      <c r="M65" s="31" t="n">
-        <v>10.538</v>
-      </c>
-      <c r="N65" s="31" t="n">
-        <v>10</v>
-      </c>
-      <c r="O65" s="31" t="n">
-        <v>8.929</v>
-      </c>
-      <c r="P65" s="31" t="n">
-        <v>9.571</v>
-      </c>
-      <c r="Q65" s="34" t="inlineStr">
-        <is>
-          <t>Opp Batter K/G</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="30" t="inlineStr">
         <is>
-          <t>1st Inn R/G</t>
+          <t>Runs/G</t>
         </is>
       </c>
       <c r="B66" s="31" t="n">
-        <v>0.595</v>
+        <v>4.132</v>
       </c>
       <c r="C66" s="31" t="n">
-        <v>0.621</v>
+        <v>4.433</v>
       </c>
       <c r="D66" s="31" t="n">
-        <v>0.421</v>
+        <v>4.65</v>
       </c>
       <c r="E66" s="31" t="n">
-        <v>0.429</v>
+        <v>4.867</v>
       </c>
       <c r="F66" s="31" t="n">
-        <v>0</v>
+        <v>3.9</v>
       </c>
       <c r="G66" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H66" s="33" t="inlineStr">
-        <is>
-          <t>26th</t>
-        </is>
-      </c>
-      <c r="I66" s="31" t="inlineStr"/>
-      <c r="J66" s="32" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="H66" s="32" t="inlineStr">
+        <is>
+          <t>8th</t>
+        </is>
+      </c>
+      <c r="I66" s="31" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="J66" s="35" t="inlineStr">
+        <is>
+          <t>11th</t>
+        </is>
+      </c>
+      <c r="K66" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="L66" s="31" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="M66" s="31" t="n">
+        <v>3.267</v>
+      </c>
+      <c r="N66" s="31" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="O66" s="31" t="n">
+        <v>4.033</v>
+      </c>
+      <c r="P66" s="31" t="n">
+        <v>3.784</v>
+      </c>
+      <c r="Q66" s="34" t="inlineStr">
+        <is>
+          <t>Opp Runs/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="30" t="inlineStr">
+        <is>
+          <t>Hits/G</t>
+        </is>
+      </c>
+      <c r="B67" s="31" t="n">
+        <v>7.216</v>
+      </c>
+      <c r="C67" s="31" t="n">
+        <v>7.345</v>
+      </c>
+      <c r="D67" s="31" t="n">
+        <v>7.632</v>
+      </c>
+      <c r="E67" s="31" t="n">
+        <v>8</v>
+      </c>
+      <c r="F67" s="31" t="n">
+        <v>7.667</v>
+      </c>
+      <c r="G67" s="31" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="H67" s="35" t="inlineStr">
+        <is>
+          <t>16th</t>
+        </is>
+      </c>
+      <c r="I67" s="31" t="inlineStr"/>
+      <c r="J67" s="32" t="inlineStr">
+        <is>
+          <t>4th</t>
+        </is>
+      </c>
+      <c r="K67" s="31" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="L67" s="31" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="M67" s="31" t="n">
+        <v>6.308</v>
+      </c>
+      <c r="N67" s="31" t="n">
+        <v>6.722</v>
+      </c>
+      <c r="O67" s="31" t="n">
+        <v>7.536</v>
+      </c>
+      <c r="P67" s="31" t="n">
+        <v>7.371</v>
+      </c>
+      <c r="Q67" s="34" t="inlineStr">
+        <is>
+          <t>Opp Hits/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="30" t="inlineStr">
+        <is>
+          <t>HR/G</t>
+        </is>
+      </c>
+      <c r="B68" s="31" t="n">
+        <v>1.216</v>
+      </c>
+      <c r="C68" s="31" t="n">
+        <v>1.241</v>
+      </c>
+      <c r="D68" s="31" t="n">
+        <v>1.263</v>
+      </c>
+      <c r="E68" s="31" t="n">
+        <v>1.643</v>
+      </c>
+      <c r="F68" s="31" t="n">
+        <v>0.889</v>
+      </c>
+      <c r="G68" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H68" s="35" t="inlineStr">
+        <is>
+          <t>13th</t>
+        </is>
+      </c>
+      <c r="I68" s="31" t="inlineStr"/>
+      <c r="J68" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K68" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L68" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M68" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N68" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O68" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P68" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q68" s="34" t="inlineStr">
+        <is>
+          <t>Opp HR/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="30" t="inlineStr">
+        <is>
+          <t>Batter K/G</t>
+        </is>
+      </c>
+      <c r="B69" s="31" t="n">
+        <v>9.27</v>
+      </c>
+      <c r="C69" s="31" t="n">
+        <v>9.103</v>
+      </c>
+      <c r="D69" s="31" t="n">
+        <v>9.420999999999999</v>
+      </c>
+      <c r="E69" s="31" t="n">
+        <v>9.286</v>
+      </c>
+      <c r="F69" s="31" t="n">
+        <v>8.888999999999999</v>
+      </c>
+      <c r="G69" s="31" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="H69" s="33" t="inlineStr">
+        <is>
+          <t>22nd</t>
+        </is>
+      </c>
+      <c r="I69" s="31" t="inlineStr"/>
+      <c r="J69" s="32" t="inlineStr">
         <is>
           <t>5th</t>
         </is>
       </c>
-      <c r="K66" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="L66" s="31" t="n">
-        <v>0.125</v>
-      </c>
-      <c r="M66" s="31" t="n">
-        <v>0.231</v>
-      </c>
-      <c r="N66" s="31" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="O66" s="31" t="n">
-        <v>0.357</v>
-      </c>
-      <c r="P66" s="31" t="n">
-        <v>0.486</v>
-      </c>
-      <c r="Q66" s="34" t="inlineStr">
-        <is>
-          <t>Opp 1st Inn R/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="28" t="inlineStr">
-        <is>
-          <t>Milwaukee Brewers offense vs Cincinnati Reds defense</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="29" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="B69" s="29" t="inlineStr">
-        <is>
-          <t>A Season</t>
-        </is>
-      </c>
-      <c r="C69" s="29" t="inlineStr">
-        <is>
-          <t>A L30</t>
-        </is>
-      </c>
-      <c r="D69" s="29" t="inlineStr">
-        <is>
-          <t>A L20</t>
-        </is>
-      </c>
-      <c r="E69" s="29" t="inlineStr">
-        <is>
-          <t>A L15</t>
-        </is>
-      </c>
-      <c r="F69" s="29" t="inlineStr">
-        <is>
-          <t>A L10</t>
-        </is>
-      </c>
-      <c r="G69" s="29" t="inlineStr">
-        <is>
-          <t>A L5</t>
-        </is>
-      </c>
-      <c r="H69" s="29" t="inlineStr">
-        <is>
-          <t>A Rk</t>
-        </is>
-      </c>
-      <c r="I69" s="29" t="inlineStr">
-        <is>
-          <t>Adv</t>
-        </is>
-      </c>
-      <c r="J69" s="29" t="inlineStr">
-        <is>
-          <t>H Rk</t>
-        </is>
-      </c>
-      <c r="K69" s="29" t="inlineStr">
-        <is>
-          <t>H L5</t>
-        </is>
-      </c>
-      <c r="L69" s="29" t="inlineStr">
-        <is>
-          <t>H L10</t>
-        </is>
-      </c>
-      <c r="M69" s="29" t="inlineStr">
-        <is>
-          <t>H L15</t>
-        </is>
-      </c>
-      <c r="N69" s="29" t="inlineStr">
-        <is>
-          <t>H L20</t>
-        </is>
-      </c>
-      <c r="O69" s="29" t="inlineStr">
-        <is>
-          <t>H L30</t>
-        </is>
-      </c>
-      <c r="P69" s="29" t="inlineStr">
-        <is>
-          <t>H Season</t>
-        </is>
-      </c>
-      <c r="Q69" s="29" t="inlineStr">
-        <is>
-          <t>Opp stat</t>
+      <c r="K69" s="31" t="n">
+        <v>10</v>
+      </c>
+      <c r="L69" s="31" t="n">
+        <v>10.625</v>
+      </c>
+      <c r="M69" s="31" t="n">
+        <v>10.538</v>
+      </c>
+      <c r="N69" s="31" t="n">
+        <v>10</v>
+      </c>
+      <c r="O69" s="31" t="n">
+        <v>8.929</v>
+      </c>
+      <c r="P69" s="31" t="n">
+        <v>9.571</v>
+      </c>
+      <c r="Q69" s="34" t="inlineStr">
+        <is>
+          <t>Opp Batter K/G</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="30" t="inlineStr">
         <is>
-          <t>Runs/G</t>
+          <t>1st Inn R/G</t>
         </is>
       </c>
       <c r="B70" s="31" t="n">
-        <v>4.703</v>
+        <v>0.595</v>
       </c>
       <c r="C70" s="31" t="n">
-        <v>4.133</v>
+        <v>0.621</v>
       </c>
       <c r="D70" s="31" t="n">
-        <v>4.25</v>
+        <v>0.421</v>
       </c>
       <c r="E70" s="31" t="n">
-        <v>3.733</v>
+        <v>0.429</v>
       </c>
       <c r="F70" s="31" t="n">
-        <v>4.2</v>
+        <v>0</v>
       </c>
       <c r="G70" s="31" t="n">
-        <v>4</v>
-      </c>
-      <c r="H70" s="35" t="inlineStr">
-        <is>
-          <t>15th</t>
-        </is>
-      </c>
-      <c r="I70" s="31" t="inlineStr">
-        <is>
-          <t>★★</t>
-        </is>
-      </c>
-      <c r="J70" s="33" t="inlineStr">
-        <is>
-          <t>25th</t>
+        <v>0</v>
+      </c>
+      <c r="H70" s="33" t="inlineStr">
+        <is>
+          <t>26th</t>
+        </is>
+      </c>
+      <c r="I70" s="31" t="inlineStr"/>
+      <c r="J70" s="32" t="inlineStr">
+        <is>
+          <t>5th</t>
         </is>
       </c>
       <c r="K70" s="31" t="n">
-        <v>5.2</v>
+        <v>0</v>
       </c>
       <c r="L70" s="31" t="n">
-        <v>6</v>
+        <v>0.125</v>
       </c>
       <c r="M70" s="31" t="n">
-        <v>6</v>
+        <v>0.231</v>
       </c>
       <c r="N70" s="31" t="n">
-        <v>5.15</v>
+        <v>0.333</v>
       </c>
       <c r="O70" s="31" t="n">
-        <v>4.933</v>
+        <v>0.357</v>
       </c>
       <c r="P70" s="31" t="n">
-        <v>4.658</v>
+        <v>0.486</v>
       </c>
       <c r="Q70" s="34" t="inlineStr">
         <is>
-          <t>Opp Runs/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="30" t="inlineStr">
-        <is>
-          <t>Hits/G</t>
-        </is>
-      </c>
-      <c r="B71" s="31" t="n">
-        <v>7.629</v>
-      </c>
-      <c r="C71" s="31" t="n">
-        <v>7.143</v>
-      </c>
-      <c r="D71" s="31" t="n">
-        <v>7.389</v>
-      </c>
-      <c r="E71" s="31" t="n">
-        <v>7</v>
-      </c>
-      <c r="F71" s="31" t="n">
-        <v>7.625</v>
-      </c>
-      <c r="G71" s="31" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="H71" s="35" t="inlineStr">
-        <is>
-          <t>18th</t>
-        </is>
-      </c>
-      <c r="I71" s="31" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="J71" s="33" t="inlineStr">
-        <is>
-          <t>21st</t>
-        </is>
-      </c>
-      <c r="K71" s="31" t="n">
-        <v>8</v>
-      </c>
-      <c r="L71" s="31" t="n">
-        <v>8</v>
-      </c>
-      <c r="M71" s="31" t="n">
-        <v>8.714</v>
-      </c>
-      <c r="N71" s="31" t="n">
-        <v>8.263</v>
-      </c>
-      <c r="O71" s="31" t="n">
-        <v>8.207000000000001</v>
-      </c>
-      <c r="P71" s="31" t="n">
-        <v>8.054</v>
-      </c>
-      <c r="Q71" s="34" t="inlineStr">
-        <is>
-          <t>Opp Hits/G</t>
+          <t>Opp 1st Inn R/G</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="30" t="inlineStr">
-        <is>
-          <t>HR/G</t>
-        </is>
-      </c>
-      <c r="B72" s="31" t="n">
-        <v>0.657</v>
-      </c>
-      <c r="C72" s="31" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D72" s="31" t="n">
-        <v>0.278</v>
-      </c>
-      <c r="E72" s="31" t="n">
-        <v>0.308</v>
-      </c>
-      <c r="F72" s="31" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G72" s="31" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H72" s="33" t="inlineStr">
-        <is>
-          <t>28th</t>
-        </is>
-      </c>
-      <c r="I72" s="31" t="inlineStr"/>
-      <c r="J72" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K72" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L72" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M72" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N72" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O72" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P72" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q72" s="34" t="inlineStr">
-        <is>
-          <t>Opp HR/G</t>
+      <c r="A72" s="28" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers offense vs Cincinnati Reds defense</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="30" t="inlineStr">
-        <is>
-          <t>Batter K/G</t>
-        </is>
-      </c>
-      <c r="B73" s="31" t="n">
-        <v>8.228999999999999</v>
-      </c>
-      <c r="C73" s="31" t="n">
-        <v>8.179</v>
-      </c>
-      <c r="D73" s="31" t="n">
-        <v>7.944</v>
-      </c>
-      <c r="E73" s="31" t="n">
-        <v>8.077</v>
-      </c>
-      <c r="F73" s="31" t="n">
-        <v>7.875</v>
-      </c>
-      <c r="G73" s="31" t="n">
-        <v>8</v>
-      </c>
-      <c r="H73" s="35" t="inlineStr">
-        <is>
-          <t>12th</t>
-        </is>
-      </c>
-      <c r="I73" s="31" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="J73" s="35" t="inlineStr">
-        <is>
-          <t>16th</t>
-        </is>
-      </c>
-      <c r="K73" s="31" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="L73" s="31" t="n">
-        <v>6.667</v>
-      </c>
-      <c r="M73" s="31" t="n">
-        <v>7.143</v>
-      </c>
-      <c r="N73" s="31" t="n">
-        <v>7.105</v>
-      </c>
-      <c r="O73" s="31" t="n">
-        <v>6.966</v>
-      </c>
-      <c r="P73" s="31" t="n">
-        <v>7.432</v>
-      </c>
-      <c r="Q73" s="34" t="inlineStr">
-        <is>
-          <t>Opp Batter K/G</t>
+      <c r="A73" s="29" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B73" s="29" t="inlineStr">
+        <is>
+          <t>A Season</t>
+        </is>
+      </c>
+      <c r="C73" s="29" t="inlineStr">
+        <is>
+          <t>A L30</t>
+        </is>
+      </c>
+      <c r="D73" s="29" t="inlineStr">
+        <is>
+          <t>A L20</t>
+        </is>
+      </c>
+      <c r="E73" s="29" t="inlineStr">
+        <is>
+          <t>A L15</t>
+        </is>
+      </c>
+      <c r="F73" s="29" t="inlineStr">
+        <is>
+          <t>A L10</t>
+        </is>
+      </c>
+      <c r="G73" s="29" t="inlineStr">
+        <is>
+          <t>A L5</t>
+        </is>
+      </c>
+      <c r="H73" s="29" t="inlineStr">
+        <is>
+          <t>A Rk</t>
+        </is>
+      </c>
+      <c r="I73" s="29" t="inlineStr">
+        <is>
+          <t>Adv</t>
+        </is>
+      </c>
+      <c r="J73" s="29" t="inlineStr">
+        <is>
+          <t>H Rk</t>
+        </is>
+      </c>
+      <c r="K73" s="29" t="inlineStr">
+        <is>
+          <t>H L5</t>
+        </is>
+      </c>
+      <c r="L73" s="29" t="inlineStr">
+        <is>
+          <t>H L10</t>
+        </is>
+      </c>
+      <c r="M73" s="29" t="inlineStr">
+        <is>
+          <t>H L15</t>
+        </is>
+      </c>
+      <c r="N73" s="29" t="inlineStr">
+        <is>
+          <t>H L20</t>
+        </is>
+      </c>
+      <c r="O73" s="29" t="inlineStr">
+        <is>
+          <t>H L30</t>
+        </is>
+      </c>
+      <c r="P73" s="29" t="inlineStr">
+        <is>
+          <t>H Season</t>
+        </is>
+      </c>
+      <c r="Q73" s="29" t="inlineStr">
+        <is>
+          <t>Opp stat</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="30" t="inlineStr">
         <is>
+          <t>Runs/G</t>
+        </is>
+      </c>
+      <c r="B74" s="31" t="n">
+        <v>4.703</v>
+      </c>
+      <c r="C74" s="31" t="n">
+        <v>4.133</v>
+      </c>
+      <c r="D74" s="31" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="E74" s="31" t="n">
+        <v>3.733</v>
+      </c>
+      <c r="F74" s="31" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="G74" s="31" t="n">
+        <v>4</v>
+      </c>
+      <c r="H74" s="35" t="inlineStr">
+        <is>
+          <t>15th</t>
+        </is>
+      </c>
+      <c r="I74" s="31" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="J74" s="33" t="inlineStr">
+        <is>
+          <t>25th</t>
+        </is>
+      </c>
+      <c r="K74" s="31" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="L74" s="31" t="n">
+        <v>6</v>
+      </c>
+      <c r="M74" s="31" t="n">
+        <v>6</v>
+      </c>
+      <c r="N74" s="31" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="O74" s="31" t="n">
+        <v>4.933</v>
+      </c>
+      <c r="P74" s="31" t="n">
+        <v>4.658</v>
+      </c>
+      <c r="Q74" s="34" t="inlineStr">
+        <is>
+          <t>Opp Runs/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="30" t="inlineStr">
+        <is>
+          <t>Hits/G</t>
+        </is>
+      </c>
+      <c r="B75" s="31" t="n">
+        <v>7.629</v>
+      </c>
+      <c r="C75" s="31" t="n">
+        <v>7.143</v>
+      </c>
+      <c r="D75" s="31" t="n">
+        <v>7.389</v>
+      </c>
+      <c r="E75" s="31" t="n">
+        <v>7</v>
+      </c>
+      <c r="F75" s="31" t="n">
+        <v>7.625</v>
+      </c>
+      <c r="G75" s="31" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="H75" s="35" t="inlineStr">
+        <is>
+          <t>18th</t>
+        </is>
+      </c>
+      <c r="I75" s="31" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="J75" s="33" t="inlineStr">
+        <is>
+          <t>21st</t>
+        </is>
+      </c>
+      <c r="K75" s="31" t="n">
+        <v>8</v>
+      </c>
+      <c r="L75" s="31" t="n">
+        <v>8</v>
+      </c>
+      <c r="M75" s="31" t="n">
+        <v>8.714</v>
+      </c>
+      <c r="N75" s="31" t="n">
+        <v>8.263</v>
+      </c>
+      <c r="O75" s="31" t="n">
+        <v>8.207000000000001</v>
+      </c>
+      <c r="P75" s="31" t="n">
+        <v>8.054</v>
+      </c>
+      <c r="Q75" s="34" t="inlineStr">
+        <is>
+          <t>Opp Hits/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="30" t="inlineStr">
+        <is>
+          <t>HR/G</t>
+        </is>
+      </c>
+      <c r="B76" s="31" t="n">
+        <v>0.657</v>
+      </c>
+      <c r="C76" s="31" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D76" s="31" t="n">
+        <v>0.278</v>
+      </c>
+      <c r="E76" s="31" t="n">
+        <v>0.308</v>
+      </c>
+      <c r="F76" s="31" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G76" s="31" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H76" s="33" t="inlineStr">
+        <is>
+          <t>28th</t>
+        </is>
+      </c>
+      <c r="I76" s="31" t="inlineStr"/>
+      <c r="J76" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K76" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L76" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M76" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N76" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O76" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P76" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q76" s="34" t="inlineStr">
+        <is>
+          <t>Opp HR/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="30" t="inlineStr">
+        <is>
+          <t>Batter K/G</t>
+        </is>
+      </c>
+      <c r="B77" s="31" t="n">
+        <v>8.228999999999999</v>
+      </c>
+      <c r="C77" s="31" t="n">
+        <v>8.179</v>
+      </c>
+      <c r="D77" s="31" t="n">
+        <v>7.944</v>
+      </c>
+      <c r="E77" s="31" t="n">
+        <v>8.077</v>
+      </c>
+      <c r="F77" s="31" t="n">
+        <v>7.875</v>
+      </c>
+      <c r="G77" s="31" t="n">
+        <v>8</v>
+      </c>
+      <c r="H77" s="35" t="inlineStr">
+        <is>
+          <t>12th</t>
+        </is>
+      </c>
+      <c r="I77" s="31" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="J77" s="35" t="inlineStr">
+        <is>
+          <t>16th</t>
+        </is>
+      </c>
+      <c r="K77" s="31" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="L77" s="31" t="n">
+        <v>6.667</v>
+      </c>
+      <c r="M77" s="31" t="n">
+        <v>7.143</v>
+      </c>
+      <c r="N77" s="31" t="n">
+        <v>7.105</v>
+      </c>
+      <c r="O77" s="31" t="n">
+        <v>6.966</v>
+      </c>
+      <c r="P77" s="31" t="n">
+        <v>7.432</v>
+      </c>
+      <c r="Q77" s="34" t="inlineStr">
+        <is>
+          <t>Opp Batter K/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="30" t="inlineStr">
+        <is>
           <t>1st Inn R/G</t>
         </is>
       </c>
-      <c r="B74" s="31" t="n">
+      <c r="B78" s="31" t="n">
         <v>0.629</v>
       </c>
-      <c r="C74" s="31" t="n">
+      <c r="C78" s="31" t="n">
         <v>0.536</v>
       </c>
-      <c r="D74" s="31" t="n">
+      <c r="D78" s="31" t="n">
         <v>0.5</v>
       </c>
-      <c r="E74" s="31" t="n">
+      <c r="E78" s="31" t="n">
         <v>0.6919999999999999</v>
       </c>
-      <c r="F74" s="31" t="n">
+      <c r="F78" s="31" t="n">
         <v>1.125</v>
       </c>
-      <c r="G74" s="31" t="n">
+      <c r="G78" s="31" t="n">
         <v>1.6</v>
       </c>
-      <c r="H74" s="32" t="inlineStr">
+      <c r="H78" s="32" t="inlineStr">
         <is>
           <t>2nd</t>
         </is>
       </c>
-      <c r="I74" s="31" t="inlineStr">
+      <c r="I78" s="31" t="inlineStr">
         <is>
           <t>★</t>
         </is>
       </c>
-      <c r="J74" s="32" t="inlineStr">
+      <c r="J78" s="32" t="inlineStr">
         <is>
           <t>8th</t>
         </is>
       </c>
-      <c r="K74" s="31" t="n">
+      <c r="K78" s="31" t="n">
         <v>0.2</v>
       </c>
-      <c r="L74" s="31" t="n">
+      <c r="L78" s="31" t="n">
         <v>0.111</v>
       </c>
-      <c r="M74" s="31" t="n">
+      <c r="M78" s="31" t="n">
         <v>0.286</v>
       </c>
-      <c r="N74" s="31" t="n">
+      <c r="N78" s="31" t="n">
         <v>0.421</v>
       </c>
-      <c r="O74" s="31" t="n">
+      <c r="O78" s="31" t="n">
         <v>0.483</v>
       </c>
-      <c r="P74" s="31" t="n">
+      <c r="P78" s="31" t="n">
         <v>0.459</v>
       </c>
-      <c r="Q74" s="34" t="inlineStr">
+      <c r="Q78" s="34" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>
@@ -5381,7 +5381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q77"/>
+  <dimension ref="A1:Q74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5398,815 +5398,815 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="28" t="inlineStr">
+        <is>
+          <t>San Diego Padres offense vs Chicago Cubs defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="29" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B61" s="29" t="inlineStr">
+        <is>
+          <t>A Season</t>
+        </is>
+      </c>
+      <c r="C61" s="29" t="inlineStr">
+        <is>
+          <t>A L30</t>
+        </is>
+      </c>
+      <c r="D61" s="29" t="inlineStr">
+        <is>
+          <t>A L20</t>
+        </is>
+      </c>
+      <c r="E61" s="29" t="inlineStr">
+        <is>
+          <t>A L15</t>
+        </is>
+      </c>
+      <c r="F61" s="29" t="inlineStr">
+        <is>
+          <t>A L10</t>
+        </is>
+      </c>
+      <c r="G61" s="29" t="inlineStr">
+        <is>
+          <t>A L5</t>
+        </is>
+      </c>
+      <c r="H61" s="29" t="inlineStr">
+        <is>
+          <t>A Rk</t>
+        </is>
+      </c>
+      <c r="I61" s="29" t="inlineStr">
+        <is>
+          <t>Adv</t>
+        </is>
+      </c>
+      <c r="J61" s="29" t="inlineStr">
+        <is>
+          <t>H Rk</t>
+        </is>
+      </c>
+      <c r="K61" s="29" t="inlineStr">
+        <is>
+          <t>H L5</t>
+        </is>
+      </c>
+      <c r="L61" s="29" t="inlineStr">
+        <is>
+          <t>H L10</t>
+        </is>
+      </c>
+      <c r="M61" s="29" t="inlineStr">
+        <is>
+          <t>H L15</t>
+        </is>
+      </c>
+      <c r="N61" s="29" t="inlineStr">
+        <is>
+          <t>H L20</t>
+        </is>
+      </c>
+      <c r="O61" s="29" t="inlineStr">
+        <is>
+          <t>H L30</t>
+        </is>
+      </c>
+      <c r="P61" s="29" t="inlineStr">
+        <is>
+          <t>H Season</t>
+        </is>
+      </c>
+      <c r="Q61" s="29" t="inlineStr">
+        <is>
+          <t>Opp stat</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="30" t="inlineStr">
+        <is>
+          <t>Runs/G</t>
+        </is>
+      </c>
+      <c r="B62" s="31" t="n">
+        <v>4.279</v>
+      </c>
+      <c r="C62" s="31" t="n">
+        <v>4.433</v>
+      </c>
+      <c r="D62" s="31" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="E62" s="31" t="n">
+        <v>3.733</v>
+      </c>
+      <c r="F62" s="31" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="G62" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="H62" s="35" t="inlineStr">
+        <is>
+          <t>19th</t>
+        </is>
+      </c>
+      <c r="I62" s="31" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="J62" s="33" t="inlineStr">
+        <is>
+          <t>24th</t>
+        </is>
+      </c>
+      <c r="K62" s="31" t="n">
+        <v>5</v>
+      </c>
+      <c r="L62" s="31" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="M62" s="31" t="n">
+        <v>5</v>
+      </c>
+      <c r="N62" s="31" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="O62" s="31" t="n">
+        <v>4.767</v>
+      </c>
+      <c r="P62" s="31" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="Q62" s="34" t="inlineStr">
+        <is>
+          <t>Opp Runs/G</t>
+        </is>
+      </c>
+    </row>
     <row r="63">
-      <c r="A63" s="28" t="inlineStr">
-        <is>
-          <t>San Diego Padres offense vs Chicago Cubs defense</t>
+      <c r="A63" s="30" t="inlineStr">
+        <is>
+          <t>Hits/G</t>
+        </is>
+      </c>
+      <c r="B63" s="31" t="n">
+        <v>7.139</v>
+      </c>
+      <c r="C63" s="31" t="n">
+        <v>7.167</v>
+      </c>
+      <c r="D63" s="31" t="n">
+        <v>6.444</v>
+      </c>
+      <c r="E63" s="31" t="n">
+        <v>6.357</v>
+      </c>
+      <c r="F63" s="31" t="n">
+        <v>5.111</v>
+      </c>
+      <c r="G63" s="31" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="H63" s="33" t="inlineStr">
+        <is>
+          <t>27th</t>
+        </is>
+      </c>
+      <c r="I63" s="31" t="inlineStr"/>
+      <c r="J63" s="33" t="inlineStr">
+        <is>
+          <t>25th</t>
+        </is>
+      </c>
+      <c r="K63" s="31" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="L63" s="31" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="M63" s="31" t="n">
+        <v>8</v>
+      </c>
+      <c r="N63" s="31" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="O63" s="31" t="n">
+        <v>7.966</v>
+      </c>
+      <c r="P63" s="31" t="n">
+        <v>7.595</v>
+      </c>
+      <c r="Q63" s="34" t="inlineStr">
+        <is>
+          <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="29" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="B64" s="29" t="inlineStr">
-        <is>
-          <t>A Season</t>
-        </is>
-      </c>
-      <c r="C64" s="29" t="inlineStr">
-        <is>
-          <t>A L30</t>
-        </is>
-      </c>
-      <c r="D64" s="29" t="inlineStr">
-        <is>
-          <t>A L20</t>
-        </is>
-      </c>
-      <c r="E64" s="29" t="inlineStr">
-        <is>
-          <t>A L15</t>
-        </is>
-      </c>
-      <c r="F64" s="29" t="inlineStr">
-        <is>
-          <t>A L10</t>
-        </is>
-      </c>
-      <c r="G64" s="29" t="inlineStr">
-        <is>
-          <t>A L5</t>
-        </is>
-      </c>
-      <c r="H64" s="29" t="inlineStr">
-        <is>
-          <t>A Rk</t>
-        </is>
-      </c>
-      <c r="I64" s="29" t="inlineStr">
-        <is>
-          <t>Adv</t>
-        </is>
-      </c>
-      <c r="J64" s="29" t="inlineStr">
-        <is>
-          <t>H Rk</t>
-        </is>
-      </c>
-      <c r="K64" s="29" t="inlineStr">
-        <is>
-          <t>H L5</t>
-        </is>
-      </c>
-      <c r="L64" s="29" t="inlineStr">
-        <is>
-          <t>H L10</t>
-        </is>
-      </c>
-      <c r="M64" s="29" t="inlineStr">
-        <is>
-          <t>H L15</t>
-        </is>
-      </c>
-      <c r="N64" s="29" t="inlineStr">
-        <is>
-          <t>H L20</t>
-        </is>
-      </c>
-      <c r="O64" s="29" t="inlineStr">
-        <is>
-          <t>H L30</t>
-        </is>
-      </c>
-      <c r="P64" s="29" t="inlineStr">
-        <is>
-          <t>H Season</t>
-        </is>
-      </c>
-      <c r="Q64" s="29" t="inlineStr">
-        <is>
-          <t>Opp stat</t>
+      <c r="A64" s="30" t="inlineStr">
+        <is>
+          <t>HR/G</t>
+        </is>
+      </c>
+      <c r="B64" s="31" t="n">
+        <v>0.972</v>
+      </c>
+      <c r="C64" s="31" t="n">
+        <v>1.167</v>
+      </c>
+      <c r="D64" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="E64" s="31" t="n">
+        <v>1.286</v>
+      </c>
+      <c r="F64" s="31" t="n">
+        <v>1.111</v>
+      </c>
+      <c r="G64" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H64" s="35" t="inlineStr">
+        <is>
+          <t>15th</t>
+        </is>
+      </c>
+      <c r="I64" s="31" t="inlineStr"/>
+      <c r="J64" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K64" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L64" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M64" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N64" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O64" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P64" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q64" s="34" t="inlineStr">
+        <is>
+          <t>Opp HR/G</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="30" t="inlineStr">
         <is>
-          <t>Runs/G</t>
+          <t>Batter K/G</t>
         </is>
       </c>
       <c r="B65" s="31" t="n">
-        <v>4.279</v>
+        <v>8.138999999999999</v>
       </c>
       <c r="C65" s="31" t="n">
-        <v>4.433</v>
+        <v>8.042</v>
       </c>
       <c r="D65" s="31" t="n">
-        <v>3.55</v>
+        <v>9</v>
       </c>
       <c r="E65" s="31" t="n">
-        <v>3.733</v>
+        <v>8.714</v>
       </c>
       <c r="F65" s="31" t="n">
-        <v>2.9</v>
+        <v>7.889</v>
       </c>
       <c r="G65" s="31" t="n">
-        <v>3</v>
-      </c>
-      <c r="H65" s="35" t="inlineStr">
-        <is>
-          <t>19th</t>
+        <v>7.2</v>
+      </c>
+      <c r="H65" s="32" t="inlineStr">
+        <is>
+          <t>5th</t>
         </is>
       </c>
       <c r="I65" s="31" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="J65" s="33" t="inlineStr">
         <is>
-          <t>24th</t>
+          <t>25th</t>
         </is>
       </c>
       <c r="K65" s="31" t="n">
-        <v>5</v>
+        <v>7.4</v>
       </c>
       <c r="L65" s="31" t="n">
-        <v>4.6</v>
+        <v>7.3</v>
       </c>
       <c r="M65" s="31" t="n">
-        <v>5</v>
+        <v>7.2</v>
       </c>
       <c r="N65" s="31" t="n">
-        <v>4.25</v>
+        <v>7.35</v>
       </c>
       <c r="O65" s="31" t="n">
-        <v>4.767</v>
+        <v>7.552</v>
       </c>
       <c r="P65" s="31" t="n">
-        <v>4.5</v>
+        <v>7.838</v>
       </c>
       <c r="Q65" s="34" t="inlineStr">
         <is>
-          <t>Opp Runs/G</t>
+          <t>Opp Batter K/G</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="30" t="inlineStr">
         <is>
+          <t>1st Inn R/G</t>
+        </is>
+      </c>
+      <c r="B66" s="31" t="n">
+        <v>0.222</v>
+      </c>
+      <c r="C66" s="31" t="n">
+        <v>0.292</v>
+      </c>
+      <c r="D66" s="31" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="E66" s="31" t="n">
+        <v>0.429</v>
+      </c>
+      <c r="F66" s="31" t="n">
+        <v>0.556</v>
+      </c>
+      <c r="G66" s="31" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H66" s="35" t="inlineStr">
+        <is>
+          <t>11th</t>
+        </is>
+      </c>
+      <c r="I66" s="31" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J66" s="33" t="inlineStr">
+        <is>
+          <t>28th</t>
+        </is>
+      </c>
+      <c r="K66" s="31" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="L66" s="31" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="M66" s="31" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="N66" s="31" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O66" s="31" t="n">
+        <v>0.414</v>
+      </c>
+      <c r="P66" s="31" t="n">
+        <v>0.405</v>
+      </c>
+      <c r="Q66" s="34" t="inlineStr">
+        <is>
+          <t>Opp 1st Inn R/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="28" t="inlineStr">
+        <is>
+          <t>Chicago Cubs offense vs San Diego Padres defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="29" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="B69" s="29" t="inlineStr">
+        <is>
+          <t>A Season</t>
+        </is>
+      </c>
+      <c r="C69" s="29" t="inlineStr">
+        <is>
+          <t>A L30</t>
+        </is>
+      </c>
+      <c r="D69" s="29" t="inlineStr">
+        <is>
+          <t>A L20</t>
+        </is>
+      </c>
+      <c r="E69" s="29" t="inlineStr">
+        <is>
+          <t>A L15</t>
+        </is>
+      </c>
+      <c r="F69" s="29" t="inlineStr">
+        <is>
+          <t>A L10</t>
+        </is>
+      </c>
+      <c r="G69" s="29" t="inlineStr">
+        <is>
+          <t>A L5</t>
+        </is>
+      </c>
+      <c r="H69" s="29" t="inlineStr">
+        <is>
+          <t>A Rk</t>
+        </is>
+      </c>
+      <c r="I69" s="29" t="inlineStr">
+        <is>
+          <t>Adv</t>
+        </is>
+      </c>
+      <c r="J69" s="29" t="inlineStr">
+        <is>
+          <t>H Rk</t>
+        </is>
+      </c>
+      <c r="K69" s="29" t="inlineStr">
+        <is>
+          <t>H L5</t>
+        </is>
+      </c>
+      <c r="L69" s="29" t="inlineStr">
+        <is>
+          <t>H L10</t>
+        </is>
+      </c>
+      <c r="M69" s="29" t="inlineStr">
+        <is>
+          <t>H L15</t>
+        </is>
+      </c>
+      <c r="N69" s="29" t="inlineStr">
+        <is>
+          <t>H L20</t>
+        </is>
+      </c>
+      <c r="O69" s="29" t="inlineStr">
+        <is>
+          <t>H L30</t>
+        </is>
+      </c>
+      <c r="P69" s="29" t="inlineStr">
+        <is>
+          <t>H Season</t>
+        </is>
+      </c>
+      <c r="Q69" s="29" t="inlineStr">
+        <is>
+          <t>Opp stat</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="30" t="inlineStr">
+        <is>
+          <t>Runs/G</t>
+        </is>
+      </c>
+      <c r="B70" s="31" t="n">
+        <v>4.947</v>
+      </c>
+      <c r="C70" s="31" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="D70" s="31" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="E70" s="31" t="n">
+        <v>4.267</v>
+      </c>
+      <c r="F70" s="31" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="G70" s="31" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H70" s="33" t="inlineStr">
+        <is>
+          <t>30th</t>
+        </is>
+      </c>
+      <c r="I70" s="31" t="inlineStr"/>
+      <c r="J70" s="32" t="inlineStr">
+        <is>
+          <t>4th</t>
+        </is>
+      </c>
+      <c r="K70" s="31" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="L70" s="31" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="M70" s="31" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="N70" s="31" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="O70" s="31" t="n">
+        <v>3.667</v>
+      </c>
+      <c r="P70" s="31" t="n">
+        <v>3.674</v>
+      </c>
+      <c r="Q70" s="34" t="inlineStr">
+        <is>
+          <t>Opp Runs/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="30" t="inlineStr">
+        <is>
           <t>Hits/G</t>
         </is>
       </c>
-      <c r="B66" s="31" t="n">
-        <v>7.139</v>
-      </c>
-      <c r="C66" s="31" t="n">
-        <v>7.167</v>
-      </c>
-      <c r="D66" s="31" t="n">
-        <v>6.444</v>
-      </c>
-      <c r="E66" s="31" t="n">
-        <v>6.357</v>
-      </c>
-      <c r="F66" s="31" t="n">
-        <v>5.111</v>
-      </c>
-      <c r="G66" s="31" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="H66" s="33" t="inlineStr">
-        <is>
-          <t>27th</t>
-        </is>
-      </c>
-      <c r="I66" s="31" t="inlineStr"/>
-      <c r="J66" s="33" t="inlineStr">
-        <is>
-          <t>25th</t>
-        </is>
-      </c>
-      <c r="K66" s="31" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="L66" s="31" t="n">
-        <v>7.7</v>
-      </c>
-      <c r="M66" s="31" t="n">
-        <v>8</v>
-      </c>
-      <c r="N66" s="31" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="O66" s="31" t="n">
-        <v>7.966</v>
-      </c>
-      <c r="P66" s="31" t="n">
-        <v>7.595</v>
-      </c>
-      <c r="Q66" s="34" t="inlineStr">
+      <c r="B71" s="31" t="n">
+        <v>8.432</v>
+      </c>
+      <c r="C71" s="31" t="n">
+        <v>8.965999999999999</v>
+      </c>
+      <c r="D71" s="31" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="E71" s="31" t="n">
+        <v>8.333</v>
+      </c>
+      <c r="F71" s="31" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="G71" s="31" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="H71" s="33" t="inlineStr">
+        <is>
+          <t>30th</t>
+        </is>
+      </c>
+      <c r="I71" s="31" t="inlineStr"/>
+      <c r="J71" s="35" t="inlineStr">
+        <is>
+          <t>19th</t>
+        </is>
+      </c>
+      <c r="K71" s="31" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="L71" s="31" t="n">
+        <v>7.778</v>
+      </c>
+      <c r="M71" s="31" t="n">
+        <v>8.856999999999999</v>
+      </c>
+      <c r="N71" s="31" t="n">
+        <v>8.444000000000001</v>
+      </c>
+      <c r="O71" s="31" t="n">
+        <v>8.125</v>
+      </c>
+      <c r="P71" s="31" t="n">
+        <v>8.111000000000001</v>
+      </c>
+      <c r="Q71" s="34" t="inlineStr">
         <is>
           <t>Opp Hits/G</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="30" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="30" t="inlineStr">
         <is>
           <t>HR/G</t>
         </is>
       </c>
-      <c r="B67" s="31" t="n">
-        <v>0.972</v>
-      </c>
-      <c r="C67" s="31" t="n">
-        <v>1.167</v>
-      </c>
-      <c r="D67" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="E67" s="31" t="n">
-        <v>1.286</v>
-      </c>
-      <c r="F67" s="31" t="n">
-        <v>1.111</v>
-      </c>
-      <c r="G67" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="H67" s="35" t="inlineStr">
-        <is>
-          <t>15th</t>
-        </is>
-      </c>
-      <c r="I67" s="31" t="inlineStr"/>
-      <c r="J67" s="34" t="inlineStr">
+      <c r="B72" s="31" t="n">
+        <v>1.135</v>
+      </c>
+      <c r="C72" s="31" t="n">
+        <v>1.241</v>
+      </c>
+      <c r="D72" s="31" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="E72" s="31" t="n">
+        <v>1.133</v>
+      </c>
+      <c r="F72" s="31" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G72" s="31" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H72" s="33" t="inlineStr">
+        <is>
+          <t>24th</t>
+        </is>
+      </c>
+      <c r="I72" s="31" t="inlineStr"/>
+      <c r="J72" s="34" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K67" s="31" t="inlineStr">
+      <c r="K72" s="31" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L67" s="31" t="inlineStr">
+      <c r="L72" s="31" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M67" s="31" t="inlineStr">
+      <c r="M72" s="31" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N67" s="31" t="inlineStr">
+      <c r="N72" s="31" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="O67" s="31" t="inlineStr">
+      <c r="O72" s="31" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="P67" s="31" t="inlineStr">
+      <c r="P72" s="31" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Q67" s="34" t="inlineStr">
+      <c r="Q72" s="34" t="inlineStr">
         <is>
           <t>Opp HR/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="30" t="inlineStr">
-        <is>
-          <t>Batter K/G</t>
-        </is>
-      </c>
-      <c r="B68" s="31" t="n">
-        <v>8.138999999999999</v>
-      </c>
-      <c r="C68" s="31" t="n">
-        <v>8.042</v>
-      </c>
-      <c r="D68" s="31" t="n">
-        <v>9</v>
-      </c>
-      <c r="E68" s="31" t="n">
-        <v>8.714</v>
-      </c>
-      <c r="F68" s="31" t="n">
-        <v>7.889</v>
-      </c>
-      <c r="G68" s="31" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="H68" s="32" t="inlineStr">
-        <is>
-          <t>5th</t>
-        </is>
-      </c>
-      <c r="I68" s="31" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J68" s="33" t="inlineStr">
-        <is>
-          <t>25th</t>
-        </is>
-      </c>
-      <c r="K68" s="31" t="n">
-        <v>7.4</v>
-      </c>
-      <c r="L68" s="31" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="M68" s="31" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="N68" s="31" t="n">
-        <v>7.35</v>
-      </c>
-      <c r="O68" s="31" t="n">
-        <v>7.552</v>
-      </c>
-      <c r="P68" s="31" t="n">
-        <v>7.838</v>
-      </c>
-      <c r="Q68" s="34" t="inlineStr">
-        <is>
-          <t>Opp Batter K/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="30" t="inlineStr">
-        <is>
-          <t>1st Inn R/G</t>
-        </is>
-      </c>
-      <c r="B69" s="31" t="n">
-        <v>0.222</v>
-      </c>
-      <c r="C69" s="31" t="n">
-        <v>0.292</v>
-      </c>
-      <c r="D69" s="31" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="E69" s="31" t="n">
-        <v>0.429</v>
-      </c>
-      <c r="F69" s="31" t="n">
-        <v>0.556</v>
-      </c>
-      <c r="G69" s="31" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="H69" s="35" t="inlineStr">
-        <is>
-          <t>11th</t>
-        </is>
-      </c>
-      <c r="I69" s="31" t="inlineStr">
-        <is>
-          <t>★★★</t>
-        </is>
-      </c>
-      <c r="J69" s="33" t="inlineStr">
-        <is>
-          <t>28th</t>
-        </is>
-      </c>
-      <c r="K69" s="31" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="L69" s="31" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="M69" s="31" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="N69" s="31" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="O69" s="31" t="n">
-        <v>0.414</v>
-      </c>
-      <c r="P69" s="31" t="n">
-        <v>0.405</v>
-      </c>
-      <c r="Q69" s="34" t="inlineStr">
-        <is>
-          <t>Opp 1st Inn R/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="28" t="inlineStr">
-        <is>
-          <t>Chicago Cubs offense vs San Diego Padres defense</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="29" t="inlineStr">
-        <is>
-          <t>Stat</t>
-        </is>
-      </c>
-      <c r="B72" s="29" t="inlineStr">
-        <is>
-          <t>A Season</t>
-        </is>
-      </c>
-      <c r="C72" s="29" t="inlineStr">
-        <is>
-          <t>A L30</t>
-        </is>
-      </c>
-      <c r="D72" s="29" t="inlineStr">
-        <is>
-          <t>A L20</t>
-        </is>
-      </c>
-      <c r="E72" s="29" t="inlineStr">
-        <is>
-          <t>A L15</t>
-        </is>
-      </c>
-      <c r="F72" s="29" t="inlineStr">
-        <is>
-          <t>A L10</t>
-        </is>
-      </c>
-      <c r="G72" s="29" t="inlineStr">
-        <is>
-          <t>A L5</t>
-        </is>
-      </c>
-      <c r="H72" s="29" t="inlineStr">
-        <is>
-          <t>A Rk</t>
-        </is>
-      </c>
-      <c r="I72" s="29" t="inlineStr">
-        <is>
-          <t>Adv</t>
-        </is>
-      </c>
-      <c r="J72" s="29" t="inlineStr">
-        <is>
-          <t>H Rk</t>
-        </is>
-      </c>
-      <c r="K72" s="29" t="inlineStr">
-        <is>
-          <t>H L5</t>
-        </is>
-      </c>
-      <c r="L72" s="29" t="inlineStr">
-        <is>
-          <t>H L10</t>
-        </is>
-      </c>
-      <c r="M72" s="29" t="inlineStr">
-        <is>
-          <t>H L15</t>
-        </is>
-      </c>
-      <c r="N72" s="29" t="inlineStr">
-        <is>
-          <t>H L20</t>
-        </is>
-      </c>
-      <c r="O72" s="29" t="inlineStr">
-        <is>
-          <t>H L30</t>
-        </is>
-      </c>
-      <c r="P72" s="29" t="inlineStr">
-        <is>
-          <t>H Season</t>
-        </is>
-      </c>
-      <c r="Q72" s="29" t="inlineStr">
-        <is>
-          <t>Opp stat</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="30" t="inlineStr">
         <is>
-          <t>Runs/G</t>
+          <t>Batter K/G</t>
         </is>
       </c>
       <c r="B73" s="31" t="n">
-        <v>4.947</v>
+        <v>8.541</v>
       </c>
       <c r="C73" s="31" t="n">
-        <v>5.2</v>
+        <v>8.516999999999999</v>
       </c>
       <c r="D73" s="31" t="n">
-        <v>4.9</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="E73" s="31" t="n">
-        <v>4.267</v>
+        <v>8.6</v>
       </c>
       <c r="F73" s="31" t="n">
-        <v>3.2</v>
+        <v>8.5</v>
       </c>
       <c r="G73" s="31" t="n">
-        <v>1.4</v>
+        <v>10</v>
       </c>
       <c r="H73" s="33" t="inlineStr">
         <is>
-          <t>30th</t>
+          <t>25th</t>
         </is>
       </c>
       <c r="I73" s="31" t="inlineStr"/>
-      <c r="J73" s="32" t="inlineStr">
-        <is>
-          <t>4th</t>
+      <c r="J73" s="33" t="inlineStr">
+        <is>
+          <t>24th</t>
         </is>
       </c>
       <c r="K73" s="31" t="n">
-        <v>2.4</v>
+        <v>7.4</v>
       </c>
       <c r="L73" s="31" t="n">
-        <v>3.4</v>
+        <v>8.333</v>
       </c>
       <c r="M73" s="31" t="n">
-        <v>4.4</v>
+        <v>7.5</v>
       </c>
       <c r="N73" s="31" t="n">
-        <v>3.95</v>
+        <v>8.167</v>
       </c>
       <c r="O73" s="31" t="n">
-        <v>3.667</v>
+        <v>8.708</v>
       </c>
       <c r="P73" s="31" t="n">
-        <v>3.674</v>
+        <v>8.805999999999999</v>
       </c>
       <c r="Q73" s="34" t="inlineStr">
         <is>
-          <t>Opp Runs/G</t>
+          <t>Opp Batter K/G</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="30" t="inlineStr">
         <is>
-          <t>Hits/G</t>
+          <t>1st Inn R/G</t>
         </is>
       </c>
       <c r="B74" s="31" t="n">
-        <v>8.432</v>
+        <v>0.297</v>
       </c>
       <c r="C74" s="31" t="n">
-        <v>8.965999999999999</v>
+        <v>0.276</v>
       </c>
       <c r="D74" s="31" t="n">
-        <v>8.699999999999999</v>
+        <v>0.35</v>
       </c>
       <c r="E74" s="31" t="n">
-        <v>8.333</v>
+        <v>0.2</v>
       </c>
       <c r="F74" s="31" t="n">
-        <v>6.2</v>
+        <v>0.2</v>
       </c>
       <c r="G74" s="31" t="n">
-        <v>4.6</v>
+        <v>0</v>
       </c>
       <c r="H74" s="33" t="inlineStr">
         <is>
-          <t>30th</t>
+          <t>29th</t>
         </is>
       </c>
       <c r="I74" s="31" t="inlineStr"/>
-      <c r="J74" s="35" t="inlineStr">
-        <is>
-          <t>19th</t>
+      <c r="J74" s="33" t="inlineStr">
+        <is>
+          <t>25th</t>
         </is>
       </c>
       <c r="K74" s="31" t="n">
-        <v>7.8</v>
+        <v>1</v>
       </c>
       <c r="L74" s="31" t="n">
-        <v>7.778</v>
+        <v>0.556</v>
       </c>
       <c r="M74" s="31" t="n">
-        <v>8.856999999999999</v>
+        <v>0.429</v>
       </c>
       <c r="N74" s="31" t="n">
-        <v>8.444000000000001</v>
+        <v>0.333</v>
       </c>
       <c r="O74" s="31" t="n">
-        <v>8.125</v>
+        <v>0.333</v>
       </c>
       <c r="P74" s="31" t="n">
-        <v>8.111000000000001</v>
+        <v>0.417</v>
       </c>
       <c r="Q74" s="34" t="inlineStr">
-        <is>
-          <t>Opp Hits/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="30" t="inlineStr">
-        <is>
-          <t>HR/G</t>
-        </is>
-      </c>
-      <c r="B75" s="31" t="n">
-        <v>1.135</v>
-      </c>
-      <c r="C75" s="31" t="n">
-        <v>1.241</v>
-      </c>
-      <c r="D75" s="31" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="E75" s="31" t="n">
-        <v>1.133</v>
-      </c>
-      <c r="F75" s="31" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G75" s="31" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H75" s="33" t="inlineStr">
-        <is>
-          <t>24th</t>
-        </is>
-      </c>
-      <c r="I75" s="31" t="inlineStr"/>
-      <c r="J75" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K75" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L75" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M75" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N75" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O75" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P75" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q75" s="34" t="inlineStr">
-        <is>
-          <t>Opp HR/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="30" t="inlineStr">
-        <is>
-          <t>Batter K/G</t>
-        </is>
-      </c>
-      <c r="B76" s="31" t="n">
-        <v>8.541</v>
-      </c>
-      <c r="C76" s="31" t="n">
-        <v>8.516999999999999</v>
-      </c>
-      <c r="D76" s="31" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="E76" s="31" t="n">
-        <v>8.6</v>
-      </c>
-      <c r="F76" s="31" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="G76" s="31" t="n">
-        <v>10</v>
-      </c>
-      <c r="H76" s="33" t="inlineStr">
-        <is>
-          <t>25th</t>
-        </is>
-      </c>
-      <c r="I76" s="31" t="inlineStr"/>
-      <c r="J76" s="33" t="inlineStr">
-        <is>
-          <t>24th</t>
-        </is>
-      </c>
-      <c r="K76" s="31" t="n">
-        <v>7.4</v>
-      </c>
-      <c r="L76" s="31" t="n">
-        <v>8.333</v>
-      </c>
-      <c r="M76" s="31" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="N76" s="31" t="n">
-        <v>8.167</v>
-      </c>
-      <c r="O76" s="31" t="n">
-        <v>8.708</v>
-      </c>
-      <c r="P76" s="31" t="n">
-        <v>8.805999999999999</v>
-      </c>
-      <c r="Q76" s="34" t="inlineStr">
-        <is>
-          <t>Opp Batter K/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="30" t="inlineStr">
-        <is>
-          <t>1st Inn R/G</t>
-        </is>
-      </c>
-      <c r="B77" s="31" t="n">
-        <v>0.297</v>
-      </c>
-      <c r="C77" s="31" t="n">
-        <v>0.276</v>
-      </c>
-      <c r="D77" s="31" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="E77" s="31" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F77" s="31" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G77" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="H77" s="33" t="inlineStr">
-        <is>
-          <t>29th</t>
-        </is>
-      </c>
-      <c r="I77" s="31" t="inlineStr"/>
-      <c r="J77" s="33" t="inlineStr">
-        <is>
-          <t>25th</t>
-        </is>
-      </c>
-      <c r="K77" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="L77" s="31" t="n">
-        <v>0.556</v>
-      </c>
-      <c r="M77" s="31" t="n">
-        <v>0.429</v>
-      </c>
-      <c r="N77" s="31" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="O77" s="31" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="P77" s="31" t="n">
-        <v>0.417</v>
-      </c>
-      <c r="Q77" s="34" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>
@@ -7995,7 +7995,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P22"/>
+  <dimension ref="A1:P21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8139,13 +8139,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.5502970297029702</v>
+        <v>0.554</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-122</v>
+        <v>-124</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -8169,7 +8169,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 55.0% (fair -122). Your call.</t>
+          <t>Model 55.4% (fair -124). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -8205,7 +8205,7 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.4879295154185022</v>
+        <v>0.4875330396475771</v>
       </c>
       <c r="G6" s="14" t="n">
         <v>105</v>
@@ -8271,13 +8271,13 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.6443409836065574</v>
+        <v>0.6433344398340248</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-181</v>
+        <v>-180</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>-144</v>
+        <v>-141</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -8301,7 +8301,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 64.4% (fair -181). Your call.</t>
+          <t>Model 64.3% (fair -180). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -8313,17 +8313,17 @@
     <row r="8">
       <c r="A8" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>Minnesota Twins @ Houston Astros</t>
+          <t>Tampa Bay Rays @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="D8" s="20" t="inlineStr">
@@ -8333,17 +8333,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.4803964757709251</v>
+        <v>0.5051851851851852</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>108</v>
+        <v>-102</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -8367,7 +8367,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 48.0% (fair +108). Your call.</t>
+          <t>Model 50.5% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -8379,17 +8379,17 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Texas Rangers @ Cleveland Guardians</t>
+          <t>Minnesota Twins @ Houston Astros</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>22:40</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -8399,17 +8399,17 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.5318627450980392</v>
+        <v>0.4803964757709251</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-114</v>
+        <v>108</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>104</v>
+        <v>127</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -8433,7 +8433,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 53.2% (fair -114). Your call.</t>
+          <t>Model 48.0% (fair +108). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -8450,12 +8450,12 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Kansas City Royals</t>
+          <t>Texas Rangers @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>23:40</t>
+          <t>22:40</t>
         </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
@@ -8465,17 +8465,17 @@
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.5011627906976744</v>
+        <v>0.534264705882353</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-100</v>
+        <v>-115</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -8499,7 +8499,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 50.1% (fair -100). Your call.</t>
+          <t>Model 53.4% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -8535,13 +8535,13 @@
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.4633913043478262</v>
+        <v>0.4607659574468085</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -8565,7 +8565,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 46.3% (fair +116). Your call.</t>
+          <t>Model 46.1% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -8582,12 +8582,12 @@
       </c>
       <c r="B12" s="20" t="inlineStr">
         <is>
-          <t>New York Mets @ Toronto Blue Jays</t>
+          <t>Pittsburgh Pirates @ Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
         <is>
-          <t>23:07</t>
+          <t>22:40</t>
         </is>
       </c>
       <c r="D12" s="20" t="inlineStr">
@@ -8597,17 +8597,17 @@
       </c>
       <c r="E12" s="20" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.4800900900900902</v>
+        <v>0.383273381294964</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>108</v>
+        <v>161</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>122</v>
+        <v>178</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -8631,7 +8631,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 48.0% (fair +108). Your call.</t>
+          <t>Model 38.3% (fair +161). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -8643,17 +8643,17 @@
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Philadelphia Phillies</t>
+          <t>New York Mets @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>22:40</t>
+          <t>23:07</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
@@ -8663,17 +8663,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.3814748201438848</v>
+        <v>0.4869124423963134</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>162</v>
+        <v>105</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>178</v>
+        <v>117</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -8697,7 +8697,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 38.1% (fair +162). Your call.</t>
+          <t>Model 48.7% (fair +105). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -8714,12 +8714,12 @@
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>New York Mets @ Toronto Blue Jays</t>
+          <t>Detroit Tigers @ New York Yankees</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>23:07</t>
+          <t>23:05</t>
         </is>
       </c>
       <c r="D14" s="20" t="inlineStr">
@@ -8729,17 +8729,17 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4849769585253456</v>
+        <v>0.4528755364806866</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>117</v>
+        <v>133</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -8763,7 +8763,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 48.5% (fair +106). Your call.</t>
+          <t>Model 45.3% (fair +121). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -8841,17 +8841,17 @@
     <row r="16">
       <c r="A16" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Chicago Cubs</t>
+          <t>St. Louis Cardinals @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>00:05</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="D16" s="20" t="inlineStr">
@@ -8861,17 +8861,17 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>St. Louis Cardinals</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.4308298755186722</v>
+        <v>0.4469957081545065</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -8895,7 +8895,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 43.1% (fair +132). Your call.</t>
+          <t>Model 44.7% (fair +124). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -8912,12 +8912,12 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>Detroit Tigers @ New York Yankees</t>
+          <t>Chicago White Sox @ Baltimore Orioles</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>23:05</t>
+          <t>22:35</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -8927,17 +8927,17 @@
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.456079295154185</v>
+        <v>0.4603111111111111</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -8961,7 +8961,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 45.6% (fair +119). Your call.</t>
+          <t>Model 46.0% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -8973,17 +8973,17 @@
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>Detroit Tigers @ New York Yankees</t>
+          <t>San Diego Padres @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
-          <t>23:05</t>
+          <t>00:05</t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
@@ -8993,17 +8993,17 @@
       </c>
       <c r="E18" s="20" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5888532188841202</v>
+        <v>0.4344957983193278</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-143</v>
+        <v>130</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>-133</v>
+        <v>138</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -9027,7 +9027,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 58.9% (fair -143). Your call.</t>
+          <t>Model 43.4% (fair +130). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -9039,17 +9039,17 @@
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Baltimore Orioles</t>
+          <t>Detroit Tigers @ New York Yankees</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>22:35</t>
+          <t>23:05</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -9059,17 +9059,17 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.462286995515695</v>
+        <v>0.5899377682403434</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>116</v>
+        <v>-144</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>123</v>
+        <v>-133</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -9093,7 +9093,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 46.2% (fair +116). Your call.</t>
+          <t>Model 59.0% (fair -144). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -9110,12 +9110,12 @@
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Milwaukee Brewers</t>
+          <t>San Diego Padres @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C20" s="20" t="inlineStr">
         <is>
-          <t>23:40</t>
+          <t>00:05</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
@@ -9125,17 +9125,17 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.638612927756654</v>
+        <v>0.5867982832618026</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>-177</v>
+        <v>-142</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>-163</v>
+        <v>-133</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -9159,7 +9159,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 63.9% (fair -177). Your call.</t>
+          <t>Model 58.7% (fair -142). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -9171,37 +9171,37 @@
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Chicago Cubs</t>
+          <t>Cincinnati Reds @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>00:05</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>San Diego Padres +1.5</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.5796304347826088</v>
+        <v>0.6435444444444444</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>-138</v>
+        <v>-181</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>-130</v>
+        <v>-170</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -9225,7 +9225,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 58.0% (fair -138). Your call.</t>
+          <t>Model 64.4% (fair -181). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -9234,75 +9234,9 @@
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="20" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="B22" s="20" t="inlineStr">
-        <is>
-          <t>San Diego Padres @ Chicago Cubs</t>
-        </is>
-      </c>
-      <c r="C22" s="20" t="inlineStr">
-        <is>
-          <t>00:05</t>
-        </is>
-      </c>
-      <c r="D22" s="20" t="inlineStr">
-        <is>
-          <t>Moneyline</t>
-        </is>
-      </c>
-      <c r="E22" s="20" t="inlineStr">
-        <is>
-          <t>Chicago Cubs</t>
-        </is>
-      </c>
-      <c r="F22" s="13" t="n">
-        <v>0.5836017167381974</v>
-      </c>
-      <c r="G22" s="14" t="n">
-        <v>-140</v>
-      </c>
-      <c r="H22" s="15" t="n">
-        <v>-133</v>
-      </c>
-      <c r="I22" s="13">
-        <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
-        <v/>
-      </c>
-      <c r="J22" s="16">
-        <f>IF($H$22="","",$F$22*IF($H$22&lt;0,-100/$H$22,$H$22/100)-(1-$F$22))</f>
-        <v/>
-      </c>
-      <c r="K22" s="17">
-        <f>IF($H$22="","",MAX(0,($F$22*IF($H$22&lt;0,-100/$H$22,$H$22/100)-(1-$F$22))/IF($H$22&lt;0,-100/$H$22,$H$22/100))*'Settings'!$B$3)</f>
-        <v/>
-      </c>
-      <c r="L22" s="18">
-        <f>IF($H$22="","",ROUND(MIN($K$22,'Settings'!$B$5)*'Settings'!$B$2,2))</f>
-        <v/>
-      </c>
-      <c r="M22" s="12">
-        <f>IF($J$22="","",IF($J$22&lt;0,"Pass",IF($J$22&lt;'Settings'!$B$4,"Thin",IF($J$22&lt;0.06,"✅ Sharp band",IF($J$22&lt;0.08,"Strong","⚠ Verify (stale?)")))))</f>
-        <v/>
-      </c>
-      <c r="N22" s="19" t="inlineStr">
-        <is>
-          <t>Model 58.4% (fair -140). Your call.</t>
-        </is>
-      </c>
-      <c r="O22" s="15" t="n"/>
-      <c r="P22" s="16">
-        <f>IF(OR($H$22="",$O$22=""),"",(1+IF($H$22&lt;0,-100/$H$22,$H$22/100))/(1+IF($O$22&lt;0,-100/$O$22,$O$22/100))-1)</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CE4B"/>
-  <conditionalFormatting sqref="J5:J22">
+  <conditionalFormatting sqref="J5:J21">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="-0.05"/>
@@ -9468,13 +9402,13 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.462286995515695</v>
+        <v>0.4603111111111111</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -9498,7 +9432,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 46.2% (fair +116). Your call.</t>
+          <t>Model 46.0% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -9534,13 +9468,13 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.5377222222222222</v>
+        <v>0.5397220264317181</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-116</v>
+        <v>-117</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>-125</v>
+        <v>-127</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -9564,7 +9498,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 53.8% (fair -116). Your call.</t>
+          <t>Model 54.0% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -9596,7 +9530,7 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 9</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
@@ -9606,7 +9540,7 @@
         <v>110</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -9662,7 +9596,7 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Under 9</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
@@ -9672,7 +9606,7 @@
         <v>-110</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -9804,7 +9738,7 @@
         <v>-155</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -9864,13 +9798,13 @@
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.5502970297029702</v>
+        <v>0.554</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-122</v>
+        <v>-124</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -9894,7 +9828,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 55.0% (fair -122). Your call.</t>
+          <t>Model 55.4% (fair -124). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -9930,13 +9864,13 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.4497089108910891</v>
+        <v>0.445990099009901</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>-102</v>
+        <v>102</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -9960,7 +9894,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 45.0% (fair +122). Your call.</t>
+          <t>Model 44.6% (fair +124). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -9992,17 +9926,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Over 9</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.4931</v>
+        <v>0.5928</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>103</v>
+        <v>-146</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -10026,7 +9960,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 49.3% (fair +103). Your call.</t>
+          <t>Model 59.3% (fair -146). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -10058,17 +9992,17 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Under 9</t>
+          <t>Under 8.5</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.5069</v>
+        <v>0.4072</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>-103</v>
+        <v>146</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>100</v>
+        <v>118</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -10092,7 +10026,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 50.7% (fair -103). Your call.</t>
+          <t>Model 40.7% (fair +146). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -10134,7 +10068,7 @@
         <v>255</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -10200,7 +10134,7 @@
         <v>-255</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -10260,13 +10194,13 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.456079295154185</v>
+        <v>0.4528755364806866</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -10290,7 +10224,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 45.6% (fair +119). Your call.</t>
+          <t>Model 45.3% (fair +121). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -10326,10 +10260,10 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5439300429184549</v>
+        <v>0.5471266094420602</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-119</v>
+        <v>-121</v>
       </c>
       <c r="H18" s="15" t="n">
         <v>-133</v>
@@ -10356,7 +10290,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 54.4% (fair -119). Your call.</t>
+          <t>Model 54.7% (fair -121). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -10398,7 +10332,7 @@
         <v>106</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -10656,10 +10590,10 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.4849769585253456</v>
+        <v>0.4869124423963134</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H23" s="15" t="n">
         <v>117</v>
@@ -10686,7 +10620,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 48.5% (fair +106). Your call.</t>
+          <t>Model 48.7% (fair +105). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -10722,13 +10656,13 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5150181818181818</v>
+        <v>0.5130851851851852</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-106</v>
+        <v>-105</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>-120</v>
+        <v>-116</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -10752,7 +10686,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 51.5% (fair -106). Your call.</t>
+          <t>Model 51.3% (fair -105). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -10794,7 +10728,7 @@
         <v>133</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>108</v>
+        <v>-104</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -10860,7 +10794,7 @@
         <v>-133</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -11058,7 +10992,7 @@
         <v>157</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -11124,7 +11058,7 @@
         <v>-157</v>
       </c>
       <c r="H30" s="15" t="n">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="I30" s="13">
         <f>IF($H$30="","",IF($H$30&lt;0,-$H$30/(-$H$30+100),100/($H$30+100)))</f>
@@ -11180,7 +11114,7 @@
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
-          <t>Over 9</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="F31" s="13" t="n">
@@ -11190,7 +11124,7 @@
         <v>109</v>
       </c>
       <c r="H31" s="15" t="n">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="I31" s="13">
         <f>IF($H$31="","",IF($H$31&lt;0,-$H$31/(-$H$31+100),100/($H$31+100)))</f>
@@ -11246,7 +11180,7 @@
       </c>
       <c r="E32" s="20" t="inlineStr">
         <is>
-          <t>Under 9</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F32" s="13" t="n">
@@ -11256,7 +11190,7 @@
         <v>-109</v>
       </c>
       <c r="H32" s="15" t="n">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="I32" s="13">
         <f>IF($H$32="","",IF($H$32&lt;0,-$H$32/(-$H$32+100),100/($H$32+100)))</f>
@@ -11322,7 +11256,7 @@
         <v>111</v>
       </c>
       <c r="H33" s="15" t="n">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="I33" s="13">
         <f>IF($H$33="","",IF($H$33&lt;0,-$H$33/(-$H$33+100),100/($H$33+100)))</f>
@@ -11388,7 +11322,7 @@
         <v>-111</v>
       </c>
       <c r="H34" s="15" t="n">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="I34" s="13">
         <f>IF($H$34="","",IF($H$34&lt;0,-$H$34/(-$H$34+100),100/($H$34+100)))</f>
@@ -11448,13 +11382,13 @@
         </is>
       </c>
       <c r="F35" s="13" t="n">
-        <v>0.4633913043478262</v>
+        <v>0.4607659574468085</v>
       </c>
       <c r="G35" s="14" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H35" s="15" t="n">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="I35" s="13">
         <f>IF($H$35="","",IF($H$35&lt;0,-$H$35/(-$H$35+100),100/($H$35+100)))</f>
@@ -11478,7 +11412,7 @@
       </c>
       <c r="N35" s="19" t="inlineStr">
         <is>
-          <t>Model 46.3% (fair +116). Your call.</t>
+          <t>Model 46.1% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O35" s="15" t="n"/>
@@ -11514,10 +11448,10 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.5366236051502147</v>
+        <v>0.5392493562231759</v>
       </c>
       <c r="G36" s="14" t="n">
-        <v>-116</v>
+        <v>-117</v>
       </c>
       <c r="H36" s="15" t="n">
         <v>-133</v>
@@ -11544,7 +11478,7 @@
       </c>
       <c r="N36" s="19" t="inlineStr">
         <is>
-          <t>Model 53.7% (fair -116). Your call.</t>
+          <t>Model 53.9% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O36" s="15" t="n"/>
@@ -11586,7 +11520,7 @@
         <v>161</v>
       </c>
       <c r="H37" s="15" t="n">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="I37" s="13">
         <f>IF($H$37="","",IF($H$37&lt;0,-$H$37/(-$H$37+100),100/($H$37+100)))</f>
@@ -11652,7 +11586,7 @@
         <v>-161</v>
       </c>
       <c r="H38" s="15" t="n">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="I38" s="13">
         <f>IF($H$38="","",IF($H$38&lt;0,-$H$38/(-$H$38+100),100/($H$38+100)))</f>
@@ -11718,7 +11652,7 @@
         <v>179</v>
       </c>
       <c r="H39" s="15" t="n">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="I39" s="13">
         <f>IF($H$39="","",IF($H$39&lt;0,-$H$39/(-$H$39+100),100/($H$39+100)))</f>
@@ -11844,10 +11778,10 @@
         </is>
       </c>
       <c r="F41" s="13" t="n">
-        <v>0.3556302521008404</v>
+        <v>0.3566806722689076</v>
       </c>
       <c r="G41" s="14" t="n">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="H41" s="15" t="n">
         <v>138</v>
@@ -11874,7 +11808,7 @@
       </c>
       <c r="N41" s="19" t="inlineStr">
         <is>
-          <t>Model 35.6% (fair +181). Your call.</t>
+          <t>Model 35.7% (fair +180). Your call.</t>
         </is>
       </c>
       <c r="O41" s="15" t="n"/>
@@ -11910,13 +11844,13 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.6443409836065574</v>
+        <v>0.6433344398340248</v>
       </c>
       <c r="G42" s="14" t="n">
-        <v>-181</v>
+        <v>-180</v>
       </c>
       <c r="H42" s="15" t="n">
-        <v>-144</v>
+        <v>-141</v>
       </c>
       <c r="I42" s="13">
         <f>IF($H$42="","",IF($H$42&lt;0,-$H$42/(-$H$42+100),100/($H$42+100)))</f>
@@ -11940,7 +11874,7 @@
       </c>
       <c r="N42" s="19" t="inlineStr">
         <is>
-          <t>Model 64.4% (fair -181). Your call.</t>
+          <t>Model 64.3% (fair -180). Your call.</t>
         </is>
       </c>
       <c r="O42" s="15" t="n"/>
@@ -11972,7 +11906,7 @@
       </c>
       <c r="E43" s="12" t="inlineStr">
         <is>
-          <t>Over 9</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="F43" s="13" t="n">
@@ -11982,7 +11916,7 @@
         <v>111</v>
       </c>
       <c r="H43" s="15" t="n">
-        <v>106</v>
+        <v>130</v>
       </c>
       <c r="I43" s="13">
         <f>IF($H$43="","",IF($H$43&lt;0,-$H$43/(-$H$43+100),100/($H$43+100)))</f>
@@ -12038,7 +11972,7 @@
       </c>
       <c r="E44" s="20" t="inlineStr">
         <is>
-          <t>Under 9</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F44" s="13" t="n">
@@ -12048,7 +11982,7 @@
         <v>-111</v>
       </c>
       <c r="H44" s="15" t="n">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="I44" s="13">
         <f>IF($H$44="","",IF($H$44&lt;0,-$H$44/(-$H$44+100),100/($H$44+100)))</f>
@@ -12114,7 +12048,7 @@
         <v>-133</v>
       </c>
       <c r="H45" s="15" t="n">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="I45" s="13">
         <f>IF($H$45="","",IF($H$45&lt;0,-$H$45/(-$H$45+100),100/($H$45+100)))</f>
@@ -12180,7 +12114,7 @@
         <v>133</v>
       </c>
       <c r="H46" s="15" t="n">
-        <v>-104</v>
+        <v>-105</v>
       </c>
       <c r="I46" s="13">
         <f>IF($H$46="","",IF($H$46&lt;0,-$H$46/(-$H$46+100),100/($H$46+100)))</f>
@@ -12240,13 +12174,13 @@
         </is>
       </c>
       <c r="F47" s="13" t="n">
-        <v>0.4308298755186722</v>
+        <v>0.4344957983193278</v>
       </c>
       <c r="G47" s="14" t="n">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="H47" s="15" t="n">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="I47" s="13">
         <f>IF($H$47="","",IF($H$47&lt;0,-$H$47/(-$H$47+100),100/($H$47+100)))</f>
@@ -12270,7 +12204,7 @@
       </c>
       <c r="N47" s="19" t="inlineStr">
         <is>
-          <t>Model 43.1% (fair +132). Your call.</t>
+          <t>Model 43.4% (fair +130). Your call.</t>
         </is>
       </c>
       <c r="O47" s="15" t="n"/>
@@ -12306,13 +12240,13 @@
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.5692131147540984</v>
+        <v>0.5655100840336135</v>
       </c>
       <c r="G48" s="14" t="n">
-        <v>-132</v>
+        <v>-130</v>
       </c>
       <c r="H48" s="15" t="n">
-        <v>-144</v>
+        <v>-138</v>
       </c>
       <c r="I48" s="13">
         <f>IF($H$48="","",IF($H$48&lt;0,-$H$48/(-$H$48+100),100/($H$48+100)))</f>
@@ -12336,7 +12270,7 @@
       </c>
       <c r="N48" s="19" t="inlineStr">
         <is>
-          <t>Model 56.9% (fair -132). Your call.</t>
+          <t>Model 56.6% (fair -130). Your call.</t>
         </is>
       </c>
       <c r="O48" s="15" t="n"/>
@@ -12368,7 +12302,7 @@
       </c>
       <c r="E49" s="12" t="inlineStr">
         <is>
-          <t>Over 12.5</t>
+          <t>Over 12</t>
         </is>
       </c>
       <c r="F49" s="13" t="n">
@@ -12378,7 +12312,7 @@
         <v>767</v>
       </c>
       <c r="H49" s="15" t="n">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="I49" s="13">
         <f>IF($H$49="","",IF($H$49&lt;0,-$H$49/(-$H$49+100),100/($H$49+100)))</f>
@@ -12434,7 +12368,7 @@
       </c>
       <c r="E50" s="20" t="inlineStr">
         <is>
-          <t>Under 12.5</t>
+          <t>Under 12</t>
         </is>
       </c>
       <c r="F50" s="13" t="n">
@@ -12504,13 +12438,13 @@
         </is>
       </c>
       <c r="F51" s="13" t="n">
-        <v>0.4203862660944206</v>
+        <v>0.4092</v>
       </c>
       <c r="G51" s="14" t="n">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="H51" s="15" t="n">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="I51" s="13">
         <f>IF($H$51="","",IF($H$51&lt;0,-$H$51/(-$H$51+100),100/($H$51+100)))</f>
@@ -12534,7 +12468,7 @@
       </c>
       <c r="N51" s="19" t="inlineStr">
         <is>
-          <t>Model 42.0% (fair +138). Your call.</t>
+          <t>Model 40.9% (fair +144). Your call.</t>
         </is>
       </c>
       <c r="O51" s="15" t="n"/>
@@ -12570,13 +12504,13 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.5796304347826088</v>
+        <v>0.5908</v>
       </c>
       <c r="G52" s="14" t="n">
-        <v>-138</v>
+        <v>-144</v>
       </c>
       <c r="H52" s="15" t="n">
-        <v>-130</v>
+        <v>101</v>
       </c>
       <c r="I52" s="13">
         <f>IF($H$52="","",IF($H$52&lt;0,-$H$52/(-$H$52+100),100/($H$52+100)))</f>
@@ -12600,7 +12534,7 @@
       </c>
       <c r="N52" s="19" t="inlineStr">
         <is>
-          <t>Model 58.0% (fair -138). Your call.</t>
+          <t>Model 59.1% (fair -144). Your call.</t>
         </is>
       </c>
       <c r="O52" s="15" t="n"/>
@@ -12774,7 +12708,7 @@
         <v>107</v>
       </c>
       <c r="H55" s="15" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="I55" s="13">
         <f>IF($H$55="","",IF($H$55&lt;0,-$H$55/(-$H$55+100),100/($H$55+100)))</f>
@@ -12906,7 +12840,7 @@
         <v>183</v>
       </c>
       <c r="H57" s="15" t="n">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="I57" s="13">
         <f>IF($H$57="","",IF($H$57&lt;0,-$H$57/(-$H$57+100),100/($H$57+100)))</f>
@@ -12972,7 +12906,7 @@
         <v>-183</v>
       </c>
       <c r="H58" s="15" t="n">
-        <v>-118</v>
+        <v>-121</v>
       </c>
       <c r="I58" s="13">
         <f>IF($H$58="","",IF($H$58&lt;0,-$H$58/(-$H$58+100),100/($H$58+100)))</f>
@@ -13032,13 +12966,13 @@
         </is>
       </c>
       <c r="F59" s="13" t="n">
-        <v>0.5120283185840708</v>
+        <v>0.5124757709251102</v>
       </c>
       <c r="G59" s="14" t="n">
         <v>-105</v>
       </c>
       <c r="H59" s="15" t="n">
-        <v>-126</v>
+        <v>-127</v>
       </c>
       <c r="I59" s="13">
         <f>IF($H$59="","",IF($H$59&lt;0,-$H$59/(-$H$59+100),100/($H$59+100)))</f>
@@ -13098,7 +13032,7 @@
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>0.4879295154185022</v>
+        <v>0.4875330396475771</v>
       </c>
       <c r="G60" s="14" t="n">
         <v>105</v>
@@ -13160,17 +13094,17 @@
       </c>
       <c r="E61" s="12" t="inlineStr">
         <is>
-          <t>Over 11.5</t>
+          <t>Over 12</t>
         </is>
       </c>
       <c r="F61" s="13" t="n">
-        <v>0.378</v>
+        <v>0.2727</v>
       </c>
       <c r="G61" s="14" t="n">
-        <v>165</v>
+        <v>267</v>
       </c>
       <c r="H61" s="15" t="n">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="I61" s="13">
         <f>IF($H$61="","",IF($H$61&lt;0,-$H$61/(-$H$61+100),100/($H$61+100)))</f>
@@ -13194,7 +13128,7 @@
       </c>
       <c r="N61" s="19" t="inlineStr">
         <is>
-          <t>Model 37.8% (fair +165). Your call.</t>
+          <t>Model 27.3% (fair +267). Your call.</t>
         </is>
       </c>
       <c r="O61" s="15" t="n"/>
@@ -13226,17 +13160,17 @@
       </c>
       <c r="E62" s="20" t="inlineStr">
         <is>
-          <t>Under 11.5</t>
+          <t>Under 12</t>
         </is>
       </c>
       <c r="F62" s="13" t="n">
-        <v>0.622</v>
+        <v>0.7273000000000001</v>
       </c>
       <c r="G62" s="14" t="n">
-        <v>-165</v>
+        <v>-267</v>
       </c>
       <c r="H62" s="15" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="I62" s="13">
         <f>IF($H$62="","",IF($H$62&lt;0,-$H$62/(-$H$62+100),100/($H$62+100)))</f>
@@ -13260,7 +13194,7 @@
       </c>
       <c r="N62" s="19" t="inlineStr">
         <is>
-          <t>Model 62.2% (fair -165). Your call.</t>
+          <t>Model 72.7% (fair -267). Your call.</t>
         </is>
       </c>
       <c r="O62" s="15" t="n"/>
@@ -13944,10 +13878,10 @@
         </is>
       </c>
       <c r="F73" s="13" t="n">
-        <v>0.5318627450980392</v>
+        <v>0.534264705882353</v>
       </c>
       <c r="G73" s="14" t="n">
-        <v>-114</v>
+        <v>-115</v>
       </c>
       <c r="H73" s="15" t="n">
         <v>104</v>
@@ -13974,7 +13908,7 @@
       </c>
       <c r="N73" s="19" t="inlineStr">
         <is>
-          <t>Model 53.2% (fair -114). Your call.</t>
+          <t>Model 53.4% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O73" s="15" t="n"/>
@@ -14010,13 +13944,13 @@
         </is>
       </c>
       <c r="F74" s="13" t="n">
-        <v>0.4681529411764705</v>
+        <v>0.46575</v>
       </c>
       <c r="G74" s="14" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H74" s="15" t="n">
-        <v>-104</v>
+        <v>100</v>
       </c>
       <c r="I74" s="13">
         <f>IF($H$74="","",IF($H$74&lt;0,-$H$74/(-$H$74+100),100/($H$74+100)))</f>
@@ -14040,7 +13974,7 @@
       </c>
       <c r="N74" s="19" t="inlineStr">
         <is>
-          <t>Model 46.8% (fair +114). Your call.</t>
+          <t>Model 46.6% (fair +115). Your call.</t>
         </is>
       </c>
       <c r="O74" s="15" t="n"/>
@@ -14076,10 +14010,10 @@
         </is>
       </c>
       <c r="F75" s="13" t="n">
-        <v>0.3814748201438848</v>
+        <v>0.383273381294964</v>
       </c>
       <c r="G75" s="14" t="n">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H75" s="15" t="n">
         <v>178</v>
@@ -14106,7 +14040,7 @@
       </c>
       <c r="N75" s="19" t="inlineStr">
         <is>
-          <t>Model 38.1% (fair +162). Your call.</t>
+          <t>Model 38.3% (fair +161). Your call.</t>
         </is>
       </c>
       <c r="O75" s="15" t="n"/>
@@ -14142,13 +14076,13 @@
         </is>
       </c>
       <c r="F76" s="13" t="n">
-        <v>0.6185475524475526</v>
+        <v>0.6167251798561151</v>
       </c>
       <c r="G76" s="14" t="n">
-        <v>-162</v>
+        <v>-161</v>
       </c>
       <c r="H76" s="15" t="n">
-        <v>-186</v>
+        <v>-178</v>
       </c>
       <c r="I76" s="13">
         <f>IF($H$76="","",IF($H$76&lt;0,-$H$76/(-$H$76+100),100/($H$76+100)))</f>
@@ -14172,7 +14106,7 @@
       </c>
       <c r="N76" s="19" t="inlineStr">
         <is>
-          <t>Model 61.9% (fair -162). Your call.</t>
+          <t>Model 61.7% (fair -161). Your call.</t>
         </is>
       </c>
       <c r="O76" s="15" t="n"/>
@@ -14208,13 +14142,13 @@
         </is>
       </c>
       <c r="F77" s="13" t="n">
-        <v>0.4111453744493392</v>
+        <v>0.4100873362445415</v>
       </c>
       <c r="G77" s="14" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H77" s="15" t="n">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="I77" s="13">
         <f>IF($H$77="","",IF($H$77&lt;0,-$H$77/(-$H$77+100),100/($H$77+100)))</f>
@@ -14238,7 +14172,7 @@
       </c>
       <c r="N77" s="19" t="inlineStr">
         <is>
-          <t>Model 41.1% (fair +143). Your call.</t>
+          <t>Model 41.0% (fair +144). Your call.</t>
         </is>
       </c>
       <c r="O77" s="15" t="n"/>
@@ -14274,10 +14208,10 @@
         </is>
       </c>
       <c r="F78" s="13" t="n">
-        <v>0.5888532188841202</v>
+        <v>0.5899377682403434</v>
       </c>
       <c r="G78" s="14" t="n">
-        <v>-143</v>
+        <v>-144</v>
       </c>
       <c r="H78" s="15" t="n">
         <v>-133</v>
@@ -14304,7 +14238,7 @@
       </c>
       <c r="N78" s="19" t="inlineStr">
         <is>
-          <t>Model 58.9% (fair -143). Your call.</t>
+          <t>Model 59.0% (fair -144). Your call.</t>
         </is>
       </c>
       <c r="O78" s="15" t="n"/>
@@ -14340,10 +14274,10 @@
         </is>
       </c>
       <c r="F79" s="13" t="n">
-        <v>0.4800900900900902</v>
+        <v>0.505</v>
       </c>
       <c r="G79" s="14" t="n">
-        <v>108</v>
+        <v>-102</v>
       </c>
       <c r="H79" s="15" t="n">
         <v>122</v>
@@ -14370,7 +14304,7 @@
       </c>
       <c r="N79" s="19" t="inlineStr">
         <is>
-          <t>Model 48.0% (fair +108). Your call.</t>
+          <t>Model 50.5% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O79" s="15" t="n"/>
@@ -14406,13 +14340,13 @@
         </is>
       </c>
       <c r="F80" s="13" t="n">
-        <v>0.5199221198156682</v>
+        <v>0.495</v>
       </c>
       <c r="G80" s="14" t="n">
-        <v>-108</v>
+        <v>102</v>
       </c>
       <c r="H80" s="15" t="n">
-        <v>-117</v>
+        <v>-111</v>
       </c>
       <c r="I80" s="13">
         <f>IF($H$80="","",IF($H$80&lt;0,-$H$80/(-$H$80+100),100/($H$80+100)))</f>
@@ -14436,7 +14370,7 @@
       </c>
       <c r="N80" s="19" t="inlineStr">
         <is>
-          <t>Model 52.0% (fair -108). Your call.</t>
+          <t>Model 49.5% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O80" s="15" t="n"/>
@@ -14478,7 +14412,7 @@
         <v>-121</v>
       </c>
       <c r="H81" s="15" t="n">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="I81" s="13">
         <f>IF($H$81="","",IF($H$81&lt;0,-$H$81/(-$H$81+100),100/($H$81+100)))</f>
@@ -14604,13 +14538,13 @@
         </is>
       </c>
       <c r="F83" s="13" t="n">
-        <v>0.4510810810810811</v>
+        <v>0.4469957081545065</v>
       </c>
       <c r="G83" s="14" t="n">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H83" s="15" t="n">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="I83" s="13">
         <f>IF($H$83="","",IF($H$83&lt;0,-$H$83/(-$H$83+100),100/($H$83+100)))</f>
@@ -14634,7 +14568,7 @@
       </c>
       <c r="N83" s="19" t="inlineStr">
         <is>
-          <t>Model 45.1% (fair +122). Your call.</t>
+          <t>Model 44.7% (fair +124). Your call.</t>
         </is>
       </c>
       <c r="O83" s="15" t="n"/>
@@ -14670,13 +14604,13 @@
         </is>
       </c>
       <c r="F84" s="13" t="n">
-        <v>0.5489316872427984</v>
+        <v>0.5530436974789915</v>
       </c>
       <c r="G84" s="14" t="n">
-        <v>-122</v>
+        <v>-124</v>
       </c>
       <c r="H84" s="15" t="n">
-        <v>-143</v>
+        <v>-138</v>
       </c>
       <c r="I84" s="13">
         <f>IF($H$84="","",IF($H$84&lt;0,-$H$84/(-$H$84+100),100/($H$84+100)))</f>
@@ -14700,7 +14634,7 @@
       </c>
       <c r="N84" s="19" t="inlineStr">
         <is>
-          <t>Model 54.9% (fair -122). Your call.</t>
+          <t>Model 55.3% (fair -124). Your call.</t>
         </is>
       </c>
       <c r="O84" s="15" t="n"/>
@@ -14736,13 +14670,13 @@
         </is>
       </c>
       <c r="F85" s="13" t="n">
-        <v>0.4988246696035242</v>
+        <v>0.4947967741935483</v>
       </c>
       <c r="G85" s="14" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H85" s="15" t="n">
-        <v>-127</v>
+        <v>-117</v>
       </c>
       <c r="I85" s="13">
         <f>IF($H$85="","",IF($H$85&lt;0,-$H$85/(-$H$85+100),100/($H$85+100)))</f>
@@ -14766,7 +14700,7 @@
       </c>
       <c r="N85" s="19" t="inlineStr">
         <is>
-          <t>Model 49.9% (fair +100). Your call.</t>
+          <t>Model 49.5% (fair +102). Your call.</t>
         </is>
       </c>
       <c r="O85" s="15" t="n"/>
@@ -14802,13 +14736,13 @@
         </is>
       </c>
       <c r="F86" s="13" t="n">
-        <v>0.5011627906976744</v>
+        <v>0.5051851851851852</v>
       </c>
       <c r="G86" s="14" t="n">
-        <v>-100</v>
+        <v>-102</v>
       </c>
       <c r="H86" s="15" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I86" s="13">
         <f>IF($H$86="","",IF($H$86&lt;0,-$H$86/(-$H$86+100),100/($H$86+100)))</f>
@@ -14832,7 +14766,7 @@
       </c>
       <c r="N86" s="19" t="inlineStr">
         <is>
-          <t>Model 50.1% (fair -100). Your call.</t>
+          <t>Model 50.5% (fair -102). Your call.</t>
         </is>
       </c>
       <c r="O86" s="15" t="n"/>
@@ -14868,13 +14802,13 @@
         </is>
       </c>
       <c r="F87" s="13" t="n">
-        <v>0.3613688212927757</v>
+        <v>0.3564444444444445</v>
       </c>
       <c r="G87" s="14" t="n">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="H87" s="15" t="n">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="I87" s="13">
         <f>IF($H$87="","",IF($H$87&lt;0,-$H$87/(-$H$87+100),100/($H$87+100)))</f>
@@ -14898,7 +14832,7 @@
       </c>
       <c r="N87" s="19" t="inlineStr">
         <is>
-          <t>Model 36.1% (fair +177). Your call.</t>
+          <t>Model 35.6% (fair +181). Your call.</t>
         </is>
       </c>
       <c r="O87" s="15" t="n"/>
@@ -14934,13 +14868,13 @@
         </is>
       </c>
       <c r="F88" s="13" t="n">
-        <v>0.638612927756654</v>
+        <v>0.6435444444444444</v>
       </c>
       <c r="G88" s="14" t="n">
-        <v>-177</v>
+        <v>-181</v>
       </c>
       <c r="H88" s="15" t="n">
-        <v>-163</v>
+        <v>-170</v>
       </c>
       <c r="I88" s="13">
         <f>IF($H$88="","",IF($H$88&lt;0,-$H$88/(-$H$88+100),100/($H$88+100)))</f>
@@ -14964,7 +14898,7 @@
       </c>
       <c r="N88" s="19" t="inlineStr">
         <is>
-          <t>Model 63.9% (fair -177). Your call.</t>
+          <t>Model 64.4% (fair -181). Your call.</t>
         </is>
       </c>
       <c r="O88" s="15" t="n"/>
@@ -15000,13 +14934,13 @@
         </is>
       </c>
       <c r="F89" s="13" t="n">
-        <v>0.4163876651982379</v>
+        <v>0.413175965665236</v>
       </c>
       <c r="G89" s="14" t="n">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="H89" s="15" t="n">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="I89" s="13">
         <f>IF($H$89="","",IF($H$89&lt;0,-$H$89/(-$H$89+100),100/($H$89+100)))</f>
@@ -15030,7 +14964,7 @@
       </c>
       <c r="N89" s="19" t="inlineStr">
         <is>
-          <t>Model 41.6% (fair +140). Your call.</t>
+          <t>Model 41.3% (fair +142). Your call.</t>
         </is>
       </c>
       <c r="O89" s="15" t="n"/>
@@ -15066,10 +15000,10 @@
         </is>
       </c>
       <c r="F90" s="13" t="n">
-        <v>0.5836017167381974</v>
+        <v>0.5867982832618026</v>
       </c>
       <c r="G90" s="14" t="n">
-        <v>-140</v>
+        <v>-142</v>
       </c>
       <c r="H90" s="15" t="n">
         <v>-133</v>
@@ -15096,7 +15030,7 @@
       </c>
       <c r="N90" s="19" t="inlineStr">
         <is>
-          <t>Model 58.4% (fair -140). Your call.</t>
+          <t>Model 58.7% (fair -142). Your call.</t>
         </is>
       </c>
       <c r="O90" s="15" t="n"/>

</xml_diff>

<commit_message>
data: hourly update 2026-06-29 16:58Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-06-29.xlsx
+++ b/data/output/workbook/2026-06-29.xlsx
@@ -580,7 +580,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10125075" cy="9401175"/>
+    <ext cx="10125075" cy="9810750"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -953,7 +953,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 09:09</t>
+          <t>2026-06-29 12:57</t>
         </is>
       </c>
     </row>
@@ -5381,7 +5381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q74"/>
+  <dimension ref="A1:Q77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5398,815 +5398,815 @@
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="28" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="28" t="inlineStr">
         <is>
           <t>San Diego Padres offense vs Chicago Cubs defense</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="29" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="29" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B61" s="29" t="inlineStr">
+      <c r="B64" s="29" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C61" s="29" t="inlineStr">
+      <c r="C64" s="29" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D61" s="29" t="inlineStr">
+      <c r="D64" s="29" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E61" s="29" t="inlineStr">
+      <c r="E64" s="29" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F61" s="29" t="inlineStr">
+      <c r="F64" s="29" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G61" s="29" t="inlineStr">
+      <c r="G64" s="29" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H61" s="29" t="inlineStr">
+      <c r="H64" s="29" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I61" s="29" t="inlineStr">
+      <c r="I64" s="29" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J61" s="29" t="inlineStr">
+      <c r="J64" s="29" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K61" s="29" t="inlineStr">
+      <c r="K64" s="29" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L61" s="29" t="inlineStr">
+      <c r="L64" s="29" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M61" s="29" t="inlineStr">
+      <c r="M64" s="29" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N61" s="29" t="inlineStr">
+      <c r="N64" s="29" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O61" s="29" t="inlineStr">
+      <c r="O64" s="29" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P61" s="29" t="inlineStr">
+      <c r="P64" s="29" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q61" s="29" t="inlineStr">
+      <c r="Q64" s="29" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="30" t="inlineStr">
-        <is>
-          <t>Runs/G</t>
-        </is>
-      </c>
-      <c r="B62" s="31" t="n">
-        <v>4.279</v>
-      </c>
-      <c r="C62" s="31" t="n">
-        <v>4.433</v>
-      </c>
-      <c r="D62" s="31" t="n">
-        <v>3.55</v>
-      </c>
-      <c r="E62" s="31" t="n">
-        <v>3.733</v>
-      </c>
-      <c r="F62" s="31" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="G62" s="31" t="n">
-        <v>3</v>
-      </c>
-      <c r="H62" s="35" t="inlineStr">
-        <is>
-          <t>19th</t>
-        </is>
-      </c>
-      <c r="I62" s="31" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="J62" s="33" t="inlineStr">
-        <is>
-          <t>24th</t>
-        </is>
-      </c>
-      <c r="K62" s="31" t="n">
-        <v>5</v>
-      </c>
-      <c r="L62" s="31" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="M62" s="31" t="n">
-        <v>5</v>
-      </c>
-      <c r="N62" s="31" t="n">
-        <v>4.25</v>
-      </c>
-      <c r="O62" s="31" t="n">
-        <v>4.767</v>
-      </c>
-      <c r="P62" s="31" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="Q62" s="34" t="inlineStr">
-        <is>
-          <t>Opp Runs/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="30" t="inlineStr">
-        <is>
-          <t>Hits/G</t>
-        </is>
-      </c>
-      <c r="B63" s="31" t="n">
-        <v>7.139</v>
-      </c>
-      <c r="C63" s="31" t="n">
-        <v>7.167</v>
-      </c>
-      <c r="D63" s="31" t="n">
-        <v>6.444</v>
-      </c>
-      <c r="E63" s="31" t="n">
-        <v>6.357</v>
-      </c>
-      <c r="F63" s="31" t="n">
-        <v>5.111</v>
-      </c>
-      <c r="G63" s="31" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="H63" s="33" t="inlineStr">
-        <is>
-          <t>27th</t>
-        </is>
-      </c>
-      <c r="I63" s="31" t="inlineStr"/>
-      <c r="J63" s="33" t="inlineStr">
-        <is>
-          <t>25th</t>
-        </is>
-      </c>
-      <c r="K63" s="31" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="L63" s="31" t="n">
-        <v>7.7</v>
-      </c>
-      <c r="M63" s="31" t="n">
-        <v>8</v>
-      </c>
-      <c r="N63" s="31" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="O63" s="31" t="n">
-        <v>7.966</v>
-      </c>
-      <c r="P63" s="31" t="n">
-        <v>7.595</v>
-      </c>
-      <c r="Q63" s="34" t="inlineStr">
-        <is>
-          <t>Opp Hits/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="30" t="inlineStr">
-        <is>
-          <t>HR/G</t>
-        </is>
-      </c>
-      <c r="B64" s="31" t="n">
-        <v>0.972</v>
-      </c>
-      <c r="C64" s="31" t="n">
-        <v>1.167</v>
-      </c>
-      <c r="D64" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="E64" s="31" t="n">
-        <v>1.286</v>
-      </c>
-      <c r="F64" s="31" t="n">
-        <v>1.111</v>
-      </c>
-      <c r="G64" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="H64" s="35" t="inlineStr">
-        <is>
-          <t>15th</t>
-        </is>
-      </c>
-      <c r="I64" s="31" t="inlineStr"/>
-      <c r="J64" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K64" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L64" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M64" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N64" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O64" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P64" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q64" s="34" t="inlineStr">
-        <is>
-          <t>Opp HR/G</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="30" t="inlineStr">
         <is>
-          <t>Batter K/G</t>
+          <t>Runs/G</t>
         </is>
       </c>
       <c r="B65" s="31" t="n">
-        <v>8.138999999999999</v>
+        <v>4.279</v>
       </c>
       <c r="C65" s="31" t="n">
-        <v>8.042</v>
+        <v>4.433</v>
       </c>
       <c r="D65" s="31" t="n">
-        <v>9</v>
+        <v>3.55</v>
       </c>
       <c r="E65" s="31" t="n">
-        <v>8.714</v>
+        <v>3.733</v>
       </c>
       <c r="F65" s="31" t="n">
-        <v>7.889</v>
+        <v>2.9</v>
       </c>
       <c r="G65" s="31" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="H65" s="32" t="inlineStr">
-        <is>
-          <t>5th</t>
+        <v>3</v>
+      </c>
+      <c r="H65" s="35" t="inlineStr">
+        <is>
+          <t>19th</t>
         </is>
       </c>
       <c r="I65" s="31" t="inlineStr">
         <is>
-          <t>★★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="J65" s="33" t="inlineStr">
         <is>
-          <t>25th</t>
+          <t>24th</t>
         </is>
       </c>
       <c r="K65" s="31" t="n">
-        <v>7.4</v>
+        <v>5</v>
       </c>
       <c r="L65" s="31" t="n">
-        <v>7.3</v>
+        <v>4.6</v>
       </c>
       <c r="M65" s="31" t="n">
-        <v>7.2</v>
+        <v>5</v>
       </c>
       <c r="N65" s="31" t="n">
-        <v>7.35</v>
+        <v>4.25</v>
       </c>
       <c r="O65" s="31" t="n">
-        <v>7.552</v>
+        <v>4.767</v>
       </c>
       <c r="P65" s="31" t="n">
-        <v>7.838</v>
+        <v>4.5</v>
       </c>
       <c r="Q65" s="34" t="inlineStr">
         <is>
-          <t>Opp Batter K/G</t>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="30" t="inlineStr">
         <is>
+          <t>Hits/G</t>
+        </is>
+      </c>
+      <c r="B66" s="31" t="n">
+        <v>7.139</v>
+      </c>
+      <c r="C66" s="31" t="n">
+        <v>7.167</v>
+      </c>
+      <c r="D66" s="31" t="n">
+        <v>6.444</v>
+      </c>
+      <c r="E66" s="31" t="n">
+        <v>6.357</v>
+      </c>
+      <c r="F66" s="31" t="n">
+        <v>5.111</v>
+      </c>
+      <c r="G66" s="31" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="H66" s="33" t="inlineStr">
+        <is>
+          <t>27th</t>
+        </is>
+      </c>
+      <c r="I66" s="31" t="inlineStr"/>
+      <c r="J66" s="33" t="inlineStr">
+        <is>
+          <t>25th</t>
+        </is>
+      </c>
+      <c r="K66" s="31" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="L66" s="31" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="M66" s="31" t="n">
+        <v>8</v>
+      </c>
+      <c r="N66" s="31" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="O66" s="31" t="n">
+        <v>7.966</v>
+      </c>
+      <c r="P66" s="31" t="n">
+        <v>7.595</v>
+      </c>
+      <c r="Q66" s="34" t="inlineStr">
+        <is>
+          <t>Opp Hits/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="30" t="inlineStr">
+        <is>
+          <t>HR/G</t>
+        </is>
+      </c>
+      <c r="B67" s="31" t="n">
+        <v>0.972</v>
+      </c>
+      <c r="C67" s="31" t="n">
+        <v>1.167</v>
+      </c>
+      <c r="D67" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" s="31" t="n">
+        <v>1.286</v>
+      </c>
+      <c r="F67" s="31" t="n">
+        <v>1.111</v>
+      </c>
+      <c r="G67" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H67" s="35" t="inlineStr">
+        <is>
+          <t>15th</t>
+        </is>
+      </c>
+      <c r="I67" s="31" t="inlineStr"/>
+      <c r="J67" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K67" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L67" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M67" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N67" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O67" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P67" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q67" s="34" t="inlineStr">
+        <is>
+          <t>Opp HR/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="30" t="inlineStr">
+        <is>
+          <t>Batter K/G</t>
+        </is>
+      </c>
+      <c r="B68" s="31" t="n">
+        <v>8.138999999999999</v>
+      </c>
+      <c r="C68" s="31" t="n">
+        <v>8.042</v>
+      </c>
+      <c r="D68" s="31" t="n">
+        <v>9</v>
+      </c>
+      <c r="E68" s="31" t="n">
+        <v>8.714</v>
+      </c>
+      <c r="F68" s="31" t="n">
+        <v>7.889</v>
+      </c>
+      <c r="G68" s="31" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="H68" s="32" t="inlineStr">
+        <is>
+          <t>5th</t>
+        </is>
+      </c>
+      <c r="I68" s="31" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="J68" s="33" t="inlineStr">
+        <is>
+          <t>25th</t>
+        </is>
+      </c>
+      <c r="K68" s="31" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="L68" s="31" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="M68" s="31" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="N68" s="31" t="n">
+        <v>7.35</v>
+      </c>
+      <c r="O68" s="31" t="n">
+        <v>7.552</v>
+      </c>
+      <c r="P68" s="31" t="n">
+        <v>7.838</v>
+      </c>
+      <c r="Q68" s="34" t="inlineStr">
+        <is>
+          <t>Opp Batter K/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="30" t="inlineStr">
+        <is>
           <t>1st Inn R/G</t>
         </is>
       </c>
-      <c r="B66" s="31" t="n">
+      <c r="B69" s="31" t="n">
         <v>0.222</v>
       </c>
-      <c r="C66" s="31" t="n">
+      <c r="C69" s="31" t="n">
         <v>0.292</v>
       </c>
-      <c r="D66" s="31" t="n">
+      <c r="D69" s="31" t="n">
         <v>0.333</v>
       </c>
-      <c r="E66" s="31" t="n">
+      <c r="E69" s="31" t="n">
         <v>0.429</v>
       </c>
-      <c r="F66" s="31" t="n">
+      <c r="F69" s="31" t="n">
         <v>0.556</v>
       </c>
-      <c r="G66" s="31" t="n">
+      <c r="G69" s="31" t="n">
         <v>0.8</v>
       </c>
-      <c r="H66" s="35" t="inlineStr">
+      <c r="H69" s="35" t="inlineStr">
         <is>
           <t>11th</t>
         </is>
       </c>
-      <c r="I66" s="31" t="inlineStr">
+      <c r="I69" s="31" t="inlineStr">
         <is>
           <t>★★★</t>
         </is>
       </c>
-      <c r="J66" s="33" t="inlineStr">
+      <c r="J69" s="33" t="inlineStr">
         <is>
           <t>28th</t>
         </is>
       </c>
-      <c r="K66" s="31" t="n">
+      <c r="K69" s="31" t="n">
         <v>1.2</v>
       </c>
-      <c r="L66" s="31" t="n">
+      <c r="L69" s="31" t="n">
         <v>0.9</v>
       </c>
-      <c r="M66" s="31" t="n">
+      <c r="M69" s="31" t="n">
         <v>0.6</v>
       </c>
-      <c r="N66" s="31" t="n">
+      <c r="N69" s="31" t="n">
         <v>0.5</v>
       </c>
-      <c r="O66" s="31" t="n">
+      <c r="O69" s="31" t="n">
         <v>0.414</v>
       </c>
-      <c r="P66" s="31" t="n">
+      <c r="P69" s="31" t="n">
         <v>0.405</v>
       </c>
-      <c r="Q66" s="34" t="inlineStr">
+      <c r="Q69" s="34" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="28" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="28" t="inlineStr">
         <is>
           <t>Chicago Cubs offense vs San Diego Padres defense</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="29" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="29" t="inlineStr">
         <is>
           <t>Stat</t>
         </is>
       </c>
-      <c r="B69" s="29" t="inlineStr">
+      <c r="B72" s="29" t="inlineStr">
         <is>
           <t>A Season</t>
         </is>
       </c>
-      <c r="C69" s="29" t="inlineStr">
+      <c r="C72" s="29" t="inlineStr">
         <is>
           <t>A L30</t>
         </is>
       </c>
-      <c r="D69" s="29" t="inlineStr">
+      <c r="D72" s="29" t="inlineStr">
         <is>
           <t>A L20</t>
         </is>
       </c>
-      <c r="E69" s="29" t="inlineStr">
+      <c r="E72" s="29" t="inlineStr">
         <is>
           <t>A L15</t>
         </is>
       </c>
-      <c r="F69" s="29" t="inlineStr">
+      <c r="F72" s="29" t="inlineStr">
         <is>
           <t>A L10</t>
         </is>
       </c>
-      <c r="G69" s="29" t="inlineStr">
+      <c r="G72" s="29" t="inlineStr">
         <is>
           <t>A L5</t>
         </is>
       </c>
-      <c r="H69" s="29" t="inlineStr">
+      <c r="H72" s="29" t="inlineStr">
         <is>
           <t>A Rk</t>
         </is>
       </c>
-      <c r="I69" s="29" t="inlineStr">
+      <c r="I72" s="29" t="inlineStr">
         <is>
           <t>Adv</t>
         </is>
       </c>
-      <c r="J69" s="29" t="inlineStr">
+      <c r="J72" s="29" t="inlineStr">
         <is>
           <t>H Rk</t>
         </is>
       </c>
-      <c r="K69" s="29" t="inlineStr">
+      <c r="K72" s="29" t="inlineStr">
         <is>
           <t>H L5</t>
         </is>
       </c>
-      <c r="L69" s="29" t="inlineStr">
+      <c r="L72" s="29" t="inlineStr">
         <is>
           <t>H L10</t>
         </is>
       </c>
-      <c r="M69" s="29" t="inlineStr">
+      <c r="M72" s="29" t="inlineStr">
         <is>
           <t>H L15</t>
         </is>
       </c>
-      <c r="N69" s="29" t="inlineStr">
+      <c r="N72" s="29" t="inlineStr">
         <is>
           <t>H L20</t>
         </is>
       </c>
-      <c r="O69" s="29" t="inlineStr">
+      <c r="O72" s="29" t="inlineStr">
         <is>
           <t>H L30</t>
         </is>
       </c>
-      <c r="P69" s="29" t="inlineStr">
+      <c r="P72" s="29" t="inlineStr">
         <is>
           <t>H Season</t>
         </is>
       </c>
-      <c r="Q69" s="29" t="inlineStr">
+      <c r="Q72" s="29" t="inlineStr">
         <is>
           <t>Opp stat</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="30" t="inlineStr">
-        <is>
-          <t>Runs/G</t>
-        </is>
-      </c>
-      <c r="B70" s="31" t="n">
-        <v>4.947</v>
-      </c>
-      <c r="C70" s="31" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="D70" s="31" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="E70" s="31" t="n">
-        <v>4.267</v>
-      </c>
-      <c r="F70" s="31" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="G70" s="31" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="H70" s="33" t="inlineStr">
-        <is>
-          <t>30th</t>
-        </is>
-      </c>
-      <c r="I70" s="31" t="inlineStr"/>
-      <c r="J70" s="32" t="inlineStr">
-        <is>
-          <t>4th</t>
-        </is>
-      </c>
-      <c r="K70" s="31" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="L70" s="31" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="M70" s="31" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="N70" s="31" t="n">
-        <v>3.95</v>
-      </c>
-      <c r="O70" s="31" t="n">
-        <v>3.667</v>
-      </c>
-      <c r="P70" s="31" t="n">
-        <v>3.674</v>
-      </c>
-      <c r="Q70" s="34" t="inlineStr">
-        <is>
-          <t>Opp Runs/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="30" t="inlineStr">
-        <is>
-          <t>Hits/G</t>
-        </is>
-      </c>
-      <c r="B71" s="31" t="n">
-        <v>8.432</v>
-      </c>
-      <c r="C71" s="31" t="n">
-        <v>8.965999999999999</v>
-      </c>
-      <c r="D71" s="31" t="n">
-        <v>8.699999999999999</v>
-      </c>
-      <c r="E71" s="31" t="n">
-        <v>8.333</v>
-      </c>
-      <c r="F71" s="31" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="G71" s="31" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="H71" s="33" t="inlineStr">
-        <is>
-          <t>30th</t>
-        </is>
-      </c>
-      <c r="I71" s="31" t="inlineStr"/>
-      <c r="J71" s="35" t="inlineStr">
-        <is>
-          <t>19th</t>
-        </is>
-      </c>
-      <c r="K71" s="31" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="L71" s="31" t="n">
-        <v>7.778</v>
-      </c>
-      <c r="M71" s="31" t="n">
-        <v>8.856999999999999</v>
-      </c>
-      <c r="N71" s="31" t="n">
-        <v>8.444000000000001</v>
-      </c>
-      <c r="O71" s="31" t="n">
-        <v>8.125</v>
-      </c>
-      <c r="P71" s="31" t="n">
-        <v>8.111000000000001</v>
-      </c>
-      <c r="Q71" s="34" t="inlineStr">
-        <is>
-          <t>Opp Hits/G</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="30" t="inlineStr">
-        <is>
-          <t>HR/G</t>
-        </is>
-      </c>
-      <c r="B72" s="31" t="n">
-        <v>1.135</v>
-      </c>
-      <c r="C72" s="31" t="n">
-        <v>1.241</v>
-      </c>
-      <c r="D72" s="31" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="E72" s="31" t="n">
-        <v>1.133</v>
-      </c>
-      <c r="F72" s="31" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G72" s="31" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H72" s="33" t="inlineStr">
-        <is>
-          <t>24th</t>
-        </is>
-      </c>
-      <c r="I72" s="31" t="inlineStr"/>
-      <c r="J72" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K72" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L72" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M72" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N72" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O72" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P72" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q72" s="34" t="inlineStr">
-        <is>
-          <t>Opp HR/G</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="30" t="inlineStr">
         <is>
-          <t>Batter K/G</t>
+          <t>Runs/G</t>
         </is>
       </c>
       <c r="B73" s="31" t="n">
-        <v>8.541</v>
+        <v>4.947</v>
       </c>
       <c r="C73" s="31" t="n">
-        <v>8.516999999999999</v>
+        <v>5.2</v>
       </c>
       <c r="D73" s="31" t="n">
-        <v>8.199999999999999</v>
+        <v>4.9</v>
       </c>
       <c r="E73" s="31" t="n">
-        <v>8.6</v>
+        <v>4.267</v>
       </c>
       <c r="F73" s="31" t="n">
-        <v>8.5</v>
+        <v>3.2</v>
       </c>
       <c r="G73" s="31" t="n">
-        <v>10</v>
+        <v>1.4</v>
       </c>
       <c r="H73" s="33" t="inlineStr">
         <is>
-          <t>25th</t>
+          <t>30th</t>
         </is>
       </c>
       <c r="I73" s="31" t="inlineStr"/>
-      <c r="J73" s="33" t="inlineStr">
-        <is>
-          <t>24th</t>
+      <c r="J73" s="32" t="inlineStr">
+        <is>
+          <t>4th</t>
         </is>
       </c>
       <c r="K73" s="31" t="n">
-        <v>7.4</v>
+        <v>2.4</v>
       </c>
       <c r="L73" s="31" t="n">
-        <v>8.333</v>
+        <v>3.4</v>
       </c>
       <c r="M73" s="31" t="n">
-        <v>7.5</v>
+        <v>4.4</v>
       </c>
       <c r="N73" s="31" t="n">
-        <v>8.167</v>
+        <v>3.95</v>
       </c>
       <c r="O73" s="31" t="n">
-        <v>8.708</v>
+        <v>3.667</v>
       </c>
       <c r="P73" s="31" t="n">
-        <v>8.805999999999999</v>
+        <v>3.674</v>
       </c>
       <c r="Q73" s="34" t="inlineStr">
         <is>
-          <t>Opp Batter K/G</t>
+          <t>Opp Runs/G</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="30" t="inlineStr">
         <is>
+          <t>Hits/G</t>
+        </is>
+      </c>
+      <c r="B74" s="31" t="n">
+        <v>8.432</v>
+      </c>
+      <c r="C74" s="31" t="n">
+        <v>8.965999999999999</v>
+      </c>
+      <c r="D74" s="31" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="E74" s="31" t="n">
+        <v>8.333</v>
+      </c>
+      <c r="F74" s="31" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="G74" s="31" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="H74" s="33" t="inlineStr">
+        <is>
+          <t>30th</t>
+        </is>
+      </c>
+      <c r="I74" s="31" t="inlineStr"/>
+      <c r="J74" s="35" t="inlineStr">
+        <is>
+          <t>19th</t>
+        </is>
+      </c>
+      <c r="K74" s="31" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="L74" s="31" t="n">
+        <v>7.778</v>
+      </c>
+      <c r="M74" s="31" t="n">
+        <v>8.856999999999999</v>
+      </c>
+      <c r="N74" s="31" t="n">
+        <v>8.444000000000001</v>
+      </c>
+      <c r="O74" s="31" t="n">
+        <v>8.125</v>
+      </c>
+      <c r="P74" s="31" t="n">
+        <v>8.111000000000001</v>
+      </c>
+      <c r="Q74" s="34" t="inlineStr">
+        <is>
+          <t>Opp Hits/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="30" t="inlineStr">
+        <is>
+          <t>HR/G</t>
+        </is>
+      </c>
+      <c r="B75" s="31" t="n">
+        <v>1.135</v>
+      </c>
+      <c r="C75" s="31" t="n">
+        <v>1.241</v>
+      </c>
+      <c r="D75" s="31" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="E75" s="31" t="n">
+        <v>1.133</v>
+      </c>
+      <c r="F75" s="31" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G75" s="31" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H75" s="33" t="inlineStr">
+        <is>
+          <t>24th</t>
+        </is>
+      </c>
+      <c r="I75" s="31" t="inlineStr"/>
+      <c r="J75" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K75" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L75" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M75" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N75" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O75" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P75" s="31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q75" s="34" t="inlineStr">
+        <is>
+          <t>Opp HR/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="30" t="inlineStr">
+        <is>
+          <t>Batter K/G</t>
+        </is>
+      </c>
+      <c r="B76" s="31" t="n">
+        <v>8.541</v>
+      </c>
+      <c r="C76" s="31" t="n">
+        <v>8.516999999999999</v>
+      </c>
+      <c r="D76" s="31" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="E76" s="31" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="F76" s="31" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="G76" s="31" t="n">
+        <v>10</v>
+      </c>
+      <c r="H76" s="33" t="inlineStr">
+        <is>
+          <t>25th</t>
+        </is>
+      </c>
+      <c r="I76" s="31" t="inlineStr"/>
+      <c r="J76" s="33" t="inlineStr">
+        <is>
+          <t>24th</t>
+        </is>
+      </c>
+      <c r="K76" s="31" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="L76" s="31" t="n">
+        <v>8.333</v>
+      </c>
+      <c r="M76" s="31" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="N76" s="31" t="n">
+        <v>8.167</v>
+      </c>
+      <c r="O76" s="31" t="n">
+        <v>8.708</v>
+      </c>
+      <c r="P76" s="31" t="n">
+        <v>8.805999999999999</v>
+      </c>
+      <c r="Q76" s="34" t="inlineStr">
+        <is>
+          <t>Opp Batter K/G</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="30" t="inlineStr">
+        <is>
           <t>1st Inn R/G</t>
         </is>
       </c>
-      <c r="B74" s="31" t="n">
+      <c r="B77" s="31" t="n">
         <v>0.297</v>
       </c>
-      <c r="C74" s="31" t="n">
+      <c r="C77" s="31" t="n">
         <v>0.276</v>
       </c>
-      <c r="D74" s="31" t="n">
+      <c r="D77" s="31" t="n">
         <v>0.35</v>
       </c>
-      <c r="E74" s="31" t="n">
+      <c r="E77" s="31" t="n">
         <v>0.2</v>
       </c>
-      <c r="F74" s="31" t="n">
+      <c r="F77" s="31" t="n">
         <v>0.2</v>
       </c>
-      <c r="G74" s="31" t="n">
+      <c r="G77" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="H74" s="33" t="inlineStr">
+      <c r="H77" s="33" t="inlineStr">
         <is>
           <t>29th</t>
         </is>
       </c>
-      <c r="I74" s="31" t="inlineStr"/>
-      <c r="J74" s="33" t="inlineStr">
+      <c r="I77" s="31" t="inlineStr"/>
+      <c r="J77" s="33" t="inlineStr">
         <is>
           <t>25th</t>
         </is>
       </c>
-      <c r="K74" s="31" t="n">
+      <c r="K77" s="31" t="n">
         <v>1</v>
       </c>
-      <c r="L74" s="31" t="n">
+      <c r="L77" s="31" t="n">
         <v>0.556</v>
       </c>
-      <c r="M74" s="31" t="n">
+      <c r="M77" s="31" t="n">
         <v>0.429</v>
       </c>
-      <c r="N74" s="31" t="n">
+      <c r="N77" s="31" t="n">
         <v>0.333</v>
       </c>
-      <c r="O74" s="31" t="n">
+      <c r="O77" s="31" t="n">
         <v>0.333</v>
       </c>
-      <c r="P74" s="31" t="n">
+      <c r="P77" s="31" t="n">
         <v>0.417</v>
       </c>
-      <c r="Q74" s="34" t="inlineStr">
+      <c r="Q77" s="34" t="inlineStr">
         <is>
           <t>Opp 1st Inn R/G</t>
         </is>
@@ -8120,32 +8120,32 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Philadelphia Phillies</t>
+          <t>New York Mets @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>22:40</t>
+          <t>23:07</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Under 9</t>
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.554</v>
+        <v>0.5757692307692307</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-124</v>
+        <v>-136</v>
       </c>
       <c r="H5" s="15" t="n">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="I5" s="13">
         <f>IF($H$5="","",IF($H$5&lt;0,-$H$5/(-$H$5+100),100/($H$5+100)))</f>
@@ -8169,7 +8169,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 55.4% (fair -124). Your call.</t>
+          <t>Model 57.6% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -8186,12 +8186,12 @@
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>Miami Marlins @ Colorado Rockies</t>
+          <t>Cincinnati Reds @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>00:40</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
@@ -8201,17 +8201,17 @@
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.4875330396475771</v>
+        <v>0.6390913043478261</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>105</v>
+        <v>-177</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>127</v>
+        <v>-130</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -8235,7 +8235,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 48.8% (fair +105). Your call.</t>
+          <t>Model 63.9% (fair -177). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -8252,12 +8252,12 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Milwaukee Brewers</t>
+          <t>Miami Marlins @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>23:40</t>
+          <t>00:40</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
@@ -8267,17 +8267,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.6433344398340248</v>
+        <v>0.4846521739130435</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-180</v>
+        <v>106</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>-141</v>
+        <v>130</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -8301,7 +8301,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 64.3% (fair -180). Your call.</t>
+          <t>Model 48.5% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -8313,17 +8313,17 @@
     <row r="8">
       <c r="A8" s="20" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Kansas City Royals</t>
+          <t>Pittsburgh Pirates @ Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>23:40</t>
+          <t>22:40</t>
         </is>
       </c>
       <c r="D8" s="20" t="inlineStr">
@@ -8333,17 +8333,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5051851851851852</v>
+        <v>0.5502970297029702</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-102</v>
+        <v>-122</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -8367,7 +8367,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 50.5% (fair -102). Your call.</t>
+          <t>Model 55.0% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -8379,17 +8379,17 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Minnesota Twins @ Houston Astros</t>
+          <t>Texas Rangers @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>22:40</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -8399,17 +8399,17 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.4803964757709251</v>
+        <v>0.5318269230769231</v>
       </c>
       <c r="G9" s="14" t="n">
+        <v>-114</v>
+      </c>
+      <c r="H9" s="15" t="n">
         <v>108</v>
-      </c>
-      <c r="H9" s="15" t="n">
-        <v>127</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -8433,7 +8433,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 48.0% (fair +108). Your call.</t>
+          <t>Model 53.2% (fair -114). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -8445,17 +8445,17 @@
     <row r="10">
       <c r="A10" s="20" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>Texas Rangers @ Cleveland Guardians</t>
+          <t>Minnesota Twins @ Houston Astros</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>22:40</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
@@ -8465,17 +8465,17 @@
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.534264705882353</v>
+        <v>0.4787826086956522</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-115</v>
+        <v>109</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>104</v>
+        <v>130</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -8499,7 +8499,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 53.4% (fair -115). Your call.</t>
+          <t>Model 47.9% (fair +109). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -8511,17 +8511,17 @@
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Texas Rangers @ Cleveland Guardians</t>
+          <t>Tampa Bay Rays @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -8531,17 +8531,17 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.4607659574468085</v>
+        <v>0.5077674418604651</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>117</v>
+        <v>-103</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>135</v>
+        <v>115</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -8565,7 +8565,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 46.1% (fair +117). Your call.</t>
+          <t>Model 50.8% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -8577,17 +8577,17 @@
     <row r="12">
       <c r="A12" s="20" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B12" s="20" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Philadelphia Phillies</t>
+          <t>Texas Rangers @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
         <is>
-          <t>22:40</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D12" s="20" t="inlineStr">
@@ -8597,17 +8597,17 @@
       </c>
       <c r="E12" s="20" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.383273381294964</v>
+        <v>0.4602118644067796</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>161</v>
+        <v>117</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>178</v>
+        <v>136</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -8631,7 +8631,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 38.3% (fair +161). Your call.</t>
+          <t>Model 46.0% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -8667,10 +8667,10 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.4869124423963134</v>
+        <v>0.4864055299539171</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H13" s="15" t="n">
         <v>117</v>
@@ -8697,7 +8697,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 48.7% (fair +105). Your call.</t>
+          <t>Model 48.6% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -8714,12 +8714,12 @@
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>Detroit Tigers @ New York Yankees</t>
+          <t>San Diego Padres @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>23:05</t>
+          <t>00:05</t>
         </is>
       </c>
       <c r="D14" s="20" t="inlineStr">
@@ -8729,17 +8729,17 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4528755364806866</v>
+        <v>0.4293032786885246</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -8763,7 +8763,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 45.3% (fair +121). Your call.</t>
+          <t>Model 42.9% (fair +133). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -8775,17 +8775,17 @@
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Baltimore Orioles</t>
+          <t>Detroit Tigers @ New York Yankees</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>22:35</t>
+          <t>23:05</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -8795,17 +8795,17 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.4487124463519314</v>
+        <v>0.4607929515418502</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -8829,7 +8829,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 44.9% (fair +123). Your call.</t>
+          <t>Model 46.1% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -8846,12 +8846,12 @@
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>St. Louis Cardinals @ Atlanta Braves</t>
+          <t>Chicago White Sox @ Baltimore Orioles</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>23:15</t>
+          <t>22:35</t>
         </is>
       </c>
       <c r="D16" s="20" t="inlineStr">
@@ -8861,14 +8861,14 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>St. Louis Cardinals</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.4469957081545065</v>
+        <v>0.4487124463519314</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H16" s="15" t="n">
         <v>133</v>
@@ -8895,7 +8895,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 44.7% (fair +124). Your call.</t>
+          <t>Model 44.9% (fair +123). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -8907,17 +8907,17 @@
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Baltimore Orioles</t>
+          <t>St. Louis Cardinals @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>22:35</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -8927,17 +8927,17 @@
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>St. Louis Cardinals</t>
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.4603111111111111</v>
+        <v>0.4469957081545065</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -8961,7 +8961,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 46.0% (fair +117). Your call.</t>
+          <t>Model 44.7% (fair +124). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -8978,32 +8978,32 @@
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Chicago Cubs</t>
+          <t>Washington Nationals @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
-          <t>00:05</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E18" s="20" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Boston Red Sox -1.5</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.4344957983193278</v>
+        <v>0.4526521739130435</v>
       </c>
       <c r="G18" s="14" t="n">
+        <v>121</v>
+      </c>
+      <c r="H18" s="15" t="n">
         <v>130</v>
-      </c>
-      <c r="H18" s="15" t="n">
-        <v>138</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -9027,7 +9027,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 43.4% (fair +130). Your call.</t>
+          <t>Model 45.3% (fair +121). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -9039,17 +9039,17 @@
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Detroit Tigers @ New York Yankees</t>
+          <t>Chicago White Sox @ Baltimore Orioles</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>23:05</t>
+          <t>22:35</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -9059,17 +9059,17 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.5899377682403434</v>
+        <v>0.4603111111111111</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>-144</v>
+        <v>117</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>-133</v>
+        <v>125</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -9093,7 +9093,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 59.0% (fair -144). Your call.</t>
+          <t>Model 46.0% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -9110,12 +9110,12 @@
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Chicago Cubs</t>
+          <t>Detroit Tigers @ New York Yankees</t>
         </is>
       </c>
       <c r="C20" s="20" t="inlineStr">
         <is>
-          <t>00:05</t>
+          <t>23:05</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
@@ -9125,14 +9125,14 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.5867982832618026</v>
+        <v>0.5899377682403434</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>-142</v>
+        <v>-144</v>
       </c>
       <c r="H20" s="15" t="n">
         <v>-133</v>
@@ -9159,7 +9159,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 58.7% (fair -142). Your call.</t>
+          <t>Model 59.0% (fair -144). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -9176,12 +9176,12 @@
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Milwaukee Brewers</t>
+          <t>San Diego Padres @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>23:40</t>
+          <t>00:05</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
@@ -9191,17 +9191,17 @@
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.6435444444444444</v>
+        <v>0.5867982832618026</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>-181</v>
+        <v>-142</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>-170</v>
+        <v>-133</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -9225,7 +9225,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 64.4% (fair -181). Your call.</t>
+          <t>Model 58.7% (fair -142). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -9540,7 +9540,7 @@
         <v>110</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="I7" s="13">
         <f>IF($H$7="","",IF($H$7&lt;0,-$H$7/(-$H$7+100),100/($H$7+100)))</f>
@@ -9606,7 +9606,7 @@
         <v>-110</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -9672,7 +9672,7 @@
         <v>155</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -9738,7 +9738,7 @@
         <v>-155</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -9798,13 +9798,13 @@
         </is>
       </c>
       <c r="F11" s="13" t="n">
-        <v>0.554</v>
+        <v>0.5502970297029702</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-124</v>
+        <v>-122</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="I11" s="13">
         <f>IF($H$11="","",IF($H$11&lt;0,-$H$11/(-$H$11+100),100/($H$11+100)))</f>
@@ -9828,7 +9828,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Model 55.4% (fair -124). Your call.</t>
+          <t>Model 55.0% (fair -122). Your call.</t>
         </is>
       </c>
       <c r="O11" s="15" t="n"/>
@@ -9864,13 +9864,13 @@
         </is>
       </c>
       <c r="F12" s="13" t="n">
-        <v>0.445990099009901</v>
+        <v>0.4497089108910891</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>102</v>
+        <v>-102</v>
       </c>
       <c r="I12" s="13">
         <f>IF($H$12="","",IF($H$12&lt;0,-$H$12/(-$H$12+100),100/($H$12+100)))</f>
@@ -9894,7 +9894,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Model 44.6% (fair +124). Your call.</t>
+          <t>Model 45.0% (fair +122). Your call.</t>
         </is>
       </c>
       <c r="O12" s="15" t="n"/>
@@ -9926,17 +9926,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Over 9</t>
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>0.5928</v>
+        <v>0.4931</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>-146</v>
+        <v>103</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="I13" s="13">
         <f>IF($H$13="","",IF($H$13&lt;0,-$H$13/(-$H$13+100),100/($H$13+100)))</f>
@@ -9960,7 +9960,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Model 59.3% (fair -146). Your call.</t>
+          <t>Model 49.3% (fair +103). Your call.</t>
         </is>
       </c>
       <c r="O13" s="15" t="n"/>
@@ -9992,17 +9992,17 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Under 8.5</t>
+          <t>Under 9</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.4072</v>
+        <v>0.5069</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>146</v>
+        <v>-103</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -10026,7 +10026,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 40.7% (fair +146). Your call.</t>
+          <t>Model 50.7% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -10194,13 +10194,13 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.4528755364806866</v>
+        <v>0.4607929515418502</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -10224,7 +10224,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 45.3% (fair +121). Your call.</t>
+          <t>Model 46.1% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -10260,13 +10260,13 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5471266094420602</v>
+        <v>0.5392180180180179</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-121</v>
+        <v>-117</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>-133</v>
+        <v>-122</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -10290,7 +10290,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 54.7% (fair -121). Your call.</t>
+          <t>Model 53.9% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -10332,7 +10332,7 @@
         <v>106</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -10398,7 +10398,7 @@
         <v>-106</v>
       </c>
       <c r="H20" s="15" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="I20" s="13">
         <f>IF($H$20="","",IF($H$20&lt;0,-$H$20/(-$H$20+100),100/($H$20+100)))</f>
@@ -10464,7 +10464,7 @@
         <v>162</v>
       </c>
       <c r="H21" s="15" t="n">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="I21" s="13">
         <f>IF($H$21="","",IF($H$21&lt;0,-$H$21/(-$H$21+100),100/($H$21+100)))</f>
@@ -10530,7 +10530,7 @@
         <v>-162</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>-114</v>
+        <v>-125</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -10590,10 +10590,10 @@
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.4869124423963134</v>
+        <v>0.4864055299539171</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H23" s="15" t="n">
         <v>117</v>
@@ -10620,7 +10620,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 48.7% (fair +105). Your call.</t>
+          <t>Model 48.6% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -10656,13 +10656,13 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5130851851851852</v>
+        <v>0.5135599078341013</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-105</v>
+        <v>-106</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>-116</v>
+        <v>-117</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -10686,7 +10686,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 51.3% (fair -105). Your call.</t>
+          <t>Model 51.4% (fair -106). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -10718,17 +10718,17 @@
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Over 9</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.4297</v>
+        <v>0.4242502487562189</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>-104</v>
+        <v>-101</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -10752,7 +10752,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 43.0% (fair +133). Your call.</t>
+          <t>Model 42.4% (fair +136). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -10784,17 +10784,17 @@
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Under 8.5</t>
+          <t>Under 9</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.5703</v>
+        <v>0.5757692307692307</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>-133</v>
+        <v>-136</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>126</v>
+        <v>108</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -10818,7 +10818,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 57.0% (fair -133). Your call.</t>
+          <t>Model 57.6% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -10860,7 +10860,7 @@
         <v>187</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -10992,7 +10992,7 @@
         <v>157</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -11124,7 +11124,7 @@
         <v>109</v>
       </c>
       <c r="H31" s="15" t="n">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="I31" s="13">
         <f>IF($H$31="","",IF($H$31&lt;0,-$H$31/(-$H$31+100),100/($H$31+100)))</f>
@@ -11190,7 +11190,7 @@
         <v>-109</v>
       </c>
       <c r="H32" s="15" t="n">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="I32" s="13">
         <f>IF($H$32="","",IF($H$32&lt;0,-$H$32/(-$H$32+100),100/($H$32+100)))</f>
@@ -11250,13 +11250,13 @@
         </is>
       </c>
       <c r="F33" s="13" t="n">
-        <v>0.4737</v>
+        <v>0.4526521739130435</v>
       </c>
       <c r="G33" s="14" t="n">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="H33" s="15" t="n">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="I33" s="13">
         <f>IF($H$33="","",IF($H$33&lt;0,-$H$33/(-$H$33+100),100/($H$33+100)))</f>
@@ -11280,7 +11280,7 @@
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>Model 47.4% (fair +111). Your call.</t>
+          <t>Model 45.3% (fair +121). Your call.</t>
         </is>
       </c>
       <c r="O33" s="15" t="n"/>
@@ -11316,13 +11316,13 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.5263</v>
+        <v>0.5473384615384616</v>
       </c>
       <c r="G34" s="14" t="n">
-        <v>-111</v>
+        <v>-121</v>
       </c>
       <c r="H34" s="15" t="n">
-        <v>108</v>
+        <v>-134</v>
       </c>
       <c r="I34" s="13">
         <f>IF($H$34="","",IF($H$34&lt;0,-$H$34/(-$H$34+100),100/($H$34+100)))</f>
@@ -11346,7 +11346,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>Model 52.6% (fair -111). Your call.</t>
+          <t>Model 54.7% (fair -121). Your call.</t>
         </is>
       </c>
       <c r="O34" s="15" t="n"/>
@@ -11382,13 +11382,13 @@
         </is>
       </c>
       <c r="F35" s="13" t="n">
-        <v>0.4607659574468085</v>
+        <v>0.4602118644067796</v>
       </c>
       <c r="G35" s="14" t="n">
         <v>117</v>
       </c>
       <c r="H35" s="15" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I35" s="13">
         <f>IF($H$35="","",IF($H$35&lt;0,-$H$35/(-$H$35+100),100/($H$35+100)))</f>
@@ -11412,7 +11412,7 @@
       </c>
       <c r="N35" s="19" t="inlineStr">
         <is>
-          <t>Model 46.1% (fair +117). Your call.</t>
+          <t>Model 46.0% (fair +117). Your call.</t>
         </is>
       </c>
       <c r="O35" s="15" t="n"/>
@@ -11448,7 +11448,7 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.5392493562231759</v>
+        <v>0.5397630901287553</v>
       </c>
       <c r="G36" s="14" t="n">
         <v>-117</v>
@@ -11478,7 +11478,7 @@
       </c>
       <c r="N36" s="19" t="inlineStr">
         <is>
-          <t>Model 53.9% (fair -117). Your call.</t>
+          <t>Model 54.0% (fair -117). Your call.</t>
         </is>
       </c>
       <c r="O36" s="15" t="n"/>
@@ -11520,7 +11520,7 @@
         <v>161</v>
       </c>
       <c r="H37" s="15" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I37" s="13">
         <f>IF($H$37="","",IF($H$37&lt;0,-$H$37/(-$H$37+100),100/($H$37+100)))</f>
@@ -11652,7 +11652,7 @@
         <v>179</v>
       </c>
       <c r="H39" s="15" t="n">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="I39" s="13">
         <f>IF($H$39="","",IF($H$39&lt;0,-$H$39/(-$H$39+100),100/($H$39+100)))</f>
@@ -11778,10 +11778,10 @@
         </is>
       </c>
       <c r="F41" s="13" t="n">
-        <v>0.3566806722689076</v>
+        <v>0.3608823529411765</v>
       </c>
       <c r="G41" s="14" t="n">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="H41" s="15" t="n">
         <v>138</v>
@@ -11808,7 +11808,7 @@
       </c>
       <c r="N41" s="19" t="inlineStr">
         <is>
-          <t>Model 35.7% (fair +180). Your call.</t>
+          <t>Model 36.1% (fair +177). Your call.</t>
         </is>
       </c>
       <c r="O41" s="15" t="n"/>
@@ -11844,13 +11844,13 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.6433344398340248</v>
+        <v>0.6390913043478261</v>
       </c>
       <c r="G42" s="14" t="n">
-        <v>-180</v>
+        <v>-177</v>
       </c>
       <c r="H42" s="15" t="n">
-        <v>-141</v>
+        <v>-130</v>
       </c>
       <c r="I42" s="13">
         <f>IF($H$42="","",IF($H$42&lt;0,-$H$42/(-$H$42+100),100/($H$42+100)))</f>
@@ -11874,7 +11874,7 @@
       </c>
       <c r="N42" s="19" t="inlineStr">
         <is>
-          <t>Model 64.3% (fair -180). Your call.</t>
+          <t>Model 63.9% (fair -177). Your call.</t>
         </is>
       </c>
       <c r="O42" s="15" t="n"/>
@@ -11906,7 +11906,7 @@
       </c>
       <c r="E43" s="12" t="inlineStr">
         <is>
-          <t>Over 9.5</t>
+          <t>Over 9</t>
         </is>
       </c>
       <c r="F43" s="13" t="n">
@@ -11916,7 +11916,7 @@
         <v>111</v>
       </c>
       <c r="H43" s="15" t="n">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="I43" s="13">
         <f>IF($H$43="","",IF($H$43&lt;0,-$H$43/(-$H$43+100),100/($H$43+100)))</f>
@@ -11972,7 +11972,7 @@
       </c>
       <c r="E44" s="20" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Under 9</t>
         </is>
       </c>
       <c r="F44" s="13" t="n">
@@ -12048,7 +12048,7 @@
         <v>-133</v>
       </c>
       <c r="H45" s="15" t="n">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="I45" s="13">
         <f>IF($H$45="","",IF($H$45&lt;0,-$H$45/(-$H$45+100),100/($H$45+100)))</f>
@@ -12114,7 +12114,7 @@
         <v>133</v>
       </c>
       <c r="H46" s="15" t="n">
-        <v>-105</v>
+        <v>-112</v>
       </c>
       <c r="I46" s="13">
         <f>IF($H$46="","",IF($H$46&lt;0,-$H$46/(-$H$46+100),100/($H$46+100)))</f>
@@ -12174,13 +12174,13 @@
         </is>
       </c>
       <c r="F47" s="13" t="n">
-        <v>0.4344957983193278</v>
+        <v>0.4293032786885246</v>
       </c>
       <c r="G47" s="14" t="n">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="H47" s="15" t="n">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="I47" s="13">
         <f>IF($H$47="","",IF($H$47&lt;0,-$H$47/(-$H$47+100),100/($H$47+100)))</f>
@@ -12204,7 +12204,7 @@
       </c>
       <c r="N47" s="19" t="inlineStr">
         <is>
-          <t>Model 43.4% (fair +130). Your call.</t>
+          <t>Model 42.9% (fair +133). Your call.</t>
         </is>
       </c>
       <c r="O47" s="15" t="n"/>
@@ -12240,13 +12240,13 @@
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.5655100840336135</v>
+        <v>0.5706885245901639</v>
       </c>
       <c r="G48" s="14" t="n">
-        <v>-130</v>
+        <v>-133</v>
       </c>
       <c r="H48" s="15" t="n">
-        <v>-138</v>
+        <v>-144</v>
       </c>
       <c r="I48" s="13">
         <f>IF($H$48="","",IF($H$48&lt;0,-$H$48/(-$H$48+100),100/($H$48+100)))</f>
@@ -12270,7 +12270,7 @@
       </c>
       <c r="N48" s="19" t="inlineStr">
         <is>
-          <t>Model 56.6% (fair -130). Your call.</t>
+          <t>Model 57.1% (fair -133). Your call.</t>
         </is>
       </c>
       <c r="O48" s="15" t="n"/>
@@ -12302,17 +12302,17 @@
       </c>
       <c r="E49" s="12" t="inlineStr">
         <is>
-          <t>Over 12</t>
+          <t>Over 11.5</t>
         </is>
       </c>
       <c r="F49" s="13" t="n">
-        <v>0.1153</v>
+        <v>0.185</v>
       </c>
       <c r="G49" s="14" t="n">
-        <v>767</v>
+        <v>441</v>
       </c>
       <c r="H49" s="15" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I49" s="13">
         <f>IF($H$49="","",IF($H$49&lt;0,-$H$49/(-$H$49+100),100/($H$49+100)))</f>
@@ -12336,7 +12336,7 @@
       </c>
       <c r="N49" s="19" t="inlineStr">
         <is>
-          <t>Model 11.5% (fair +767). Your call.</t>
+          <t>Model 18.5% (fair +441). Your call.</t>
         </is>
       </c>
       <c r="O49" s="15" t="n"/>
@@ -12368,17 +12368,17 @@
       </c>
       <c r="E50" s="20" t="inlineStr">
         <is>
-          <t>Under 12</t>
+          <t>Under 11.5</t>
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.8847</v>
+        <v>0.8149999999999999</v>
       </c>
       <c r="G50" s="14" t="n">
-        <v>-767</v>
+        <v>-441</v>
       </c>
       <c r="H50" s="15" t="n">
-        <v>100</v>
+        <v>122</v>
       </c>
       <c r="I50" s="13">
         <f>IF($H$50="","",IF($H$50&lt;0,-$H$50/(-$H$50+100),100/($H$50+100)))</f>
@@ -12402,7 +12402,7 @@
       </c>
       <c r="N50" s="19" t="inlineStr">
         <is>
-          <t>Model 88.5% (fair -767). Your call.</t>
+          <t>Model 81.5% (fair -441). Your call.</t>
         </is>
       </c>
       <c r="O50" s="15" t="n"/>
@@ -12510,7 +12510,7 @@
         <v>-144</v>
       </c>
       <c r="H52" s="15" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="I52" s="13">
         <f>IF($H$52="","",IF($H$52&lt;0,-$H$52/(-$H$52+100),100/($H$52+100)))</f>
@@ -12570,13 +12570,13 @@
         </is>
       </c>
       <c r="F53" s="13" t="n">
-        <v>0.4803964757709251</v>
+        <v>0.4787826086956522</v>
       </c>
       <c r="G53" s="14" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H53" s="15" t="n">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="I53" s="13">
         <f>IF($H$53="","",IF($H$53&lt;0,-$H$53/(-$H$53+100),100/($H$53+100)))</f>
@@ -12600,7 +12600,7 @@
       </c>
       <c r="N53" s="19" t="inlineStr">
         <is>
-          <t>Model 48.0% (fair +108). Your call.</t>
+          <t>Model 47.9% (fair +109). Your call.</t>
         </is>
       </c>
       <c r="O53" s="15" t="n"/>
@@ -12636,10 +12636,10 @@
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.5195810572687225</v>
+        <v>0.5212035242290749</v>
       </c>
       <c r="G54" s="14" t="n">
-        <v>-108</v>
+        <v>-109</v>
       </c>
       <c r="H54" s="15" t="n">
         <v>-127</v>
@@ -12666,7 +12666,7 @@
       </c>
       <c r="N54" s="19" t="inlineStr">
         <is>
-          <t>Model 52.0% (fair -108). Your call.</t>
+          <t>Model 52.1% (fair -109). Your call.</t>
         </is>
       </c>
       <c r="O54" s="15" t="n"/>
@@ -12708,7 +12708,7 @@
         <v>107</v>
       </c>
       <c r="H55" s="15" t="n">
-        <v>107</v>
+        <v>-101</v>
       </c>
       <c r="I55" s="13">
         <f>IF($H$55="","",IF($H$55&lt;0,-$H$55/(-$H$55+100),100/($H$55+100)))</f>
@@ -12774,7 +12774,7 @@
         <v>-107</v>
       </c>
       <c r="H56" s="15" t="n">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="I56" s="13">
         <f>IF($H$56="","",IF($H$56&lt;0,-$H$56/(-$H$56+100),100/($H$56+100)))</f>
@@ -12840,7 +12840,7 @@
         <v>183</v>
       </c>
       <c r="H57" s="15" t="n">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="I57" s="13">
         <f>IF($H$57="","",IF($H$57&lt;0,-$H$57/(-$H$57+100),100/($H$57+100)))</f>
@@ -12906,7 +12906,7 @@
         <v>-183</v>
       </c>
       <c r="H58" s="15" t="n">
-        <v>-121</v>
+        <v>-115</v>
       </c>
       <c r="I58" s="13">
         <f>IF($H$58="","",IF($H$58&lt;0,-$H$58/(-$H$58+100),100/($H$58+100)))</f>
@@ -12966,13 +12966,13 @@
         </is>
       </c>
       <c r="F59" s="13" t="n">
-        <v>0.5124757709251102</v>
+        <v>0.5153652173913044</v>
       </c>
       <c r="G59" s="14" t="n">
-        <v>-105</v>
+        <v>-106</v>
       </c>
       <c r="H59" s="15" t="n">
-        <v>-127</v>
+        <v>-130</v>
       </c>
       <c r="I59" s="13">
         <f>IF($H$59="","",IF($H$59&lt;0,-$H$59/(-$H$59+100),100/($H$59+100)))</f>
@@ -12996,7 +12996,7 @@
       </c>
       <c r="N59" s="19" t="inlineStr">
         <is>
-          <t>Model 51.2% (fair -105). Your call.</t>
+          <t>Model 51.5% (fair -106). Your call.</t>
         </is>
       </c>
       <c r="O59" s="15" t="n"/>
@@ -13032,13 +13032,13 @@
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>0.4875330396475771</v>
+        <v>0.4846521739130435</v>
       </c>
       <c r="G60" s="14" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H60" s="15" t="n">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="I60" s="13">
         <f>IF($H$60="","",IF($H$60&lt;0,-$H$60/(-$H$60+100),100/($H$60+100)))</f>
@@ -13062,7 +13062,7 @@
       </c>
       <c r="N60" s="19" t="inlineStr">
         <is>
-          <t>Model 48.8% (fair +105). Your call.</t>
+          <t>Model 48.5% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O60" s="15" t="n"/>
@@ -13094,17 +13094,17 @@
       </c>
       <c r="E61" s="12" t="inlineStr">
         <is>
-          <t>Over 12</t>
+          <t>Over 11.5</t>
         </is>
       </c>
       <c r="F61" s="13" t="n">
-        <v>0.2727</v>
+        <v>0.378</v>
       </c>
       <c r="G61" s="14" t="n">
-        <v>267</v>
+        <v>165</v>
       </c>
       <c r="H61" s="15" t="n">
-        <v>129</v>
+        <v>-108</v>
       </c>
       <c r="I61" s="13">
         <f>IF($H$61="","",IF($H$61&lt;0,-$H$61/(-$H$61+100),100/($H$61+100)))</f>
@@ -13128,7 +13128,7 @@
       </c>
       <c r="N61" s="19" t="inlineStr">
         <is>
-          <t>Model 27.3% (fair +267). Your call.</t>
+          <t>Model 37.8% (fair +165). Your call.</t>
         </is>
       </c>
       <c r="O61" s="15" t="n"/>
@@ -13160,17 +13160,17 @@
       </c>
       <c r="E62" s="20" t="inlineStr">
         <is>
-          <t>Under 12</t>
+          <t>Under 11.5</t>
         </is>
       </c>
       <c r="F62" s="13" t="n">
-        <v>0.7273000000000001</v>
+        <v>0.622</v>
       </c>
       <c r="G62" s="14" t="n">
-        <v>-267</v>
+        <v>-165</v>
       </c>
       <c r="H62" s="15" t="n">
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="I62" s="13">
         <f>IF($H$62="","",IF($H$62&lt;0,-$H$62/(-$H$62+100),100/($H$62+100)))</f>
@@ -13194,7 +13194,7 @@
       </c>
       <c r="N62" s="19" t="inlineStr">
         <is>
-          <t>Model 72.7% (fair -267). Your call.</t>
+          <t>Model 62.2% (fair -165). Your call.</t>
         </is>
       </c>
       <c r="O62" s="15" t="n"/>
@@ -13302,7 +13302,7 @@
         <v>-144</v>
       </c>
       <c r="H64" s="15" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="I64" s="13">
         <f>IF($H$64="","",IF($H$64&lt;0,-$H$64/(-$H$64+100),100/($H$64+100)))</f>
@@ -13878,13 +13878,13 @@
         </is>
       </c>
       <c r="F73" s="13" t="n">
-        <v>0.534264705882353</v>
+        <v>0.5318269230769231</v>
       </c>
       <c r="G73" s="14" t="n">
-        <v>-115</v>
+        <v>-114</v>
       </c>
       <c r="H73" s="15" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I73" s="13">
         <f>IF($H$73="","",IF($H$73&lt;0,-$H$73/(-$H$73+100),100/($H$73+100)))</f>
@@ -13908,7 +13908,7 @@
       </c>
       <c r="N73" s="19" t="inlineStr">
         <is>
-          <t>Model 53.4% (fair -115). Your call.</t>
+          <t>Model 53.2% (fair -114). Your call.</t>
         </is>
       </c>
       <c r="O73" s="15" t="n"/>
@@ -13944,10 +13944,10 @@
         </is>
       </c>
       <c r="F74" s="13" t="n">
-        <v>0.46575</v>
+        <v>0.46815</v>
       </c>
       <c r="G74" s="14" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H74" s="15" t="n">
         <v>100</v>
@@ -13974,7 +13974,7 @@
       </c>
       <c r="N74" s="19" t="inlineStr">
         <is>
-          <t>Model 46.6% (fair +115). Your call.</t>
+          <t>Model 46.8% (fair +114). Your call.</t>
         </is>
       </c>
       <c r="O74" s="15" t="n"/>
@@ -14010,10 +14010,10 @@
         </is>
       </c>
       <c r="F75" s="13" t="n">
-        <v>0.383273381294964</v>
+        <v>0.4068</v>
       </c>
       <c r="G75" s="14" t="n">
-        <v>161</v>
+        <v>146</v>
       </c>
       <c r="H75" s="15" t="n">
         <v>178</v>
@@ -14040,7 +14040,7 @@
       </c>
       <c r="N75" s="19" t="inlineStr">
         <is>
-          <t>Model 38.3% (fair +161). Your call.</t>
+          <t>Model 40.7% (fair +146). Your call.</t>
         </is>
       </c>
       <c r="O75" s="15" t="n"/>
@@ -14076,13 +14076,13 @@
         </is>
       </c>
       <c r="F76" s="13" t="n">
-        <v>0.6167251798561151</v>
+        <v>0.5931999999999999</v>
       </c>
       <c r="G76" s="14" t="n">
-        <v>-161</v>
+        <v>-146</v>
       </c>
       <c r="H76" s="15" t="n">
-        <v>-178</v>
+        <v>-163</v>
       </c>
       <c r="I76" s="13">
         <f>IF($H$76="","",IF($H$76&lt;0,-$H$76/(-$H$76+100),100/($H$76+100)))</f>
@@ -14106,7 +14106,7 @@
       </c>
       <c r="N76" s="19" t="inlineStr">
         <is>
-          <t>Model 61.7% (fair -161). Your call.</t>
+          <t>Model 59.3% (fair -146). Your call.</t>
         </is>
       </c>
       <c r="O76" s="15" t="n"/>
@@ -14346,7 +14346,7 @@
         <v>102</v>
       </c>
       <c r="H80" s="15" t="n">
-        <v>-111</v>
+        <v>-108</v>
       </c>
       <c r="I80" s="13">
         <f>IF($H$80="","",IF($H$80&lt;0,-$H$80/(-$H$80+100),100/($H$80+100)))</f>
@@ -14670,13 +14670,13 @@
         </is>
       </c>
       <c r="F85" s="13" t="n">
-        <v>0.4947967741935483</v>
+        <v>0.4922131455399061</v>
       </c>
       <c r="G85" s="14" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H85" s="15" t="n">
-        <v>-117</v>
+        <v>-113</v>
       </c>
       <c r="I85" s="13">
         <f>IF($H$85="","",IF($H$85&lt;0,-$H$85/(-$H$85+100),100/($H$85+100)))</f>
@@ -14700,7 +14700,7 @@
       </c>
       <c r="N85" s="19" t="inlineStr">
         <is>
-          <t>Model 49.5% (fair +102). Your call.</t>
+          <t>Model 49.2% (fair +103). Your call.</t>
         </is>
       </c>
       <c r="O85" s="15" t="n"/>
@@ -14736,13 +14736,13 @@
         </is>
       </c>
       <c r="F86" s="13" t="n">
-        <v>0.5051851851851852</v>
+        <v>0.5077674418604651</v>
       </c>
       <c r="G86" s="14" t="n">
-        <v>-102</v>
+        <v>-103</v>
       </c>
       <c r="H86" s="15" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I86" s="13">
         <f>IF($H$86="","",IF($H$86&lt;0,-$H$86/(-$H$86+100),100/($H$86+100)))</f>
@@ -14766,7 +14766,7 @@
       </c>
       <c r="N86" s="19" t="inlineStr">
         <is>
-          <t>Model 50.5% (fair -102). Your call.</t>
+          <t>Model 50.8% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O86" s="15" t="n"/>
@@ -14802,13 +14802,13 @@
         </is>
       </c>
       <c r="F87" s="13" t="n">
-        <v>0.3564444444444445</v>
+        <v>0.3595057034220532</v>
       </c>
       <c r="G87" s="14" t="n">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="H87" s="15" t="n">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="I87" s="13">
         <f>IF($H$87="","",IF($H$87&lt;0,-$H$87/(-$H$87+100),100/($H$87+100)))</f>
@@ -14832,7 +14832,7 @@
       </c>
       <c r="N87" s="19" t="inlineStr">
         <is>
-          <t>Model 35.6% (fair +181). Your call.</t>
+          <t>Model 36.0% (fair +178). Your call.</t>
         </is>
       </c>
       <c r="O87" s="15" t="n"/>
@@ -14868,10 +14868,10 @@
         </is>
       </c>
       <c r="F88" s="13" t="n">
-        <v>0.6435444444444444</v>
+        <v>0.6405222222222222</v>
       </c>
       <c r="G88" s="14" t="n">
-        <v>-181</v>
+        <v>-178</v>
       </c>
       <c r="H88" s="15" t="n">
         <v>-170</v>
@@ -14898,7 +14898,7 @@
       </c>
       <c r="N88" s="19" t="inlineStr">
         <is>
-          <t>Model 64.4% (fair -181). Your call.</t>
+          <t>Model 64.1% (fair -178). Your call.</t>
         </is>
       </c>
       <c r="O88" s="15" t="n"/>
@@ -15847,10 +15847,10 @@
         </is>
       </c>
       <c r="F5" s="13" t="n">
-        <v>0.5591</v>
+        <v>0.4423</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-127</v>
+        <v>126</v>
       </c>
       <c r="H5" s="15" t="n"/>
       <c r="I5" s="13">
@@ -15875,7 +15875,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Model 55.9% (fair -127). Your call.</t>
+          <t>Model 44.2% (fair +126). Your call.</t>
         </is>
       </c>
       <c r="O5" s="15" t="n"/>
@@ -15911,10 +15911,10 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.4409</v>
+        <v>0.5577</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>127</v>
+        <v>-126</v>
       </c>
       <c r="H6" s="15" t="n"/>
       <c r="I6" s="13">
@@ -15939,7 +15939,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 44.1% (fair +127). Your call.</t>
+          <t>Model 55.8% (fair -126). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>

</xml_diff>

<commit_message>
data: hourly update 2026-06-30 00:06Z
</commit_message>
<xml_diff>
--- a/data/output/workbook/2026-06-29.xlsx
+++ b/data/output/workbook/2026-06-29.xlsx
@@ -953,7 +953,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29 18:56</t>
+          <t>2026-06-29 20:06</t>
         </is>
       </c>
     </row>
@@ -8186,32 +8186,32 @@
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Chicago Cubs</t>
+          <t>Cincinnati Reds @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>00:05</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Under 11.5</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>0.6345499999999999</v>
+        <v>0.627090990990991</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-174</v>
+        <v>-168</v>
       </c>
       <c r="H6" s="15" t="n">
-        <v>100</v>
+        <v>-122</v>
       </c>
       <c r="I6" s="13">
         <f>IF($H$6="","",IF($H$6&lt;0,-$H$6/(-$H$6+100),100/($H$6+100)))</f>
@@ -8235,7 +8235,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Model 63.5% (fair -174). Your call.</t>
+          <t>Model 62.7% (fair -168). Your call.</t>
         </is>
       </c>
       <c r="O6" s="15" t="n"/>
@@ -8252,29 +8252,29 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Miami Marlins @ Colorado Rockies</t>
+          <t>Pittsburgh Pirates @ Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>00:40</t>
+          <t>22:40</t>
         </is>
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Under 12</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.5832211538461538</v>
+        <v>0.5466346153846153</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>-140</v>
+        <v>-121</v>
       </c>
       <c r="H7" s="15" t="n">
         <v>108</v>
@@ -8301,7 +8301,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 58.3% (fair -140). Your call.</t>
+          <t>Model 54.7% (fair -121). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -8318,32 +8318,32 @@
       </c>
       <c r="B8" s="20" t="inlineStr">
         <is>
-          <t>Detroit Tigers @ New York Yankees</t>
+          <t>Washington Nationals @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>23:05</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D8" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>New York Yankees -1.5</t>
+          <t>Under 10.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.4086785714285715</v>
+        <v>0.56645</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>145</v>
+        <v>-131</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>180</v>
+        <v>100</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -8367,7 +8367,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 40.9% (fair +145). Your call.</t>
+          <t>Model 56.6% (fair -131). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -8379,37 +8379,37 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Philadelphia Phillies</t>
+          <t>Detroit Tigers @ New York Yankees</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>22:40</t>
+          <t>23:05</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>New York Yankees -1.5</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
-        <v>0.5466346153846153</v>
+        <v>0.4103260869565218</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-121</v>
+        <v>144</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>108</v>
+        <v>176</v>
       </c>
       <c r="I9" s="13">
         <f>IF($H$9="","",IF($H$9&lt;0,-$H$9/(-$H$9+100),100/($H$9+100)))</f>
@@ -8433,7 +8433,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Model 54.7% (fair -121). Your call.</t>
+          <t>Model 41.0% (fair +144). Your call.</t>
         </is>
       </c>
       <c r="O9" s="15" t="n"/>
@@ -8450,12 +8450,12 @@
       </c>
       <c r="B10" s="20" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Milwaukee Brewers</t>
+          <t>Texas Rangers @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>23:40</t>
+          <t>23:10</t>
         </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
@@ -8465,17 +8465,17 @@
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="F10" s="13" t="n">
-        <v>0.6284444444444445</v>
+        <v>0.4492</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-169</v>
+        <v>123</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>-125</v>
+        <v>150</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -8499,7 +8499,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Model 62.8% (fair -169). Your call.</t>
+          <t>Model 44.9% (fair +123). Your call.</t>
         </is>
       </c>
       <c r="O10" s="15" t="n"/>
@@ -8709,37 +8709,37 @@
     <row r="14">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>St. Louis Cardinals @ Atlanta Braves</t>
+          <t>Miami Marlins @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>23:15</t>
+          <t>00:40</t>
         </is>
       </c>
       <c r="D14" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="F14" s="13" t="n">
-        <v>0.5644039215686274</v>
+        <v>0.455</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>-130</v>
+        <v>120</v>
       </c>
       <c r="H14" s="15" t="n">
-        <v>-104</v>
+        <v>144</v>
       </c>
       <c r="I14" s="13">
         <f>IF($H$14="","",IF($H$14&lt;0,-$H$14/(-$H$14+100),100/($H$14+100)))</f>
@@ -8763,7 +8763,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Model 56.4% (fair -130). Your call.</t>
+          <t>Model 45.5% (fair +120). Your call.</t>
         </is>
       </c>
       <c r="O14" s="15" t="n"/>
@@ -8775,37 +8775,37 @@
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>Texas Rangers @ Cleveland Guardians</t>
+          <t>St. Louis Cardinals @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>0.4521311475409836</v>
+        <v>0.5644039215686274</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>121</v>
+        <v>-130</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>144</v>
+        <v>-104</v>
       </c>
       <c r="I15" s="13">
         <f>IF($H$15="","",IF($H$15&lt;0,-$H$15/(-$H$15+100),100/($H$15+100)))</f>
@@ -8829,7 +8829,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Model 45.2% (fair +121). Your call.</t>
+          <t>Model 56.4% (fair -130). Your call.</t>
         </is>
       </c>
       <c r="O15" s="15" t="n"/>
@@ -8846,12 +8846,12 @@
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>Washington Nationals @ Boston Red Sox</t>
+          <t>Pittsburgh Pirates @ Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>23:10</t>
+          <t>22:40</t>
         </is>
       </c>
       <c r="D16" s="20" t="inlineStr">
@@ -8861,17 +8861,17 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>Under 10.5</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="F16" s="13" t="n">
-        <v>0.5712057692307693</v>
+        <v>0.5266346153846153</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-133</v>
+        <v>-111</v>
       </c>
       <c r="H16" s="15" t="n">
-        <v>-108</v>
+        <v>108</v>
       </c>
       <c r="I16" s="13">
         <f>IF($H$16="","",IF($H$16&lt;0,-$H$16/(-$H$16+100),100/($H$16+100)))</f>
@@ -8895,7 +8895,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Model 57.1% (fair -133). Your call.</t>
+          <t>Model 52.7% (fair -111). Your call.</t>
         </is>
       </c>
       <c r="O16" s="15" t="n"/>
@@ -8907,17 +8907,17 @@
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>Miami Marlins @ Colorado Rockies</t>
+          <t>Texas Rangers @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>00:40</t>
+          <t>22:40</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -8927,17 +8927,17 @@
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.4599579831932774</v>
+        <v>0.5355392156862745</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>117</v>
+        <v>-115</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>138</v>
+        <v>104</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -8961,7 +8961,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 46.0% (fair +117). Your call.</t>
+          <t>Model 53.6% (fair -115). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -8973,17 +8973,17 @@
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B18" s="20" t="inlineStr">
         <is>
-          <t>Texas Rangers @ Cleveland Guardians</t>
+          <t>Minnesota Twins @ Houston Astros</t>
         </is>
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
-          <t>22:40</t>
+          <t>00:10</t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
@@ -8993,17 +8993,17 @@
       </c>
       <c r="E18" s="20" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5355392156862745</v>
+        <v>0.4803964757709251</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>-115</v>
+        <v>108</v>
       </c>
       <c r="H18" s="15" t="n">
-        <v>104</v>
+        <v>127</v>
       </c>
       <c r="I18" s="13">
         <f>IF($H$18="","",IF($H$18&lt;0,-$H$18/(-$H$18+100),100/($H$18+100)))</f>
@@ -9027,7 +9027,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 53.6% (fair -115). Your call.</t>
+          <t>Model 48.0% (fair +108). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -9039,37 +9039,37 @@
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Minnesota Twins @ Houston Astros</t>
+          <t>New York Mets @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>00:10</t>
+          <t>23:07</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Under 8</t>
         </is>
       </c>
       <c r="F19" s="13" t="n">
-        <v>0.4803964757709251</v>
+        <v>0.5213942307692307</v>
       </c>
       <c r="G19" s="14" t="n">
+        <v>-109</v>
+      </c>
+      <c r="H19" s="15" t="n">
         <v>108</v>
-      </c>
-      <c r="H19" s="15" t="n">
-        <v>127</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -9093,7 +9093,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Model 48.0% (fair +108). Your call.</t>
+          <t>Model 52.1% (fair -109). Your call.</t>
         </is>
       </c>
       <c r="O19" s="15" t="n"/>
@@ -9110,12 +9110,12 @@
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Philadelphia Phillies</t>
+          <t>Chicago White Sox @ Baltimore Orioles</t>
         </is>
       </c>
       <c r="C20" s="20" t="inlineStr">
         <is>
-          <t>22:40</t>
+          <t>22:35</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
@@ -9125,14 +9125,14 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Over 10.5</t>
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.5238461538461537</v>
+        <v>0.5167788461538462</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>-110</v>
+        <v>-107</v>
       </c>
       <c r="H20" s="15" t="n">
         <v>108</v>
@@ -9159,7 +9159,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Model 52.4% (fair -110). Your call.</t>
+          <t>Model 51.7% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O20" s="15" t="n"/>
@@ -9195,10 +9195,10 @@
         </is>
       </c>
       <c r="F21" s="13" t="n">
-        <v>0.4395491803278689</v>
+        <v>0.4399180327868852</v>
       </c>
       <c r="G21" s="14" t="n">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H21" s="15" t="n">
         <v>144</v>
@@ -9225,7 +9225,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Model 44.0% (fair +128). Your call.</t>
+          <t>Model 44.0% (fair +127). Your call.</t>
         </is>
       </c>
       <c r="O21" s="15" t="n"/>
@@ -9237,37 +9237,37 @@
     <row r="22">
       <c r="A22" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
-          <t>New York Mets @ Toronto Blue Jays</t>
+          <t>Tampa Bay Rays @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C22" s="20" t="inlineStr">
         <is>
-          <t>23:07</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="D22" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>Under 8.5</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.53515</v>
+        <v>0.5157766990291262</v>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-115</v>
+        <v>-107</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -9291,7 +9291,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Model 53.5% (fair -115). Your call.</t>
+          <t>Model 51.6% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O22" s="15" t="n"/>
@@ -9308,12 +9308,12 @@
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Kansas City Royals</t>
+          <t>Chicago White Sox @ Baltimore Orioles</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>23:40</t>
+          <t>22:35</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
@@ -9323,17 +9323,17 @@
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="F23" s="13" t="n">
-        <v>0.5129326923076922</v>
+        <v>0.4461344537815127</v>
       </c>
       <c r="G23" s="14" t="n">
-        <v>-105</v>
+        <v>124</v>
       </c>
       <c r="H23" s="15" t="n">
-        <v>108</v>
+        <v>138</v>
       </c>
       <c r="I23" s="13">
         <f>IF($H$23="","",IF($H$23&lt;0,-$H$23/(-$H$23+100),100/($H$23+100)))</f>
@@ -9357,7 +9357,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Model 51.3% (fair -105). Your call.</t>
+          <t>Model 44.6% (fair +124). Your call.</t>
         </is>
       </c>
       <c r="O23" s="15" t="n"/>
@@ -9374,32 +9374,32 @@
       </c>
       <c r="B24" s="20" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Baltimore Orioles</t>
+          <t>Tampa Bay Rays @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C24" s="20" t="inlineStr">
         <is>
-          <t>22:35</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="D24" s="20" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="E24" s="20" t="inlineStr">
         <is>
-          <t>Over 10.5</t>
+          <t>Kansas City Royals +1.5</t>
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.5120673076923077</v>
+        <v>0.626577049180328</v>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-105</v>
+        <v>-168</v>
       </c>
       <c r="H24" s="15" t="n">
-        <v>108</v>
+        <v>-144</v>
       </c>
       <c r="I24" s="13">
         <f>IF($H$24="","",IF($H$24&lt;0,-$H$24/(-$H$24+100),100/($H$24+100)))</f>
@@ -9423,7 +9423,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Model 51.2% (fair -105). Your call.</t>
+          <t>Model 62.7% (fair -168). Your call.</t>
         </is>
       </c>
       <c r="O24" s="15" t="n"/>
@@ -9435,17 +9435,17 @@
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Baltimore Orioles</t>
+          <t>New York Mets @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>22:35</t>
+          <t>23:07</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
@@ -9455,17 +9455,17 @@
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.4461344537815127</v>
+        <v>0.4864055299539171</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>124</v>
+        <v>106</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>138</v>
+        <v>117</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -9489,7 +9489,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 44.6% (fair +124). Your call.</t>
+          <t>Model 48.6% (fair +106). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -9506,32 +9506,32 @@
       </c>
       <c r="B26" s="20" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Kansas City Royals</t>
+          <t>Detroit Tigers @ New York Yankees</t>
         </is>
       </c>
       <c r="C26" s="20" t="inlineStr">
         <is>
-          <t>23:40</t>
+          <t>23:05</t>
         </is>
       </c>
       <c r="D26" s="20" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Kansas City Royals +1.5</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.6269326530612244</v>
+        <v>0.5874449339207048</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>-168</v>
+        <v>-142</v>
       </c>
       <c r="H26" s="15" t="n">
-        <v>-145</v>
+        <v>-127</v>
       </c>
       <c r="I26" s="13">
         <f>IF($H$26="","",IF($H$26&lt;0,-$H$26/(-$H$26+100),100/($H$26+100)))</f>
@@ -9555,7 +9555,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 62.7% (fair -168). Your call.</t>
+          <t>Model 58.7% (fair -142). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -9572,12 +9572,12 @@
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>New York Mets @ Toronto Blue Jays</t>
+          <t>Detroit Tigers @ New York Yankees</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>23:07</t>
+          <t>23:05</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
@@ -9587,17 +9587,17 @@
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="F27" s="13" t="n">
-        <v>0.4864055299539171</v>
+        <v>0.4580263157894736</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="I27" s="13">
         <f>IF($H$27="","",IF($H$27&lt;0,-$H$27/(-$H$27+100),100/($H$27+100)))</f>
@@ -9621,7 +9621,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Model 48.6% (fair +106). Your call.</t>
+          <t>Model 45.8% (fair +118). Your call.</t>
         </is>
       </c>
       <c r="O27" s="15" t="n"/>
@@ -9638,32 +9638,32 @@
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
-          <t>Detroit Tigers @ New York Yankees</t>
+          <t>Cincinnati Reds @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C28" s="20" t="inlineStr">
         <is>
-          <t>23:05</t>
+          <t>23:40</t>
         </is>
       </c>
       <c r="D28" s="20" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="E28" s="20" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.5874449339207048</v>
+        <v>0.5523206572769952</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-142</v>
+        <v>-123</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>-127</v>
+        <v>-113</v>
       </c>
       <c r="I28" s="13">
         <f>IF($H$28="","",IF($H$28&lt;0,-$H$28/(-$H$28+100),100/($H$28+100)))</f>
@@ -9687,7 +9687,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Model 58.7% (fair -142). Your call.</t>
+          <t>Model 55.2% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O28" s="15" t="n"/>
@@ -9699,37 +9699,37 @@
     <row r="29">
       <c r="A29" s="12" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Milwaukee Brewers</t>
+          <t>Chicago White Sox @ Baltimore Orioles</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>23:40</t>
+          <t>22:35</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="F29" s="13" t="n">
-        <v>0.5523206572769952</v>
+        <v>0.4650900900900901</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-123</v>
+        <v>115</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>-113</v>
+        <v>122</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -9753,7 +9753,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Model 55.2% (fair -123). Your call.</t>
+          <t>Model 46.5% (fair +115). Your call.</t>
         </is>
       </c>
       <c r="O29" s="15" t="n"/>
@@ -10058,14 +10058,14 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Over 9.5</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>0.4763</v>
+        <v>0.576</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>110</v>
+        <v>-136</v>
       </c>
       <c r="H7" s="15" t="n">
         <v>113</v>
@@ -10092,7 +10092,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Model 47.6% (fair +110). Your call.</t>
+          <t>Model 57.6% (fair -136). Your call.</t>
         </is>
       </c>
       <c r="O7" s="15" t="n"/>
@@ -10124,17 +10124,17 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Under 8.5</t>
         </is>
       </c>
       <c r="F8" s="13" t="n">
-        <v>0.5237000000000001</v>
+        <v>0.424</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>-110</v>
+        <v>136</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>128</v>
+        <v>105</v>
       </c>
       <c r="I8" s="13">
         <f>IF($H$8="","",IF($H$8&lt;0,-$H$8/(-$H$8+100),100/($H$8+100)))</f>
@@ -10158,7 +10158,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Model 52.4% (fair -110). Your call.</t>
+          <t>Model 42.4% (fair +136). Your call.</t>
         </is>
       </c>
       <c r="O8" s="15" t="n"/>
@@ -10266,7 +10266,7 @@
         <v>-155</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>163</v>
+        <v>130</v>
       </c>
       <c r="I10" s="13">
         <f>IF($H$10="","",IF($H$10&lt;0,-$H$10/(-$H$10+100),100/($H$10+100)))</f>
@@ -10722,13 +10722,13 @@
         </is>
       </c>
       <c r="F17" s="13" t="n">
-        <v>0.4591150442477877</v>
+        <v>0.4580263157894736</v>
       </c>
       <c r="G17" s="14" t="n">
         <v>118</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="I17" s="13">
         <f>IF($H$17="","",IF($H$17&lt;0,-$H$17/(-$H$17+100),100/($H$17+100)))</f>
@@ -10752,7 +10752,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Model 45.9% (fair +118). Your call.</t>
+          <t>Model 45.8% (fair +118). Your call.</t>
         </is>
       </c>
       <c r="O17" s="15" t="n"/>
@@ -10788,7 +10788,7 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.5408969162995595</v>
+        <v>0.5419599118942732</v>
       </c>
       <c r="G18" s="14" t="n">
         <v>-118</v>
@@ -10818,7 +10818,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Model 54.1% (fair -118). Your call.</t>
+          <t>Model 54.2% (fair -118). Your call.</t>
         </is>
       </c>
       <c r="O18" s="15" t="n"/>
@@ -10860,7 +10860,7 @@
         <v>106</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>100</v>
+        <v>-105</v>
       </c>
       <c r="I19" s="13">
         <f>IF($H$19="","",IF($H$19&lt;0,-$H$19/(-$H$19+100),100/($H$19+100)))</f>
@@ -11058,7 +11058,7 @@
         <v>-162</v>
       </c>
       <c r="H22" s="15" t="n">
-        <v>-116</v>
+        <v>-113</v>
       </c>
       <c r="I22" s="13">
         <f>IF($H$22="","",IF($H$22&lt;0,-$H$22/(-$H$22+100),100/($H$22+100)))</f>
@@ -11246,17 +11246,17 @@
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Over 9</t>
         </is>
       </c>
       <c r="F25" s="13" t="n">
-        <v>0.46485</v>
+        <v>0.3375</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>115</v>
+        <v>196</v>
       </c>
       <c r="H25" s="15" t="n">
-        <v>100</v>
+        <v>121</v>
       </c>
       <c r="I25" s="13">
         <f>IF($H$25="","",IF($H$25&lt;0,-$H$25/(-$H$25+100),100/($H$25+100)))</f>
@@ -11280,7 +11280,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Model 46.5% (fair +115). Your call.</t>
+          <t>Model 33.8% (fair +196). Your call.</t>
         </is>
       </c>
       <c r="O25" s="15" t="n"/>
@@ -11312,14 +11312,14 @@
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>Under 8.5</t>
+          <t>Under 9</t>
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.53515</v>
+        <v>0.6625</v>
       </c>
       <c r="G26" s="14" t="n">
-        <v>-115</v>
+        <v>-196</v>
       </c>
       <c r="H26" s="15" t="n">
         <v>100</v>
@@ -11346,7 +11346,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Model 53.5% (fair -115). Your call.</t>
+          <t>Model 66.2% (fair -196). Your call.</t>
         </is>
       </c>
       <c r="O26" s="15" t="n"/>
@@ -11520,7 +11520,7 @@
         <v>157</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="I29" s="13">
         <f>IF($H$29="","",IF($H$29&lt;0,-$H$29/(-$H$29+100),100/($H$29+100)))</f>
@@ -11642,14 +11642,14 @@
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
-          <t>Over 9.5</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="F31" s="13" t="n">
-        <v>0.4783</v>
+        <v>0.5783</v>
       </c>
       <c r="G31" s="14" t="n">
-        <v>109</v>
+        <v>-137</v>
       </c>
       <c r="H31" s="15" t="n">
         <v>113</v>
@@ -11676,7 +11676,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Model 47.8% (fair +109). Your call.</t>
+          <t>Model 57.8% (fair -137). Your call.</t>
         </is>
       </c>
       <c r="O31" s="15" t="n"/>
@@ -11708,17 +11708,17 @@
       </c>
       <c r="E32" s="20" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Under 8.5</t>
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.5217000000000001</v>
+        <v>0.4217</v>
       </c>
       <c r="G32" s="14" t="n">
-        <v>-109</v>
+        <v>137</v>
       </c>
       <c r="H32" s="15" t="n">
-        <v>128</v>
+        <v>105</v>
       </c>
       <c r="I32" s="13">
         <f>IF($H$32="","",IF($H$32&lt;0,-$H$32/(-$H$32+100),100/($H$32+100)))</f>
@@ -11742,7 +11742,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Model 52.2% (fair -109). Your call.</t>
+          <t>Model 42.2% (fair +137). Your call.</t>
         </is>
       </c>
       <c r="O32" s="15" t="n"/>
@@ -11784,7 +11784,7 @@
         <v>111</v>
       </c>
       <c r="H33" s="15" t="n">
-        <v>163</v>
+        <v>130</v>
       </c>
       <c r="I33" s="13">
         <f>IF($H$33="","",IF($H$33&lt;0,-$H$33/(-$H$33+100),100/($H$33+100)))</f>
@@ -11850,7 +11850,7 @@
         <v>-111</v>
       </c>
       <c r="H34" s="15" t="n">
-        <v>-130</v>
+        <v>107</v>
       </c>
       <c r="I34" s="13">
         <f>IF($H$34="","",IF($H$34&lt;0,-$H$34/(-$H$34+100),100/($H$34+100)))</f>
@@ -11910,13 +11910,13 @@
         </is>
       </c>
       <c r="F35" s="13" t="n">
-        <v>0.4521311475409836</v>
+        <v>0.4492</v>
       </c>
       <c r="G35" s="14" t="n">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="H35" s="15" t="n">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="I35" s="13">
         <f>IF($H$35="","",IF($H$35&lt;0,-$H$35/(-$H$35+100),100/($H$35+100)))</f>
@@ -11940,7 +11940,7 @@
       </c>
       <c r="N35" s="19" t="inlineStr">
         <is>
-          <t>Model 45.2% (fair +121). Your call.</t>
+          <t>Model 44.9% (fair +123). Your call.</t>
         </is>
       </c>
       <c r="O35" s="15" t="n"/>
@@ -11976,10 +11976,10 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.5479081967213115</v>
+        <v>0.5508000000000001</v>
       </c>
       <c r="G36" s="14" t="n">
-        <v>-121</v>
+        <v>-123</v>
       </c>
       <c r="H36" s="15" t="n">
         <v>-144</v>
@@ -12006,7 +12006,7 @@
       </c>
       <c r="N36" s="19" t="inlineStr">
         <is>
-          <t>Model 54.8% (fair -121). Your call.</t>
+          <t>Model 55.1% (fair -123). Your call.</t>
         </is>
       </c>
       <c r="O36" s="15" t="n"/>
@@ -12038,17 +12038,17 @@
       </c>
       <c r="E37" s="12" t="inlineStr">
         <is>
-          <t>Over 8</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="F37" s="13" t="n">
-        <v>0.3837</v>
+        <v>0.4625</v>
       </c>
       <c r="G37" s="14" t="n">
-        <v>161</v>
+        <v>116</v>
       </c>
       <c r="H37" s="15" t="n">
-        <v>112</v>
+        <v>-104</v>
       </c>
       <c r="I37" s="13">
         <f>IF($H$37="","",IF($H$37&lt;0,-$H$37/(-$H$37+100),100/($H$37+100)))</f>
@@ -12072,7 +12072,7 @@
       </c>
       <c r="N37" s="19" t="inlineStr">
         <is>
-          <t>Model 38.4% (fair +161). Your call.</t>
+          <t>Model 46.2% (fair +116). Your call.</t>
         </is>
       </c>
       <c r="O37" s="15" t="n"/>
@@ -12104,17 +12104,17 @@
       </c>
       <c r="E38" s="20" t="inlineStr">
         <is>
-          <t>Under 8</t>
+          <t>Under 7.5</t>
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.6163000000000001</v>
+        <v>0.5375</v>
       </c>
       <c r="G38" s="14" t="n">
-        <v>-161</v>
+        <v>-116</v>
       </c>
       <c r="H38" s="15" t="n">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="I38" s="13">
         <f>IF($H$38="","",IF($H$38&lt;0,-$H$38/(-$H$38+100),100/($H$38+100)))</f>
@@ -12138,7 +12138,7 @@
       </c>
       <c r="N38" s="19" t="inlineStr">
         <is>
-          <t>Model 61.6% (fair -161). Your call.</t>
+          <t>Model 53.8% (fair -116). Your call.</t>
         </is>
       </c>
       <c r="O38" s="15" t="n"/>
@@ -12306,10 +12306,10 @@
         </is>
       </c>
       <c r="F41" s="13" t="n">
-        <v>0.3715765765765766</v>
+        <v>0.3729279279279279</v>
       </c>
       <c r="G41" s="14" t="n">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H41" s="15" t="n">
         <v>122</v>
@@ -12336,7 +12336,7 @@
       </c>
       <c r="N41" s="19" t="inlineStr">
         <is>
-          <t>Model 37.2% (fair +169). Your call.</t>
+          <t>Model 37.3% (fair +168). Your call.</t>
         </is>
       </c>
       <c r="O41" s="15" t="n"/>
@@ -12372,13 +12372,13 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.6284444444444445</v>
+        <v>0.627090990990991</v>
       </c>
       <c r="G42" s="14" t="n">
-        <v>-169</v>
+        <v>-168</v>
       </c>
       <c r="H42" s="15" t="n">
-        <v>-125</v>
+        <v>-122</v>
       </c>
       <c r="I42" s="13">
         <f>IF($H$42="","",IF($H$42&lt;0,-$H$42/(-$H$42+100),100/($H$42+100)))</f>
@@ -12402,7 +12402,7 @@
       </c>
       <c r="N42" s="19" t="inlineStr">
         <is>
-          <t>Model 62.8% (fair -169). Your call.</t>
+          <t>Model 62.7% (fair -168). Your call.</t>
         </is>
       </c>
       <c r="O42" s="15" t="n"/>
@@ -12510,7 +12510,7 @@
         <v>-111</v>
       </c>
       <c r="H44" s="15" t="n">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="I44" s="13">
         <f>IF($H$44="","",IF($H$44&lt;0,-$H$44/(-$H$44+100),100/($H$44+100)))</f>
@@ -12642,7 +12642,7 @@
         <v>133</v>
       </c>
       <c r="H46" s="15" t="n">
-        <v>-119</v>
+        <v>138</v>
       </c>
       <c r="I46" s="13">
         <f>IF($H$46="","",IF($H$46&lt;0,-$H$46/(-$H$46+100),100/($H$46+100)))</f>
@@ -12834,13 +12834,13 @@
         </is>
       </c>
       <c r="F49" s="13" t="n">
-        <v>0.3654326923076923</v>
+        <v>0.2407</v>
       </c>
       <c r="G49" s="14" t="n">
-        <v>174</v>
+        <v>315</v>
       </c>
       <c r="H49" s="15" t="n">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I49" s="13">
         <f>IF($H$49="","",IF($H$49&lt;0,-$H$49/(-$H$49+100),100/($H$49+100)))</f>
@@ -12864,7 +12864,7 @@
       </c>
       <c r="N49" s="19" t="inlineStr">
         <is>
-          <t>Model 36.5% (fair +174). Your call.</t>
+          <t>Model 24.1% (fair +315). Your call.</t>
         </is>
       </c>
       <c r="O49" s="15" t="n"/>
@@ -12900,13 +12900,13 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.6345499999999999</v>
+        <v>0.7593</v>
       </c>
       <c r="G50" s="14" t="n">
-        <v>-174</v>
+        <v>-315</v>
       </c>
       <c r="H50" s="15" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="I50" s="13">
         <f>IF($H$50="","",IF($H$50&lt;0,-$H$50/(-$H$50+100),100/($H$50+100)))</f>
@@ -12930,7 +12930,7 @@
       </c>
       <c r="N50" s="19" t="inlineStr">
         <is>
-          <t>Model 63.5% (fair -174). Your call.</t>
+          <t>Model 75.9% (fair -315). Your call.</t>
         </is>
       </c>
       <c r="O50" s="15" t="n"/>
@@ -12966,7 +12966,7 @@
         </is>
       </c>
       <c r="F51" s="13" t="n">
-        <v>0.4533039647577092</v>
+        <v>0.4516299559471365</v>
       </c>
       <c r="G51" s="14" t="n">
         <v>121</v>
@@ -12996,7 +12996,7 @@
       </c>
       <c r="N51" s="19" t="inlineStr">
         <is>
-          <t>Model 45.3% (fair +121). Your call.</t>
+          <t>Model 45.2% (fair +121). Your call.</t>
         </is>
       </c>
       <c r="O51" s="15" t="n"/>
@@ -13032,13 +13032,13 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.5467061946902656</v>
+        <v>0.5483739130434783</v>
       </c>
       <c r="G52" s="14" t="n">
         <v>-121</v>
       </c>
       <c r="H52" s="15" t="n">
-        <v>-126</v>
+        <v>-130</v>
       </c>
       <c r="I52" s="13">
         <f>IF($H$52="","",IF($H$52&lt;0,-$H$52/(-$H$52+100),100/($H$52+100)))</f>
@@ -13062,7 +13062,7 @@
       </c>
       <c r="N52" s="19" t="inlineStr">
         <is>
-          <t>Model 54.7% (fair -121). Your call.</t>
+          <t>Model 54.8% (fair -121). Your call.</t>
         </is>
       </c>
       <c r="O52" s="15" t="n"/>
@@ -13236,7 +13236,7 @@
         <v>107</v>
       </c>
       <c r="H55" s="15" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I55" s="13">
         <f>IF($H$55="","",IF($H$55&lt;0,-$H$55/(-$H$55+100),100/($H$55+100)))</f>
@@ -13302,7 +13302,7 @@
         <v>-107</v>
       </c>
       <c r="H56" s="15" t="n">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="I56" s="13">
         <f>IF($H$56="","",IF($H$56&lt;0,-$H$56/(-$H$56+100),100/($H$56+100)))</f>
@@ -13494,13 +13494,13 @@
         </is>
       </c>
       <c r="F59" s="13" t="n">
-        <v>0.5400484978540773</v>
+        <v>0.5449840336134453</v>
       </c>
       <c r="G59" s="14" t="n">
-        <v>-117</v>
+        <v>-120</v>
       </c>
       <c r="H59" s="15" t="n">
-        <v>-133</v>
+        <v>-138</v>
       </c>
       <c r="I59" s="13">
         <f>IF($H$59="","",IF($H$59&lt;0,-$H$59/(-$H$59+100),100/($H$59+100)))</f>
@@ -13524,7 +13524,7 @@
       </c>
       <c r="N59" s="19" t="inlineStr">
         <is>
-          <t>Model 54.0% (fair -117). Your call.</t>
+          <t>Model 54.5% (fair -120). Your call.</t>
         </is>
       </c>
       <c r="O59" s="15" t="n"/>
@@ -13560,13 +13560,13 @@
         </is>
       </c>
       <c r="F60" s="13" t="n">
-        <v>0.4599579831932774</v>
+        <v>0.455</v>
       </c>
       <c r="G60" s="14" t="n">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="H60" s="15" t="n">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="I60" s="13">
         <f>IF($H$60="","",IF($H$60&lt;0,-$H$60/(-$H$60+100),100/($H$60+100)))</f>
@@ -13590,7 +13590,7 @@
       </c>
       <c r="N60" s="19" t="inlineStr">
         <is>
-          <t>Model 46.0% (fair +117). Your call.</t>
+          <t>Model 45.5% (fair +120). Your call.</t>
         </is>
       </c>
       <c r="O60" s="15" t="n"/>
@@ -13626,13 +13626,13 @@
         </is>
       </c>
       <c r="F61" s="13" t="n">
-        <v>0.4167694581280788</v>
+        <v>0.3201</v>
       </c>
       <c r="G61" s="14" t="n">
-        <v>140</v>
+        <v>212</v>
       </c>
       <c r="H61" s="15" t="n">
-        <v>-103</v>
+        <v>106</v>
       </c>
       <c r="I61" s="13">
         <f>IF($H$61="","",IF($H$61&lt;0,-$H$61/(-$H$61+100),100/($H$61+100)))</f>
@@ -13656,7 +13656,7 @@
       </c>
       <c r="N61" s="19" t="inlineStr">
         <is>
-          <t>Model 41.7% (fair +140). Your call.</t>
+          <t>Model 32.0% (fair +212). Your call.</t>
         </is>
       </c>
       <c r="O61" s="15" t="n"/>
@@ -13692,10 +13692,10 @@
         </is>
       </c>
       <c r="F62" s="13" t="n">
-        <v>0.5832211538461538</v>
+        <v>0.6798999999999999</v>
       </c>
       <c r="G62" s="14" t="n">
-        <v>-140</v>
+        <v>-212</v>
       </c>
       <c r="H62" s="15" t="n">
         <v>108</v>
@@ -13722,7 +13722,7 @@
       </c>
       <c r="N62" s="19" t="inlineStr">
         <is>
-          <t>Model 58.3% (fair -140). Your call.</t>
+          <t>Model 68.0% (fair -212). Your call.</t>
         </is>
       </c>
       <c r="O62" s="15" t="n"/>
@@ -13830,7 +13830,7 @@
         <v>-166</v>
       </c>
       <c r="H64" s="15" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="I64" s="13">
         <f>IF($H$64="","",IF($H$64&lt;0,-$H$64/(-$H$64+100),100/($H$64+100)))</f>
@@ -14406,10 +14406,10 @@
         </is>
       </c>
       <c r="F73" s="13" t="n">
-        <v>0.5120673076923077</v>
+        <v>0.5167788461538462</v>
       </c>
       <c r="G73" s="14" t="n">
-        <v>-105</v>
+        <v>-107</v>
       </c>
       <c r="H73" s="15" t="n">
         <v>108</v>
@@ -14436,7 +14436,7 @@
       </c>
       <c r="N73" s="19" t="inlineStr">
         <is>
-          <t>Model 51.2% (fair -105). Your call.</t>
+          <t>Model 51.7% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O73" s="15" t="n"/>
@@ -14472,13 +14472,13 @@
         </is>
       </c>
       <c r="F74" s="13" t="n">
-        <v>0.4879730769230769</v>
+        <v>0.48325</v>
       </c>
       <c r="G74" s="14" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H74" s="15" t="n">
-        <v>-108</v>
+        <v>100</v>
       </c>
       <c r="I74" s="13">
         <f>IF($H$74="","",IF($H$74&lt;0,-$H$74/(-$H$74+100),100/($H$74+100)))</f>
@@ -14502,7 +14502,7 @@
       </c>
       <c r="N74" s="19" t="inlineStr">
         <is>
-          <t>Model 48.8% (fair +105). Your call.</t>
+          <t>Model 48.3% (fair +107). Your call.</t>
         </is>
       </c>
       <c r="O74" s="15" t="n"/>
@@ -14610,7 +14610,7 @@
         <v>-144</v>
       </c>
       <c r="H76" s="15" t="n">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="I76" s="13">
         <f>IF($H$76="","",IF($H$76&lt;0,-$H$76/(-$H$76+100),100/($H$76+100)))</f>
@@ -14934,10 +14934,10 @@
         </is>
       </c>
       <c r="F81" s="13" t="n">
-        <v>0.5942372623574145</v>
+        <v>0.5914482889733841</v>
       </c>
       <c r="G81" s="14" t="n">
-        <v>-146</v>
+        <v>-145</v>
       </c>
       <c r="H81" s="15" t="n">
         <v>-163</v>
@@ -14964,7 +14964,7 @@
       </c>
       <c r="N81" s="19" t="inlineStr">
         <is>
-          <t>Model 59.4% (fair -146). Your call.</t>
+          <t>Model 59.1% (fair -145). Your call.</t>
         </is>
       </c>
       <c r="O81" s="15" t="n"/>
@@ -15000,13 +15000,13 @@
         </is>
       </c>
       <c r="F82" s="13" t="n">
-        <v>0.4057421875</v>
+        <v>0.40856</v>
       </c>
       <c r="G82" s="14" t="n">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="H82" s="15" t="n">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="I82" s="13">
         <f>IF($H$82="","",IF($H$82&lt;0,-$H$82/(-$H$82+100),100/($H$82+100)))</f>
@@ -15030,7 +15030,7 @@
       </c>
       <c r="N82" s="19" t="inlineStr">
         <is>
-          <t>Model 40.6% (fair +146). Your call.</t>
+          <t>Model 40.9% (fair +145). Your call.</t>
         </is>
       </c>
       <c r="O82" s="15" t="n"/>
@@ -15198,10 +15198,10 @@
         </is>
       </c>
       <c r="F85" s="13" t="n">
-        <v>0.5238461538461537</v>
+        <v>0.5266346153846153</v>
       </c>
       <c r="G85" s="14" t="n">
-        <v>-110</v>
+        <v>-111</v>
       </c>
       <c r="H85" s="15" t="n">
         <v>108</v>
@@ -15228,7 +15228,7 @@
       </c>
       <c r="N85" s="19" t="inlineStr">
         <is>
-          <t>Model 52.4% (fair -110). Your call.</t>
+          <t>Model 52.7% (fair -111). Your call.</t>
         </is>
       </c>
       <c r="O85" s="15" t="n"/>
@@ -15264,13 +15264,13 @@
         </is>
       </c>
       <c r="F86" s="13" t="n">
-        <v>0.476142654028436</v>
+        <v>0.4733980582524272</v>
       </c>
       <c r="G86" s="14" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H86" s="15" t="n">
-        <v>-111</v>
+        <v>-106</v>
       </c>
       <c r="I86" s="13">
         <f>IF($H$86="","",IF($H$86&lt;0,-$H$86/(-$H$86+100),100/($H$86+100)))</f>
@@ -15294,7 +15294,7 @@
       </c>
       <c r="N86" s="19" t="inlineStr">
         <is>
-          <t>Model 47.6% (fair +110). Your call.</t>
+          <t>Model 47.3% (fair +111). Your call.</t>
         </is>
       </c>
       <c r="O86" s="15" t="n"/>
@@ -15594,7 +15594,7 @@
         </is>
       </c>
       <c r="F91" s="13" t="n">
-        <v>0.4914903846153846</v>
+        <v>0.4935096153846154</v>
       </c>
       <c r="G91" s="14" t="n">
         <v>103</v>
@@ -15624,7 +15624,7 @@
       </c>
       <c r="N91" s="19" t="inlineStr">
         <is>
-          <t>Model 49.1% (fair +103). Your call.</t>
+          <t>Model 49.4% (fair +103). Your call.</t>
         </is>
       </c>
       <c r="O91" s="15" t="n"/>
@@ -15660,13 +15660,13 @@
         </is>
       </c>
       <c r="F92" s="13" t="n">
-        <v>0.5084917050691244</v>
+        <v>0.5064840375586854</v>
       </c>
       <c r="G92" s="14" t="n">
         <v>-103</v>
       </c>
       <c r="H92" s="15" t="n">
-        <v>-117</v>
+        <v>-113</v>
       </c>
       <c r="I92" s="13">
         <f>IF($H$92="","",IF($H$92&lt;0,-$H$92/(-$H$92+100),100/($H$92+100)))</f>
@@ -15690,7 +15690,7 @@
       </c>
       <c r="N92" s="19" t="inlineStr">
         <is>
-          <t>Model 50.8% (fair -103). Your call.</t>
+          <t>Model 50.6% (fair -103). Your call.</t>
         </is>
       </c>
       <c r="O92" s="15" t="n"/>
@@ -15726,13 +15726,13 @@
         </is>
       </c>
       <c r="F93" s="13" t="n">
-        <v>0.4086785714285715</v>
+        <v>0.4103260869565218</v>
       </c>
       <c r="G93" s="14" t="n">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H93" s="15" t="n">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="I93" s="13">
         <f>IF($H$93="","",IF($H$93&lt;0,-$H$93/(-$H$93+100),100/($H$93+100)))</f>
@@ -15756,7 +15756,7 @@
       </c>
       <c r="N93" s="19" t="inlineStr">
         <is>
-          <t>Model 40.9% (fair +145). Your call.</t>
+          <t>Model 41.0% (fair +144). Your call.</t>
         </is>
       </c>
       <c r="O93" s="15" t="n"/>
@@ -15792,10 +15792,10 @@
         </is>
       </c>
       <c r="F94" s="13" t="n">
-        <v>0.5913057553956834</v>
+        <v>0.5896410071942446</v>
       </c>
       <c r="G94" s="14" t="n">
-        <v>-145</v>
+        <v>-144</v>
       </c>
       <c r="H94" s="15" t="n">
         <v>-178</v>
@@ -15822,7 +15822,7 @@
       </c>
       <c r="N94" s="19" t="inlineStr">
         <is>
-          <t>Model 59.1% (fair -145). Your call.</t>
+          <t>Model 59.0% (fair -144). Your call.</t>
         </is>
       </c>
       <c r="O94" s="15" t="n"/>
@@ -15930,7 +15930,7 @@
         <v>102</v>
       </c>
       <c r="H96" s="15" t="n">
-        <v>-111</v>
+        <v>-110</v>
       </c>
       <c r="I96" s="13">
         <f>IF($H$96="","",IF($H$96&lt;0,-$H$96/(-$H$96+100),100/($H$96+100)))</f>
@@ -15986,17 +15986,17 @@
       </c>
       <c r="E97" s="12" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Over 8</t>
         </is>
       </c>
       <c r="F97" s="13" t="n">
-        <v>0.4414</v>
+        <v>0.4785951219512195</v>
       </c>
       <c r="G97" s="14" t="n">
-        <v>127</v>
+        <v>109</v>
       </c>
       <c r="H97" s="15" t="n">
-        <v>104</v>
+        <v>-105</v>
       </c>
       <c r="I97" s="13">
         <f>IF($H$97="","",IF($H$97&lt;0,-$H$97/(-$H$97+100),100/($H$97+100)))</f>
@@ -16020,7 +16020,7 @@
       </c>
       <c r="N97" s="19" t="inlineStr">
         <is>
-          <t>Model 44.1% (fair +127). Your call.</t>
+          <t>Model 47.9% (fair +109). Your call.</t>
         </is>
       </c>
       <c r="O97" s="15" t="n"/>
@@ -16052,14 +16052,14 @@
       </c>
       <c r="E98" s="20" t="inlineStr">
         <is>
-          <t>Under 8.5</t>
+          <t>Under 8</t>
         </is>
       </c>
       <c r="F98" s="13" t="n">
-        <v>0.5586</v>
+        <v>0.5213942307692307</v>
       </c>
       <c r="G98" s="14" t="n">
-        <v>-127</v>
+        <v>-109</v>
       </c>
       <c r="H98" s="15" t="n">
         <v>108</v>
@@ -16086,7 +16086,7 @@
       </c>
       <c r="N98" s="19" t="inlineStr">
         <is>
-          <t>Model 55.9% (fair -127). Your call.</t>
+          <t>Model 52.1% (fair -109). Your call.</t>
         </is>
       </c>
       <c r="O98" s="15" t="n"/>
@@ -16194,7 +16194,7 @@
         <v>-183</v>
       </c>
       <c r="H100" s="15" t="n">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="I100" s="13">
         <f>IF($H$100="","",IF($H$100&lt;0,-$H$100/(-$H$100+100),100/($H$100+100)))</f>
@@ -16260,7 +16260,7 @@
         <v>-121</v>
       </c>
       <c r="H101" s="15" t="n">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="I101" s="13">
         <f>IF($H$101="","",IF($H$101&lt;0,-$H$101/(-$H$101+100),100/($H$101+100)))</f>
@@ -16386,10 +16386,10 @@
         </is>
       </c>
       <c r="F103" s="13" t="n">
-        <v>0.4287980769230769</v>
+        <v>0.4335096153846154</v>
       </c>
       <c r="G103" s="14" t="n">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="H103" s="15" t="n">
         <v>108</v>
@@ -16416,7 +16416,7 @@
       </c>
       <c r="N103" s="19" t="inlineStr">
         <is>
-          <t>Model 42.9% (fair +133). Your call.</t>
+          <t>Model 43.4% (fair +131). Your call.</t>
         </is>
       </c>
       <c r="O103" s="15" t="n"/>
@@ -16452,13 +16452,13 @@
         </is>
       </c>
       <c r="F104" s="13" t="n">
-        <v>0.5712057692307693</v>
+        <v>0.56645</v>
       </c>
       <c r="G104" s="14" t="n">
-        <v>-133</v>
+        <v>-131</v>
       </c>
       <c r="H104" s="15" t="n">
-        <v>-108</v>
+        <v>100</v>
       </c>
       <c r="I104" s="13">
         <f>IF($H$104="","",IF($H$104&lt;0,-$H$104/(-$H$104+100),100/($H$104+100)))</f>
@@ -16482,7 +16482,7 @@
       </c>
       <c r="N104" s="19" t="inlineStr">
         <is>
-          <t>Model 57.1% (fair -133). Your call.</t>
+          <t>Model 56.6% (fair -131). Your call.</t>
         </is>
       </c>
       <c r="O104" s="15" t="n"/>
@@ -16518,13 +16518,13 @@
         </is>
       </c>
       <c r="F105" s="13" t="n">
-        <v>0.3563461538461538</v>
+        <v>0.3297</v>
       </c>
       <c r="G105" s="14" t="n">
-        <v>181</v>
+        <v>203</v>
       </c>
       <c r="H105" s="15" t="n">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="I105" s="13">
         <f>IF($H$105="","",IF($H$105&lt;0,-$H$105/(-$H$105+100),100/($H$105+100)))</f>
@@ -16548,7 +16548,7 @@
       </c>
       <c r="N105" s="19" t="inlineStr">
         <is>
-          <t>Model 35.6% (fair +181). Your call.</t>
+          <t>Model 33.0% (fair +203). Your call.</t>
         </is>
       </c>
       <c r="O105" s="15" t="n"/>
@@ -16584,13 +16584,13 @@
         </is>
       </c>
       <c r="F106" s="13" t="n">
-        <v>0.6436330798479087</v>
+        <v>0.6703</v>
       </c>
       <c r="G106" s="14" t="n">
-        <v>-181</v>
+        <v>-203</v>
       </c>
       <c r="H106" s="15" t="n">
-        <v>-163</v>
+        <v>156</v>
       </c>
       <c r="I106" s="13">
         <f>IF($H$106="","",IF($H$106&lt;0,-$H$106/(-$H$106+100),100/($H$106+100)))</f>
@@ -16614,7 +16614,7 @@
       </c>
       <c r="N106" s="19" t="inlineStr">
         <is>
-          <t>Model 64.4% (fair -181). Your call.</t>
+          <t>Model 67.0% (fair -203). Your call.</t>
         </is>
       </c>
       <c r="O106" s="15" t="n"/>
@@ -16650,10 +16650,10 @@
         </is>
       </c>
       <c r="F107" s="13" t="n">
-        <v>0.4395491803278689</v>
+        <v>0.4399180327868852</v>
       </c>
       <c r="G107" s="14" t="n">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H107" s="15" t="n">
         <v>144</v>
@@ -16680,7 +16680,7 @@
       </c>
       <c r="N107" s="19" t="inlineStr">
         <is>
-          <t>Model 44.0% (fair +128). Your call.</t>
+          <t>Model 44.0% (fair +127). Your call.</t>
         </is>
       </c>
       <c r="O107" s="15" t="n"/>
@@ -16716,13 +16716,13 @@
         </is>
       </c>
       <c r="F108" s="13" t="n">
-        <v>0.5604069958847737</v>
+        <v>0.5600785123966943</v>
       </c>
       <c r="G108" s="14" t="n">
         <v>-127</v>
       </c>
       <c r="H108" s="15" t="n">
-        <v>-143</v>
+        <v>-142</v>
       </c>
       <c r="I108" s="13">
         <f>IF($H$108="","",IF($H$108&lt;0,-$H$108/(-$H$108+100),100/($H$108+100)))</f>
@@ -17046,13 +17046,13 @@
         </is>
       </c>
       <c r="F113" s="13" t="n">
-        <v>0.4870322274881516</v>
+        <v>0.4842346153846154</v>
       </c>
       <c r="G113" s="14" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H113" s="15" t="n">
-        <v>-111</v>
+        <v>-108</v>
       </c>
       <c r="I113" s="13">
         <f>IF($H$113="","",IF($H$113&lt;0,-$H$113/(-$H$113+100),100/($H$113+100)))</f>
@@ -17076,7 +17076,7 @@
       </c>
       <c r="N113" s="19" t="inlineStr">
         <is>
-          <t>Model 48.7% (fair +105). Your call.</t>
+          <t>Model 48.4% (fair +107). Your call.</t>
         </is>
       </c>
       <c r="O113" s="15" t="n"/>
@@ -17112,13 +17112,13 @@
         </is>
       </c>
       <c r="F114" s="13" t="n">
-        <v>0.5129326923076922</v>
+        <v>0.5157766990291262</v>
       </c>
       <c r="G114" s="14" t="n">
-        <v>-105</v>
+        <v>-107</v>
       </c>
       <c r="H114" s="15" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="I114" s="13">
         <f>IF($H$114="","",IF($H$114&lt;0,-$H$114/(-$H$114+100),100/($H$114+100)))</f>
@@ -17142,7 +17142,7 @@
       </c>
       <c r="N114" s="19" t="inlineStr">
         <is>
-          <t>Model 51.3% (fair -105). Your call.</t>
+          <t>Model 51.6% (fair -107). Your call.</t>
         </is>
       </c>
       <c r="O114" s="15" t="n"/>
@@ -17310,13 +17310,13 @@
         </is>
       </c>
       <c r="F117" s="13" t="n">
-        <v>0.6269326530612244</v>
+        <v>0.626577049180328</v>
       </c>
       <c r="G117" s="14" t="n">
         <v>-168</v>
       </c>
       <c r="H117" s="15" t="n">
-        <v>-145</v>
+        <v>-144</v>
       </c>
       <c r="I117" s="13">
         <f>IF($H$117="","",IF($H$117&lt;0,-$H$117/(-$H$117+100),100/($H$117+100)))</f>
@@ -17376,7 +17376,7 @@
         </is>
       </c>
       <c r="F118" s="13" t="n">
-        <v>0.373109243697479</v>
+        <v>0.3734453781512606</v>
       </c>
       <c r="G118" s="14" t="n">
         <v>168</v>
@@ -17442,13 +17442,13 @@
         </is>
       </c>
       <c r="F119" s="13" t="n">
-        <v>0.3613688212927757</v>
+        <v>0.3627307692307692</v>
       </c>
       <c r="G119" s="14" t="n">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H119" s="15" t="n">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="I119" s="13">
         <f>IF($H$119="","",IF($H$119&lt;0,-$H$119/(-$H$119+100),100/($H$119+100)))</f>
@@ -17472,7 +17472,7 @@
       </c>
       <c r="N119" s="19" t="inlineStr">
         <is>
-          <t>Model 36.1% (fair +177). Your call.</t>
+          <t>Model 36.3% (fair +176). Your call.</t>
         </is>
       </c>
       <c r="O119" s="15" t="n"/>
@@ -17508,10 +17508,10 @@
         </is>
       </c>
       <c r="F120" s="13" t="n">
-        <v>0.638612927756654</v>
+        <v>0.6373114068441065</v>
       </c>
       <c r="G120" s="14" t="n">
-        <v>-177</v>
+        <v>-176</v>
       </c>
       <c r="H120" s="15" t="n">
         <v>-163</v>
@@ -17538,7 +17538,7 @@
       </c>
       <c r="N120" s="19" t="inlineStr">
         <is>
-          <t>Model 63.9% (fair -177). Your call.</t>
+          <t>Model 63.7% (fair -176). Your call.</t>
         </is>
       </c>
       <c r="O120" s="15" t="n"/>

</xml_diff>